<commit_message>
Show landed cost after uplift next to Self-Cost source cells
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
+++ b/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
@@ -775,7 +775,7 @@
     <xf numFmtId="0" fontId="11" fillId="19" borderId="10"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="10"/>
   </cellStyleXfs>
-  <cellXfs count="175">
+  <cellXfs count="176">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1256,6 +1256,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="184" fontId="8" fillId="18" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="22" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="179" fontId="38" fillId="25" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -6419,23 +6422,31 @@
     <row r="24" ht="30" customHeight="1" s="71">
       <c r="A24" s="54" t="inlineStr">
         <is>
-          <t>Landed cost per Self-Cost, 4 SKUs (Vegetable…), €/pack — before uplift</t>
+          <t>Landed cost, 4 SKUs (Vegetable…), €/pack — Self-Cost (col. B) → after uplift (col. C)</t>
         </is>
       </c>
       <c r="B24" s="149">
         <f>'Model 6 pallets'!E13</f>
         <v>1.134046875</v>
       </c>
+      <c r="C24" s="174">
+        <f>B24*(1+$G$14)</f>
+        <v>1.3835371874999998</v>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1" s="71">
       <c r="A25" s="54" t="inlineStr">
         <is>
-          <t>Landed cost per Self-Cost, 2 SKUs (Gouda, Carbonara), €/pack — before uplift</t>
+          <t>Landed cost, 2 SKUs (Gouda, Carbonara), €/pack — Self-Cost (col. B) → after uplift (col. C)</t>
         </is>
       </c>
       <c r="B25" s="149">
         <f>'Model 6 pallets'!E11</f>
         <v>1.308515625</v>
+      </c>
+      <c r="C25" s="174">
+        <f>B25*(1+$G$14)</f>
+        <v>1.5963890625000001</v>
       </c>
     </row>
   </sheetData>
@@ -7007,23 +7018,31 @@
     <row r="23" ht="30" customHeight="1" s="71">
       <c r="A23" s="54" t="inlineStr">
         <is>
-          <t>Landed cost per Self-Cost, 4 SKUs (Vegetable…), €/pack — before uplift</t>
+          <t>Landed cost, 4 SKUs (Vegetable…), €/pack — Self-Cost (col. B) → after uplift (col. C)</t>
         </is>
       </c>
       <c r="B23" s="149">
         <f>'Model 33 pallets'!E13</f>
         <v>0.882380333698031</v>
       </c>
+      <c r="C23" s="174">
+        <f>B23*(1+$G$14)</f>
+        <v>1.0765040071115979</v>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1" s="71">
       <c r="A24" s="54" t="inlineStr">
         <is>
-          <t>Landed cost per Self-Cost, 2 SKUs (Gouda, Carbonara), €/pack — before uplift</t>
+          <t>Landed cost, 2 SKUs (Gouda, Carbonara), €/pack — Self-Cost (col. B) → after uplift (col. C)</t>
         </is>
       </c>
       <c r="B24" s="149">
         <f>'Model 33 pallets'!E11</f>
         <v>1.018131154266958</v>
+      </c>
+      <c r="C24" s="174">
+        <f>B24*(1+$G$14)</f>
+        <v>1.2421200082056887</v>
       </c>
     </row>
   </sheetData>
@@ -7268,7 +7287,7 @@
         <f>ROUNDDOWN((($H9/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K9" s="174">
+      <c r="K9" s="175">
         <f>J9/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7280,7 +7299,7 @@
         <f>ROUNDDOWN((($H9/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N9" s="174">
+      <c r="N9" s="175">
         <f>M9/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -7331,7 +7350,7 @@
         <f>ROUNDDOWN((($H11/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K11" s="174">
+      <c r="K11" s="175">
         <f>J11/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7343,7 +7362,7 @@
         <f>ROUNDDOWN((($H11/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N11" s="174">
+      <c r="N11" s="175">
         <f>M11/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -7387,7 +7406,7 @@
         <f>ROUNDDOWN((($H12/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K12" s="174">
+      <c r="K12" s="175">
         <f>J12/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7399,7 +7418,7 @@
         <f>ROUNDDOWN((($H12/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N12" s="174">
+      <c r="N12" s="175">
         <f>M12/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -7444,7 +7463,7 @@
         <f>ROUNDDOWN((($H13/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K13" s="174">
+      <c r="K13" s="175">
         <f>J13/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7456,7 +7475,7 @@
         <f>ROUNDDOWN((($H13/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N13" s="174">
+      <c r="N13" s="175">
         <f>M13/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -7501,7 +7520,7 @@
         <f>ROUNDDOWN((($H14/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K14" s="174">
+      <c r="K14" s="175">
         <f>J14/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7513,7 +7532,7 @@
         <f>ROUNDDOWN((($H14/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N14" s="174">
+      <c r="N14" s="175">
         <f>M14/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -7564,7 +7583,7 @@
         <f>ROUNDDOWN((($H16/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.6</v>
       </c>
-      <c r="K16" s="174">
+      <c r="K16" s="175">
         <f>J16/0.65-1</f>
         <v>-0.07692307692307698</v>
       </c>
@@ -7576,7 +7595,7 @@
         <f>ROUNDDOWN((($H16/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.39</v>
       </c>
-      <c r="N16" s="174">
+      <c r="N16" s="175">
         <f>M16/0.65-1</f>
         <v>-0.4</v>
       </c>
@@ -7620,7 +7639,7 @@
         <f>ROUNDDOWN((($H17/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K17" s="174">
+      <c r="K17" s="175">
         <f>J17/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7632,7 +7651,7 @@
         <f>ROUNDDOWN((($H17/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.33</v>
       </c>
-      <c r="N17" s="174">
+      <c r="N17" s="175">
         <f>M17/0.65-1</f>
         <v>-0.49230769230769234</v>
       </c>
@@ -7676,7 +7695,7 @@
         <f>ROUNDDOWN((($H18/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.48</v>
       </c>
-      <c r="K18" s="174">
+      <c r="K18" s="175">
         <f>J18/0.65-1</f>
         <v>-0.2615384615384616</v>
       </c>
@@ -7688,7 +7707,7 @@
         <f>ROUNDDOWN((($H18/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.27</v>
       </c>
-      <c r="N18" s="174">
+      <c r="N18" s="175">
         <f>M18/0.65-1</f>
         <v>-0.5846153846153845</v>
       </c>
@@ -7732,7 +7751,7 @@
         <f>ROUNDDOWN((($H19/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.42</v>
       </c>
-      <c r="K19" s="174">
+      <c r="K19" s="175">
         <f>J19/0.65-1</f>
         <v>-0.3538461538461539</v>
       </c>
@@ -7744,7 +7763,7 @@
         <f>ROUNDDOWN((($H19/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.2</v>
       </c>
-      <c r="N19" s="174">
+      <c r="N19" s="175">
         <f>M19/0.65-1</f>
         <v>-0.6923076923076923</v>
       </c>
@@ -7795,7 +7814,7 @@
         <f>ROUNDDOWN((($H21/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.47</v>
       </c>
-      <c r="K21" s="174">
+      <c r="K21" s="175">
         <f>J21/0.65-1</f>
         <v>-0.27692307692307694</v>
       </c>
@@ -7807,7 +7826,7 @@
         <f>ROUNDDOWN((($H21/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.25</v>
       </c>
-      <c r="N21" s="174">
+      <c r="N21" s="175">
         <f>M21/0.65-1</f>
         <v>-0.6153846153846154</v>
       </c>
@@ -7851,7 +7870,7 @@
         <f>ROUNDDOWN((($H22/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.4</v>
       </c>
-      <c r="K22" s="174">
+      <c r="K22" s="175">
         <f>J22/0.65-1</f>
         <v>-0.3846153846153846</v>
       </c>
@@ -7863,7 +7882,7 @@
         <f>ROUNDDOWN((($H22/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.19</v>
       </c>
-      <c r="N22" s="174">
+      <c r="N22" s="175">
         <f>M22/0.65-1</f>
         <v>-0.7076923076923076</v>
       </c>
@@ -7914,7 +7933,7 @@
         <f>ROUNDDOWN((($H24/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.6</v>
       </c>
-      <c r="K24" s="174">
+      <c r="K24" s="175">
         <f>J24/0.65-1</f>
         <v>-0.07692307692307698</v>
       </c>
@@ -7926,7 +7945,7 @@
         <f>ROUNDDOWN((($H24/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.39</v>
       </c>
-      <c r="N24" s="174">
+      <c r="N24" s="175">
         <f>M24/0.65-1</f>
         <v>-0.4</v>
       </c>
@@ -7970,7 +7989,7 @@
         <f>ROUNDDOWN((($H25/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.67</v>
       </c>
-      <c r="K25" s="174">
+      <c r="K25" s="175">
         <f>J25/0.65-1</f>
         <v>0.030769230769230882</v>
       </c>
@@ -7982,7 +8001,7 @@
         <f>ROUNDDOWN((($H25/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.46</v>
       </c>
-      <c r="N25" s="174">
+      <c r="N25" s="175">
         <f>M25/0.65-1</f>
         <v>-0.29230769230769227</v>
       </c>

</xml_diff>

<commit_message>
Internal model: uplift applied on all sheets incl. Model tabs (source kept in col AL)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
+++ b/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
@@ -1964,7 +1964,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI39"/>
+  <dimension ref="A1:AL39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="4" customWidth="1" style="71" min="1" max="1"/>
@@ -1981,6 +1981,7 @@
     <col width="18" customWidth="1" style="71" min="13" max="13"/>
     <col width="31" customWidth="1" style="71" min="14" max="15"/>
     <col width="19" customWidth="1" style="71" min="16" max="35"/>
+    <col width="18" customWidth="1" style="71" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="71">
@@ -2014,7 +2015,7 @@
       </c>
       <c r="E2" s="86" t="inlineStr">
         <is>
-          <t>Ready-made landed cost from Self-Cost_Sias: AJ6:AJ11. Cost composition preserved.</t>
+          <t>Landed cost = Self-Cost_Sias (col. AL) × (1 + uplift from G14 on the "Price 120 UAH" sheet). Cost composition preserved.</t>
         </is>
       </c>
       <c r="F2" s="87" t="n"/>
@@ -2248,7 +2249,7 @@
       </c>
       <c r="E10" s="78" t="inlineStr">
         <is>
-          <t>Landed cost, EUR/pack</t>
+          <t>Landed cost incl. uplift, EUR/pack</t>
         </is>
       </c>
       <c r="F10" s="78" t="inlineStr">
@@ -2399,6 +2400,11 @@
       <c r="AI10" s="44" t="inlineStr">
         <is>
           <t>Shelf price incl. VAT, UAH</t>
+        </is>
+      </c>
+      <c r="AL10" s="84" t="inlineStr">
+        <is>
+          <t>Self-Cost source, EUR/pack (before uplift)</t>
         </is>
       </c>
     </row>
@@ -2419,80 +2425,81 @@
       <c r="D11" s="7" t="n">
         <v>123</v>
       </c>
-      <c r="E11" s="24" t="n">
-        <v>1.308515625</v>
+      <c r="E11" s="24">
+        <f>AL11*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>1.5963890625000001</v>
       </c>
       <c r="F11" s="8">
         <f>IF(AND(ISNUMBER(E11),ISNUMBER($D$8)),E11*$D$3,NA())</f>
-        <v>66.99600000000001</v>
+        <v>81.73512000000001</v>
       </c>
       <c r="G11" s="9">
         <f>F11/$D$8</f>
-        <v>148.88000000000002</v>
+        <v>181.63360000000003</v>
       </c>
       <c r="H11" s="10">
         <f>G11*$D$4</f>
-        <v>52.108000000000004</v>
+        <v>63.571760000000005</v>
       </c>
       <c r="I11" s="11">
         <f>G11-F11-H11</f>
-        <v>29.77600000000001</v>
+        <v>36.326720000000016</v>
       </c>
       <c r="J11" s="12">
         <f>I11/G11</f>
-        <v>0.20000000000000004</v>
+        <v>0.20000000000000007</v>
       </c>
       <c r="K11" s="13">
         <f>G11*$D$6</f>
-        <v>208.43200000000002</v>
+        <v>254.28704000000002</v>
       </c>
       <c r="L11" s="14">
         <f>F11/(1-$D$4)</f>
-        <v>103.07076923076924</v>
+        <v>125.74633846153847</v>
       </c>
       <c r="M11" s="14">
         <f>L11*$D$6</f>
-        <v>144.29907692307694</v>
+        <v>176.04487384615385</v>
       </c>
       <c r="N11" s="15">
         <f>G11-F11</f>
-        <v>81.88400000000001</v>
+        <v>99.89848000000002</v>
       </c>
       <c r="O11" s="16">
         <f>N11-H11</f>
-        <v>29.77600000000001</v>
+        <v>36.326720000000016</v>
       </c>
       <c r="P11" s="40">
         <f>$F11/(1-$D$4-$P$9)</f>
-        <v>191.41714285714286</v>
+        <v>233.52891428571428</v>
       </c>
       <c r="Q11" s="41">
         <f>P11*$D$4</f>
-        <v>66.996</v>
+        <v>81.73512</v>
       </c>
       <c r="R11" s="42">
         <f>P11-$F11-Q11</f>
-        <v>57.42514285714286</v>
+        <v>70.05867428571429</v>
       </c>
       <c r="S11" s="43">
         <f>R11/P11</f>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T11" s="40">
         <f>P11*$D$6</f>
-        <v>267.984</v>
+        <v>326.94048</v>
       </c>
       <c r="U11" s="40">
         <f>$F11/(1-$D$4-$U$9)</f>
-        <v>167.49</v>
+        <v>204.33780000000002</v>
       </c>
       <c r="V11" s="41">
         <f>U11*$D$4</f>
-        <v>58.6215</v>
+        <v>71.51823</v>
       </c>
       <c r="W11" s="42">
         <f>U11-$F11-V11</f>
-        <v>41.8725</v>
+        <v>51.084450000000004</v>
       </c>
       <c r="X11" s="43">
         <f>W11/U11</f>
@@ -2500,39 +2507,39 @@
       </c>
       <c r="Y11" s="40">
         <f>U11*$D$6</f>
-        <v>234.486</v>
+        <v>286.07292</v>
       </c>
       <c r="Z11" s="40">
         <f>$F11/(1-$D$4-$Z$9)</f>
-        <v>148.88000000000002</v>
+        <v>181.63360000000003</v>
       </c>
       <c r="AA11" s="41">
         <f>Z11*$D$4</f>
-        <v>52.108000000000004</v>
+        <v>63.571760000000005</v>
       </c>
       <c r="AB11" s="42">
         <f>Z11-$F11-AA11</f>
-        <v>29.77600000000001</v>
+        <v>36.326720000000016</v>
       </c>
       <c r="AC11" s="43">
         <f>AB11/Z11</f>
-        <v>0.20000000000000004</v>
+        <v>0.20000000000000007</v>
       </c>
       <c r="AD11" s="40">
         <f>Z11*$D$6</f>
-        <v>208.43200000000002</v>
+        <v>254.28704000000002</v>
       </c>
       <c r="AE11" s="40">
         <f>$F11/(1-$D$4-$AE$9)</f>
-        <v>133.99200000000002</v>
+        <v>163.47024000000002</v>
       </c>
       <c r="AF11" s="41">
         <f>AE11*$D$4</f>
-        <v>46.897200000000005</v>
+        <v>57.214584</v>
       </c>
       <c r="AG11" s="42">
         <f>AE11-$F11-AF11</f>
-        <v>20.098800000000004</v>
+        <v>24.520536000000007</v>
       </c>
       <c r="AH11" s="43">
         <f>AG11/AE11</f>
@@ -2540,7 +2547,10 @@
       </c>
       <c r="AI11" s="40">
         <f>AE11*$D$6</f>
-        <v>187.58880000000002</v>
+        <v>228.858336</v>
+      </c>
+      <c r="AL11" s="24" t="n">
+        <v>1.308515625</v>
       </c>
     </row>
     <row r="12" ht="43.5" customHeight="1" s="71">
@@ -2560,80 +2570,81 @@
       <c r="D12" s="7" t="n">
         <v>131</v>
       </c>
-      <c r="E12" s="24" t="n">
-        <v>1.308515625</v>
+      <c r="E12" s="24">
+        <f>AL12*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>1.5963890625000001</v>
       </c>
       <c r="F12" s="8">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER($D$8)),E12*$D$3,NA())</f>
-        <v>66.99600000000001</v>
+        <v>81.73512000000001</v>
       </c>
       <c r="G12" s="9">
         <f>F12/$D$8</f>
-        <v>148.88000000000002</v>
+        <v>181.63360000000003</v>
       </c>
       <c r="H12" s="10">
         <f>G12*$D$4</f>
-        <v>52.108000000000004</v>
+        <v>63.571760000000005</v>
       </c>
       <c r="I12" s="11">
         <f>G12-F12-H12</f>
-        <v>29.77600000000001</v>
+        <v>36.326720000000016</v>
       </c>
       <c r="J12" s="12">
         <f>I12/G12</f>
-        <v>0.20000000000000004</v>
+        <v>0.20000000000000007</v>
       </c>
       <c r="K12" s="13">
         <f>G12*$D$6</f>
-        <v>208.43200000000002</v>
+        <v>254.28704000000002</v>
       </c>
       <c r="L12" s="14">
         <f>F12/(1-$D$4)</f>
-        <v>103.07076923076924</v>
+        <v>125.74633846153847</v>
       </c>
       <c r="M12" s="14">
         <f>L12*$D$6</f>
-        <v>144.29907692307694</v>
+        <v>176.04487384615385</v>
       </c>
       <c r="N12" s="15">
         <f>G12-F12</f>
-        <v>81.88400000000001</v>
+        <v>99.89848000000002</v>
       </c>
       <c r="O12" s="16">
         <f>N12-H12</f>
-        <v>29.77600000000001</v>
+        <v>36.326720000000016</v>
       </c>
       <c r="P12" s="40">
         <f>$F12/(1-$D$4-$P$9)</f>
-        <v>191.41714285714286</v>
+        <v>233.52891428571428</v>
       </c>
       <c r="Q12" s="41">
         <f>P12*$D$4</f>
-        <v>66.996</v>
+        <v>81.73512</v>
       </c>
       <c r="R12" s="42">
         <f>P12-$F12-Q12</f>
-        <v>57.42514285714286</v>
+        <v>70.05867428571429</v>
       </c>
       <c r="S12" s="43">
         <f>R12/P12</f>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T12" s="40">
         <f>P12*$D$6</f>
-        <v>267.984</v>
+        <v>326.94048</v>
       </c>
       <c r="U12" s="40">
         <f>$F12/(1-$D$4-$U$9)</f>
-        <v>167.49</v>
+        <v>204.33780000000002</v>
       </c>
       <c r="V12" s="41">
         <f>U12*$D$4</f>
-        <v>58.6215</v>
+        <v>71.51823</v>
       </c>
       <c r="W12" s="42">
         <f>U12-$F12-V12</f>
-        <v>41.8725</v>
+        <v>51.084450000000004</v>
       </c>
       <c r="X12" s="43">
         <f>W12/U12</f>
@@ -2641,39 +2652,39 @@
       </c>
       <c r="Y12" s="40">
         <f>U12*$D$6</f>
-        <v>234.486</v>
+        <v>286.07292</v>
       </c>
       <c r="Z12" s="40">
         <f>$F12/(1-$D$4-$Z$9)</f>
-        <v>148.88000000000002</v>
+        <v>181.63360000000003</v>
       </c>
       <c r="AA12" s="41">
         <f>Z12*$D$4</f>
-        <v>52.108000000000004</v>
+        <v>63.571760000000005</v>
       </c>
       <c r="AB12" s="42">
         <f>Z12-$F12-AA12</f>
-        <v>29.77600000000001</v>
+        <v>36.326720000000016</v>
       </c>
       <c r="AC12" s="43">
         <f>AB12/Z12</f>
-        <v>0.20000000000000004</v>
+        <v>0.20000000000000007</v>
       </c>
       <c r="AD12" s="40">
         <f>Z12*$D$6</f>
-        <v>208.43200000000002</v>
+        <v>254.28704000000002</v>
       </c>
       <c r="AE12" s="40">
         <f>$F12/(1-$D$4-$AE$9)</f>
-        <v>133.99200000000002</v>
+        <v>163.47024000000002</v>
       </c>
       <c r="AF12" s="41">
         <f>AE12*$D$4</f>
-        <v>46.897200000000005</v>
+        <v>57.214584</v>
       </c>
       <c r="AG12" s="42">
         <f>AE12-$F12-AF12</f>
-        <v>20.098800000000004</v>
+        <v>24.520536000000007</v>
       </c>
       <c r="AH12" s="43">
         <f>AG12/AE12</f>
@@ -2681,7 +2692,10 @@
       </c>
       <c r="AI12" s="40">
         <f>AE12*$D$6</f>
-        <v>187.58880000000002</v>
+        <v>228.858336</v>
+      </c>
+      <c r="AL12" s="24" t="n">
+        <v>1.308515625</v>
       </c>
     </row>
     <row r="13" ht="43.5" customHeight="1" s="71">
@@ -2701,128 +2715,132 @@
       <c r="D13" s="7" t="n">
         <v>113</v>
       </c>
-      <c r="E13" s="24" t="n">
-        <v>1.134046875</v>
+      <c r="E13" s="24">
+        <f>AL13*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>1.3835371874999998</v>
       </c>
       <c r="F13" s="8">
         <f>IF(AND(ISNUMBER(E13),ISNUMBER($D$8)),E13*$D$3,NA())</f>
-        <v>58.063199999999995</v>
+        <v>70.837104</v>
       </c>
       <c r="G13" s="9">
         <f>F13/$D$8</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="H13" s="10">
         <f>G13*$D$4</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="I13" s="11">
         <f>G13-F13-H13</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="J13" s="12">
         <f>I13/G13</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="K13" s="13">
         <f>G13*$D$6</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="L13" s="14">
         <f>F13/(1-$D$4)</f>
-        <v>89.32799999999999</v>
+        <v>108.98016</v>
       </c>
       <c r="M13" s="14">
         <f>L13*$D$6</f>
-        <v>125.05919999999998</v>
+        <v>152.57222399999998</v>
       </c>
       <c r="N13" s="15">
         <f>G13-F13</f>
-        <v>70.96613333333332</v>
+        <v>86.57868266666667</v>
       </c>
       <c r="O13" s="16">
         <f>N13-H13</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="P13" s="40">
         <f>$F13/(1-$D$4-$P$9)</f>
-        <v>165.89485714285712</v>
+        <v>202.39172571428568</v>
       </c>
       <c r="Q13" s="41">
         <f>P13*$D$4</f>
-        <v>58.06319999999999</v>
+        <v>70.83710399999998</v>
       </c>
       <c r="R13" s="42">
         <f>P13-$F13-Q13</f>
-        <v>49.76845714285714</v>
+        <v>60.71751771428572</v>
       </c>
       <c r="S13" s="43">
         <f>R13/P13</f>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T13" s="40">
         <f>P13*$D$6</f>
-        <v>232.25279999999995</v>
+        <v>283.34841599999993</v>
       </c>
       <c r="U13" s="40">
         <f>$F13/(1-$D$4-$U$9)</f>
-        <v>145.158</v>
+        <v>177.09275999999997</v>
       </c>
       <c r="V13" s="41">
         <f>U13*$D$4</f>
-        <v>50.805299999999995</v>
+        <v>61.98246599999999</v>
       </c>
       <c r="W13" s="42">
         <f>U13-$F13-V13</f>
-        <v>36.2895</v>
+        <v>44.273189999999985</v>
       </c>
       <c r="X13" s="43">
         <f>W13/U13</f>
-        <v>0.25</v>
+        <v>0.24999999999999997</v>
       </c>
       <c r="Y13" s="40">
         <f>U13*$D$6</f>
-        <v>203.22119999999998</v>
+        <v>247.92986399999995</v>
       </c>
       <c r="Z13" s="40">
         <f>$F13/(1-$D$4-$Z$9)</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="AA13" s="41">
         <f>Z13*$D$4</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="AB13" s="42">
         <f>Z13-$F13-AA13</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="AC13" s="43">
         <f>AB13/Z13</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="AD13" s="40">
         <f>Z13*$D$6</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="AE13" s="40">
         <f>$F13/(1-$D$4-$AE$9)</f>
-        <v>116.12639999999999</v>
+        <v>141.674208</v>
       </c>
       <c r="AF13" s="41">
         <f>AE13*$D$4</f>
-        <v>40.644239999999996</v>
+        <v>49.58597279999999</v>
       </c>
       <c r="AG13" s="42">
         <f>AE13-$F13-AF13</f>
-        <v>17.41896</v>
+        <v>21.251131200000003</v>
       </c>
       <c r="AH13" s="43">
         <f>AG13/AE13</f>
-        <v>0.15</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="AI13" s="40">
         <f>AE13*$D$6</f>
-        <v>162.57695999999999</v>
+        <v>198.34389119999997</v>
+      </c>
+      <c r="AL13" s="24" t="n">
+        <v>1.134046875</v>
       </c>
     </row>
     <row r="14" ht="43.5" customHeight="1" s="71">
@@ -2842,128 +2860,132 @@
       <c r="D14" s="25" t="n">
         <v>112.5</v>
       </c>
-      <c r="E14" s="24" t="n">
-        <v>1.134046875</v>
+      <c r="E14" s="24">
+        <f>AL14*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>1.3835371874999998</v>
       </c>
       <c r="F14" s="8">
         <f>IF(AND(ISNUMBER(E14),ISNUMBER($D$8)),E14*$D$3,NA())</f>
-        <v>58.063199999999995</v>
+        <v>70.837104</v>
       </c>
       <c r="G14" s="9">
         <f>F14/$D$8</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="H14" s="10">
         <f>G14*$D$4</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="I14" s="11">
         <f>G14-F14-H14</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="J14" s="12">
         <f>I14/G14</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="K14" s="13">
         <f>G14*$D$6</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="L14" s="14">
         <f>F14/(1-$D$4)</f>
-        <v>89.32799999999999</v>
+        <v>108.98016</v>
       </c>
       <c r="M14" s="14">
         <f>L14*$D$6</f>
-        <v>125.05919999999998</v>
+        <v>152.57222399999998</v>
       </c>
       <c r="N14" s="15">
         <f>G14-F14</f>
-        <v>70.96613333333332</v>
+        <v>86.57868266666667</v>
       </c>
       <c r="O14" s="16">
         <f>N14-H14</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="P14" s="40">
         <f>$F14/(1-$D$4-$P$9)</f>
-        <v>165.89485714285712</v>
+        <v>202.39172571428568</v>
       </c>
       <c r="Q14" s="41">
         <f>P14*$D$4</f>
-        <v>58.06319999999999</v>
+        <v>70.83710399999998</v>
       </c>
       <c r="R14" s="42">
         <f>P14-$F14-Q14</f>
-        <v>49.76845714285714</v>
+        <v>60.71751771428572</v>
       </c>
       <c r="S14" s="43">
         <f>R14/P14</f>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T14" s="40">
         <f>P14*$D$6</f>
-        <v>232.25279999999995</v>
+        <v>283.34841599999993</v>
       </c>
       <c r="U14" s="40">
         <f>$F14/(1-$D$4-$U$9)</f>
-        <v>145.158</v>
+        <v>177.09275999999997</v>
       </c>
       <c r="V14" s="41">
         <f>U14*$D$4</f>
-        <v>50.805299999999995</v>
+        <v>61.98246599999999</v>
       </c>
       <c r="W14" s="42">
         <f>U14-$F14-V14</f>
-        <v>36.2895</v>
+        <v>44.273189999999985</v>
       </c>
       <c r="X14" s="43">
         <f>W14/U14</f>
-        <v>0.25</v>
+        <v>0.24999999999999997</v>
       </c>
       <c r="Y14" s="40">
         <f>U14*$D$6</f>
-        <v>203.22119999999998</v>
+        <v>247.92986399999995</v>
       </c>
       <c r="Z14" s="40">
         <f>$F14/(1-$D$4-$Z$9)</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="AA14" s="41">
         <f>Z14*$D$4</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="AB14" s="42">
         <f>Z14-$F14-AA14</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="AC14" s="43">
         <f>AB14/Z14</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="AD14" s="40">
         <f>Z14*$D$6</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="AE14" s="40">
         <f>$F14/(1-$D$4-$AE$9)</f>
-        <v>116.12639999999999</v>
+        <v>141.674208</v>
       </c>
       <c r="AF14" s="41">
         <f>AE14*$D$4</f>
-        <v>40.644239999999996</v>
+        <v>49.58597279999999</v>
       </c>
       <c r="AG14" s="42">
         <f>AE14-$F14-AF14</f>
-        <v>17.41896</v>
+        <v>21.251131200000003</v>
       </c>
       <c r="AH14" s="43">
         <f>AG14/AE14</f>
-        <v>0.15</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="AI14" s="40">
         <f>AE14*$D$6</f>
-        <v>162.57695999999999</v>
+        <v>198.34389119999997</v>
+      </c>
+      <c r="AL14" s="24" t="n">
+        <v>1.134046875</v>
       </c>
     </row>
     <row r="15" ht="43.5" customHeight="1" s="71">
@@ -2983,128 +3005,132 @@
       <c r="D15" s="7" t="n">
         <v>113</v>
       </c>
-      <c r="E15" s="24" t="n">
-        <v>1.134046875</v>
+      <c r="E15" s="24">
+        <f>AL15*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>1.3835371874999998</v>
       </c>
       <c r="F15" s="8">
         <f>IF(AND(ISNUMBER(E15),ISNUMBER($D$8)),E15*$D$3,NA())</f>
-        <v>58.063199999999995</v>
+        <v>70.837104</v>
       </c>
       <c r="G15" s="9">
         <f>F15/$D$8</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="H15" s="10">
         <f>G15*$D$4</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="I15" s="11">
         <f>G15-F15-H15</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="J15" s="12">
         <f>I15/G15</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="K15" s="13">
         <f>G15*$D$6</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="L15" s="14">
         <f>F15/(1-$D$4)</f>
-        <v>89.32799999999999</v>
+        <v>108.98016</v>
       </c>
       <c r="M15" s="14">
         <f>L15*$D$6</f>
-        <v>125.05919999999998</v>
+        <v>152.57222399999998</v>
       </c>
       <c r="N15" s="15">
         <f>G15-F15</f>
-        <v>70.96613333333332</v>
+        <v>86.57868266666667</v>
       </c>
       <c r="O15" s="16">
         <f>N15-H15</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="P15" s="40">
         <f>$F15/(1-$D$4-$P$9)</f>
-        <v>165.89485714285712</v>
+        <v>202.39172571428568</v>
       </c>
       <c r="Q15" s="41">
         <f>P15*$D$4</f>
-        <v>58.06319999999999</v>
+        <v>70.83710399999998</v>
       </c>
       <c r="R15" s="42">
         <f>P15-$F15-Q15</f>
-        <v>49.76845714285714</v>
+        <v>60.71751771428572</v>
       </c>
       <c r="S15" s="43">
         <f>R15/P15</f>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T15" s="40">
         <f>P15*$D$6</f>
-        <v>232.25279999999995</v>
+        <v>283.34841599999993</v>
       </c>
       <c r="U15" s="40">
         <f>$F15/(1-$D$4-$U$9)</f>
-        <v>145.158</v>
+        <v>177.09275999999997</v>
       </c>
       <c r="V15" s="41">
         <f>U15*$D$4</f>
-        <v>50.805299999999995</v>
+        <v>61.98246599999999</v>
       </c>
       <c r="W15" s="42">
         <f>U15-$F15-V15</f>
-        <v>36.2895</v>
+        <v>44.273189999999985</v>
       </c>
       <c r="X15" s="43">
         <f>W15/U15</f>
-        <v>0.25</v>
+        <v>0.24999999999999997</v>
       </c>
       <c r="Y15" s="40">
         <f>U15*$D$6</f>
-        <v>203.22119999999998</v>
+        <v>247.92986399999995</v>
       </c>
       <c r="Z15" s="40">
         <f>$F15/(1-$D$4-$Z$9)</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="AA15" s="41">
         <f>Z15*$D$4</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="AB15" s="42">
         <f>Z15-$F15-AA15</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="AC15" s="43">
         <f>AB15/Z15</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="AD15" s="40">
         <f>Z15*$D$6</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="AE15" s="40">
         <f>$F15/(1-$D$4-$AE$9)</f>
-        <v>116.12639999999999</v>
+        <v>141.674208</v>
       </c>
       <c r="AF15" s="41">
         <f>AE15*$D$4</f>
-        <v>40.644239999999996</v>
+        <v>49.58597279999999</v>
       </c>
       <c r="AG15" s="42">
         <f>AE15-$F15-AF15</f>
-        <v>17.41896</v>
+        <v>21.251131200000003</v>
       </c>
       <c r="AH15" s="43">
         <f>AG15/AE15</f>
-        <v>0.15</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="AI15" s="40">
         <f>AE15*$D$6</f>
-        <v>162.57695999999999</v>
+        <v>198.34389119999997</v>
+      </c>
+      <c r="AL15" s="24" t="n">
+        <v>1.134046875</v>
       </c>
     </row>
     <row r="16" ht="43.5" customHeight="1" s="71">
@@ -3124,128 +3150,132 @@
       <c r="D16" s="7" t="n">
         <v>113</v>
       </c>
-      <c r="E16" s="24" t="n">
-        <v>1.134046875</v>
+      <c r="E16" s="24">
+        <f>AL16*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>1.3835371874999998</v>
       </c>
       <c r="F16" s="8">
         <f>IF(AND(ISNUMBER(E16),ISNUMBER($D$8)),E16*$D$3,NA())</f>
-        <v>58.063199999999995</v>
+        <v>70.837104</v>
       </c>
       <c r="G16" s="9">
         <f>F16/$D$8</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="H16" s="10">
         <f>G16*$D$4</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="I16" s="11">
         <f>G16-F16-H16</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="J16" s="12">
         <f>I16/G16</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="K16" s="13">
         <f>G16*$D$6</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="L16" s="14">
         <f>F16/(1-$D$4)</f>
-        <v>89.32799999999999</v>
+        <v>108.98016</v>
       </c>
       <c r="M16" s="14">
         <f>L16*$D$6</f>
-        <v>125.05919999999998</v>
+        <v>152.57222399999998</v>
       </c>
       <c r="N16" s="15">
         <f>G16-F16</f>
-        <v>70.96613333333332</v>
+        <v>86.57868266666667</v>
       </c>
       <c r="O16" s="16">
         <f>N16-H16</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="P16" s="40">
         <f>$F16/(1-$D$4-$P$9)</f>
-        <v>165.89485714285712</v>
+        <v>202.39172571428568</v>
       </c>
       <c r="Q16" s="41">
         <f>P16*$D$4</f>
-        <v>58.06319999999999</v>
+        <v>70.83710399999998</v>
       </c>
       <c r="R16" s="42">
         <f>P16-$F16-Q16</f>
-        <v>49.76845714285714</v>
+        <v>60.71751771428572</v>
       </c>
       <c r="S16" s="43">
         <f>R16/P16</f>
-        <v>0.3</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T16" s="40">
         <f>P16*$D$6</f>
-        <v>232.25279999999995</v>
+        <v>283.34841599999993</v>
       </c>
       <c r="U16" s="40">
         <f>$F16/(1-$D$4-$U$9)</f>
-        <v>145.158</v>
+        <v>177.09275999999997</v>
       </c>
       <c r="V16" s="41">
         <f>U16*$D$4</f>
-        <v>50.805299999999995</v>
+        <v>61.98246599999999</v>
       </c>
       <c r="W16" s="42">
         <f>U16-$F16-V16</f>
-        <v>36.2895</v>
+        <v>44.273189999999985</v>
       </c>
       <c r="X16" s="43">
         <f>W16/U16</f>
-        <v>0.25</v>
+        <v>0.24999999999999997</v>
       </c>
       <c r="Y16" s="40">
         <f>U16*$D$6</f>
-        <v>203.22119999999998</v>
+        <v>247.92986399999995</v>
       </c>
       <c r="Z16" s="40">
         <f>$F16/(1-$D$4-$Z$9)</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="AA16" s="41">
         <f>Z16*$D$4</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="AB16" s="42">
         <f>Z16-$F16-AA16</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="AC16" s="43">
         <f>AB16/Z16</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="AD16" s="40">
         <f>Z16*$D$6</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="AE16" s="40">
         <f>$F16/(1-$D$4-$AE$9)</f>
-        <v>116.12639999999999</v>
+        <v>141.674208</v>
       </c>
       <c r="AF16" s="41">
         <f>AE16*$D$4</f>
-        <v>40.644239999999996</v>
+        <v>49.58597279999999</v>
       </c>
       <c r="AG16" s="42">
         <f>AE16-$F16-AF16</f>
-        <v>17.41896</v>
+        <v>21.251131200000003</v>
       </c>
       <c r="AH16" s="43">
         <f>AG16/AE16</f>
-        <v>0.15</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="AI16" s="40">
         <f>AE16*$D$6</f>
-        <v>162.57695999999999</v>
+        <v>198.34389119999997</v>
+      </c>
+      <c r="AL16" s="24" t="n">
+        <v>1.134046875</v>
       </c>
     </row>
     <row r="17"/>
@@ -3330,27 +3360,27 @@
       <c r="E22" s="65" t="n"/>
       <c r="F22" s="29">
         <f>E11</f>
-        <v>1.308515625</v>
+        <v>1.5963890625000001</v>
       </c>
       <c r="G22" s="29">
         <f>E12</f>
-        <v>1.308515625</v>
+        <v>1.5963890625000001</v>
       </c>
       <c r="H22" s="29">
         <f>E13</f>
-        <v>1.134046875</v>
+        <v>1.3835371874999998</v>
       </c>
       <c r="I22" s="29">
         <f>E14</f>
-        <v>1.134046875</v>
+        <v>1.3835371874999998</v>
       </c>
       <c r="J22" s="29">
         <f>E15</f>
-        <v>1.134046875</v>
+        <v>1.3835371874999998</v>
       </c>
       <c r="K22" s="29">
         <f>E16</f>
-        <v>1.134046875</v>
+        <v>1.3835371874999998</v>
       </c>
     </row>
     <row r="23" ht="31.05" customHeight="1" s="71">
@@ -3412,27 +3442,27 @@
       <c r="E24" s="65" t="n"/>
       <c r="F24" s="31">
         <f>F11</f>
-        <v>66.99600000000001</v>
+        <v>81.73512000000001</v>
       </c>
       <c r="G24" s="31">
         <f>F12</f>
-        <v>66.99600000000001</v>
+        <v>81.73512000000001</v>
       </c>
       <c r="H24" s="31">
         <f>F13</f>
-        <v>58.063199999999995</v>
+        <v>70.837104</v>
       </c>
       <c r="I24" s="31">
         <f>F14</f>
-        <v>58.063199999999995</v>
+        <v>70.837104</v>
       </c>
       <c r="J24" s="31">
         <f>F15</f>
-        <v>58.063199999999995</v>
+        <v>70.837104</v>
       </c>
       <c r="K24" s="31">
         <f>F16</f>
-        <v>58.063199999999995</v>
+        <v>70.837104</v>
       </c>
     </row>
     <row r="25" ht="31.05" customHeight="1" s="71">
@@ -3652,27 +3682,27 @@
       <c r="E30" s="65" t="n"/>
       <c r="F30" s="34">
         <f>G11</f>
-        <v>148.88000000000002</v>
+        <v>181.63360000000003</v>
       </c>
       <c r="G30" s="34">
         <f>G12</f>
-        <v>148.88000000000002</v>
+        <v>181.63360000000003</v>
       </c>
       <c r="H30" s="34">
         <f>G13</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="I30" s="34">
         <f>G14</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="J30" s="34">
         <f>G15</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
       <c r="K30" s="34">
         <f>G16</f>
-        <v>129.0293333333333</v>
+        <v>157.41578666666666</v>
       </c>
     </row>
     <row r="31" ht="31.05" customHeight="1" s="71">
@@ -3693,27 +3723,27 @@
       <c r="E31" s="65" t="n"/>
       <c r="F31" s="31">
         <f>N11</f>
-        <v>81.88400000000001</v>
+        <v>99.89848000000002</v>
       </c>
       <c r="G31" s="31">
         <f>N12</f>
-        <v>81.88400000000001</v>
+        <v>99.89848000000002</v>
       </c>
       <c r="H31" s="31">
         <f>N13</f>
-        <v>70.96613333333332</v>
+        <v>86.57868266666667</v>
       </c>
       <c r="I31" s="31">
         <f>N14</f>
-        <v>70.96613333333332</v>
+        <v>86.57868266666667</v>
       </c>
       <c r="J31" s="31">
         <f>N15</f>
-        <v>70.96613333333332</v>
+        <v>86.57868266666667</v>
       </c>
       <c r="K31" s="31">
         <f>N16</f>
-        <v>70.96613333333332</v>
+        <v>86.57868266666667</v>
       </c>
     </row>
     <row r="32" ht="31.05" customHeight="1" s="71">
@@ -3734,27 +3764,27 @@
       <c r="E32" s="65" t="n"/>
       <c r="F32" s="31">
         <f>H11</f>
-        <v>52.108000000000004</v>
+        <v>63.571760000000005</v>
       </c>
       <c r="G32" s="31">
         <f>H12</f>
-        <v>52.108000000000004</v>
+        <v>63.571760000000005</v>
       </c>
       <c r="H32" s="31">
         <f>H13</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="I32" s="31">
         <f>H14</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="J32" s="31">
         <f>H15</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
       <c r="K32" s="31">
         <f>H16</f>
-        <v>45.16026666666666</v>
+        <v>55.09552533333333</v>
       </c>
     </row>
     <row r="33" ht="31.05" customHeight="1" s="71">
@@ -3775,27 +3805,27 @@
       <c r="E33" s="65" t="n"/>
       <c r="F33" s="36">
         <f>I11</f>
-        <v>29.77600000000001</v>
+        <v>36.326720000000016</v>
       </c>
       <c r="G33" s="36">
         <f>I12</f>
-        <v>29.77600000000001</v>
+        <v>36.326720000000016</v>
       </c>
       <c r="H33" s="36">
         <f>I13</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="I33" s="36">
         <f>I14</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="J33" s="36">
         <f>I15</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
       <c r="K33" s="36">
         <f>I16</f>
-        <v>25.80586666666666</v>
+        <v>31.483157333333338</v>
       </c>
     </row>
     <row r="34" ht="31.05" customHeight="1" s="71">
@@ -3816,27 +3846,27 @@
       <c r="E34" s="65" t="n"/>
       <c r="F34" s="37">
         <f>J11</f>
-        <v>0.20000000000000004</v>
+        <v>0.20000000000000007</v>
       </c>
       <c r="G34" s="37">
         <f>J12</f>
-        <v>0.20000000000000004</v>
+        <v>0.20000000000000007</v>
       </c>
       <c r="H34" s="37">
         <f>J13</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="I34" s="37">
         <f>J14</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="J34" s="37">
         <f>J15</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
       <c r="K34" s="37">
         <f>J16</f>
-        <v>0.19999999999999998</v>
+        <v>0.20000000000000004</v>
       </c>
     </row>
     <row r="35" ht="31.05" customHeight="1" s="71">
@@ -3939,27 +3969,27 @@
       <c r="E37" s="65" t="n"/>
       <c r="F37" s="34">
         <f>K11</f>
-        <v>208.43200000000002</v>
+        <v>254.28704000000002</v>
       </c>
       <c r="G37" s="34">
         <f>K12</f>
-        <v>208.43200000000002</v>
+        <v>254.28704000000002</v>
       </c>
       <c r="H37" s="34">
         <f>K13</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="I37" s="34">
         <f>K14</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="J37" s="34">
         <f>K15</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
       <c r="K37" s="34">
         <f>K16</f>
-        <v>180.64106666666663</v>
+        <v>220.3821013333333</v>
       </c>
     </row>
     <row r="38" ht="31.05" customHeight="1" s="71">
@@ -3980,27 +4010,27 @@
       <c r="E38" s="65" t="n"/>
       <c r="F38" s="31">
         <f>L11</f>
-        <v>103.07076923076924</v>
+        <v>125.74633846153847</v>
       </c>
       <c r="G38" s="31">
         <f>L12</f>
-        <v>103.07076923076924</v>
+        <v>125.74633846153847</v>
       </c>
       <c r="H38" s="31">
         <f>L13</f>
-        <v>89.32799999999999</v>
+        <v>108.98016</v>
       </c>
       <c r="I38" s="31">
         <f>L14</f>
-        <v>89.32799999999999</v>
+        <v>108.98016</v>
       </c>
       <c r="J38" s="31">
         <f>L15</f>
-        <v>89.32799999999999</v>
+        <v>108.98016</v>
       </c>
       <c r="K38" s="31">
         <f>L16</f>
-        <v>89.32799999999999</v>
+        <v>108.98016</v>
       </c>
     </row>
     <row r="39" ht="31.05" customHeight="1" s="71">
@@ -4021,27 +4051,27 @@
       <c r="E39" s="65" t="n"/>
       <c r="F39" s="31">
         <f>M11</f>
-        <v>144.29907692307694</v>
+        <v>176.04487384615385</v>
       </c>
       <c r="G39" s="31">
         <f>M12</f>
-        <v>144.29907692307694</v>
+        <v>176.04487384615385</v>
       </c>
       <c r="H39" s="31">
         <f>M13</f>
-        <v>125.05919999999998</v>
+        <v>152.57222399999998</v>
       </c>
       <c r="I39" s="31">
         <f>M14</f>
-        <v>125.05919999999998</v>
+        <v>152.57222399999998</v>
       </c>
       <c r="J39" s="31">
         <f>M15</f>
-        <v>125.05919999999998</v>
+        <v>152.57222399999998</v>
       </c>
       <c r="K39" s="31">
         <f>M16</f>
-        <v>125.05919999999998</v>
+        <v>152.57222399999998</v>
       </c>
     </row>
   </sheetData>
@@ -4125,7 +4155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AI39"/>
+  <dimension ref="A1:AL39"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="4" customWidth="1" style="71" min="1" max="1"/>
@@ -4142,6 +4172,7 @@
     <col width="18" customWidth="1" style="71" min="13" max="13"/>
     <col width="31" customWidth="1" style="71" min="14" max="15"/>
     <col width="19" customWidth="1" style="71" min="16" max="35"/>
+    <col width="18" customWidth="1" style="71" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1" ht="17.25" customHeight="1" s="71">
@@ -4175,7 +4206,7 @@
       </c>
       <c r="E2" s="86" t="inlineStr">
         <is>
-          <t>Ready-made landed cost from Self-Cost_Sias: AJ30:AJ35. Cost composition preserved.</t>
+          <t>Landed cost = Self-Cost_Sias (col. AL) × (1 + uplift from G14 on the "Price 120 UAH" sheet). Cost composition preserved.</t>
         </is>
       </c>
       <c r="F2" s="87" t="n"/>
@@ -4409,7 +4440,7 @@
       </c>
       <c r="E10" s="78" t="inlineStr">
         <is>
-          <t>Landed cost, EUR/pack</t>
+          <t>Landed cost incl. uplift, EUR/pack</t>
         </is>
       </c>
       <c r="F10" s="78" t="inlineStr">
@@ -4560,6 +4591,11 @@
       <c r="AI10" s="44" t="inlineStr">
         <is>
           <t>Shelf price incl. VAT, UAH</t>
+        </is>
+      </c>
+      <c r="AL10" s="84" t="inlineStr">
+        <is>
+          <t>Self-Cost source, EUR/pack (before uplift)</t>
         </is>
       </c>
     </row>
@@ -4580,60 +4616,61 @@
       <c r="D11" s="7" t="n">
         <v>123</v>
       </c>
-      <c r="E11" s="24" t="n">
-        <v>1.018131154266958</v>
+      <c r="E11" s="24">
+        <f>AL11*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>1.2421200082056887</v>
       </c>
       <c r="F11" s="8">
         <f>IF(AND(ISNUMBER(E11),ISNUMBER($D$8)),E11*$D$3,NA())</f>
-        <v>52.12831509846825</v>
+        <v>63.596544420131266</v>
       </c>
       <c r="G11" s="9">
         <f>F11/$D$8</f>
-        <v>115.84070021881833</v>
+        <v>141.32565426695837</v>
       </c>
       <c r="H11" s="10">
         <f>G11*$D$4</f>
-        <v>40.544245076586414</v>
+        <v>49.463978993435425</v>
       </c>
       <c r="I11" s="11">
         <f>G11-F11-H11</f>
-        <v>23.168140043763664</v>
+        <v>28.265130853391675</v>
       </c>
       <c r="J11" s="12">
         <f>I11/G11</f>
-        <v>0.19999999999999998</v>
+        <v>0.2</v>
       </c>
       <c r="K11" s="13">
         <f>G11*$D$6</f>
-        <v>162.17698030634565</v>
+        <v>197.8559159737417</v>
       </c>
       <c r="L11" s="14">
         <f>F11/(1-$D$4)</f>
-        <v>80.19740784379731</v>
+        <v>97.84083756943271</v>
       </c>
       <c r="M11" s="14">
         <f>L11*$D$6</f>
-        <v>112.27637098131622</v>
+        <v>136.9771725972058</v>
       </c>
       <c r="N11" s="15">
         <f>G11-F11</f>
-        <v>63.71238512035008</v>
+        <v>77.7291098468271</v>
       </c>
       <c r="O11" s="16">
         <f>N11-H11</f>
-        <v>23.168140043763664</v>
+        <v>28.265130853391675</v>
       </c>
       <c r="P11" s="40">
         <f>$F11/(1-$D$4-$P$9)</f>
-        <v>148.9380431384807</v>
+        <v>181.70441262894647</v>
       </c>
       <c r="Q11" s="41">
         <f>P11*$D$4</f>
-        <v>52.12831509846824</v>
+        <v>63.59654442013126</v>
       </c>
       <c r="R11" s="42">
         <f>P11-$F11-Q11</f>
-        <v>44.68141294154422</v>
+        <v>54.511323788683946</v>
       </c>
       <c r="S11" s="43">
         <f>R11/P11</f>
@@ -4641,19 +4678,19 @@
       </c>
       <c r="T11" s="40">
         <f>P11*$D$6</f>
-        <v>208.51326039387297</v>
+        <v>254.38617768052504</v>
       </c>
       <c r="U11" s="40">
         <f>$F11/(1-$D$4-$U$9)</f>
-        <v>130.32078774617062</v>
+        <v>158.99136105032815</v>
       </c>
       <c r="V11" s="41">
         <f>U11*$D$4</f>
-        <v>45.61227571115972</v>
+        <v>55.64697636761485</v>
       </c>
       <c r="W11" s="42">
         <f>U11-$F11-V11</f>
-        <v>32.580196936542656</v>
+        <v>39.74784026258204</v>
       </c>
       <c r="X11" s="43">
         <f>W11/U11</f>
@@ -4661,39 +4698,39 @@
       </c>
       <c r="Y11" s="40">
         <f>U11*$D$6</f>
-        <v>182.44910284463887</v>
+        <v>222.5879054704594</v>
       </c>
       <c r="Z11" s="40">
         <f>$F11/(1-$D$4-$Z$9)</f>
-        <v>115.84070021881833</v>
+        <v>141.32565426695837</v>
       </c>
       <c r="AA11" s="41">
         <f>Z11*$D$4</f>
-        <v>40.544245076586414</v>
+        <v>49.463978993435425</v>
       </c>
       <c r="AB11" s="42">
         <f>Z11-$F11-AA11</f>
-        <v>23.168140043763664</v>
+        <v>28.265130853391675</v>
       </c>
       <c r="AC11" s="43">
         <f>AB11/Z11</f>
-        <v>0.19999999999999998</v>
+        <v>0.2</v>
       </c>
       <c r="AD11" s="40">
         <f>Z11*$D$6</f>
-        <v>162.17698030634565</v>
+        <v>197.8559159737417</v>
       </c>
       <c r="AE11" s="40">
         <f>$F11/(1-$D$4-$AE$9)</f>
-        <v>104.2566301969365</v>
+        <v>127.19308884026253</v>
       </c>
       <c r="AF11" s="41">
         <f>AE11*$D$4</f>
-        <v>36.48982056892777</v>
+        <v>44.51758109409188</v>
       </c>
       <c r="AG11" s="42">
         <f>AE11-$F11-AF11</f>
-        <v>15.63849452954048</v>
+        <v>19.078963326039386</v>
       </c>
       <c r="AH11" s="43">
         <f>AG11/AE11</f>
@@ -4701,7 +4738,10 @@
       </c>
       <c r="AI11" s="40">
         <f>AE11*$D$6</f>
-        <v>145.95928227571108</v>
+        <v>178.07032437636752</v>
+      </c>
+      <c r="AL11" s="24" t="n">
+        <v>1.018131154266958</v>
       </c>
     </row>
     <row r="12" ht="43.5" customHeight="1" s="71">
@@ -4721,60 +4761,61 @@
       <c r="D12" s="7" t="n">
         <v>131</v>
       </c>
-      <c r="E12" s="24" t="n">
-        <v>1.018131154266958</v>
+      <c r="E12" s="24">
+        <f>AL12*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>1.2421200082056887</v>
       </c>
       <c r="F12" s="8">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER($D$8)),E12*$D$3,NA())</f>
-        <v>52.12831509846825</v>
+        <v>63.596544420131266</v>
       </c>
       <c r="G12" s="9">
         <f>F12/$D$8</f>
-        <v>115.84070021881833</v>
+        <v>141.32565426695837</v>
       </c>
       <c r="H12" s="10">
         <f>G12*$D$4</f>
-        <v>40.544245076586414</v>
+        <v>49.463978993435425</v>
       </c>
       <c r="I12" s="11">
         <f>G12-F12-H12</f>
-        <v>23.168140043763664</v>
+        <v>28.265130853391675</v>
       </c>
       <c r="J12" s="12">
         <f>I12/G12</f>
-        <v>0.19999999999999998</v>
+        <v>0.2</v>
       </c>
       <c r="K12" s="13">
         <f>G12*$D$6</f>
-        <v>162.17698030634565</v>
+        <v>197.8559159737417</v>
       </c>
       <c r="L12" s="14">
         <f>F12/(1-$D$4)</f>
-        <v>80.19740784379731</v>
+        <v>97.84083756943271</v>
       </c>
       <c r="M12" s="14">
         <f>L12*$D$6</f>
-        <v>112.27637098131622</v>
+        <v>136.9771725972058</v>
       </c>
       <c r="N12" s="15">
         <f>G12-F12</f>
-        <v>63.71238512035008</v>
+        <v>77.7291098468271</v>
       </c>
       <c r="O12" s="16">
         <f>N12-H12</f>
-        <v>23.168140043763664</v>
+        <v>28.265130853391675</v>
       </c>
       <c r="P12" s="40">
         <f>$F12/(1-$D$4-$P$9)</f>
-        <v>148.9380431384807</v>
+        <v>181.70441262894647</v>
       </c>
       <c r="Q12" s="41">
         <f>P12*$D$4</f>
-        <v>52.12831509846824</v>
+        <v>63.59654442013126</v>
       </c>
       <c r="R12" s="42">
         <f>P12-$F12-Q12</f>
-        <v>44.68141294154422</v>
+        <v>54.511323788683946</v>
       </c>
       <c r="S12" s="43">
         <f>R12/P12</f>
@@ -4782,19 +4823,19 @@
       </c>
       <c r="T12" s="40">
         <f>P12*$D$6</f>
-        <v>208.51326039387297</v>
+        <v>254.38617768052504</v>
       </c>
       <c r="U12" s="40">
         <f>$F12/(1-$D$4-$U$9)</f>
-        <v>130.32078774617062</v>
+        <v>158.99136105032815</v>
       </c>
       <c r="V12" s="41">
         <f>U12*$D$4</f>
-        <v>45.61227571115972</v>
+        <v>55.64697636761485</v>
       </c>
       <c r="W12" s="42">
         <f>U12-$F12-V12</f>
-        <v>32.580196936542656</v>
+        <v>39.74784026258204</v>
       </c>
       <c r="X12" s="43">
         <f>W12/U12</f>
@@ -4802,39 +4843,39 @@
       </c>
       <c r="Y12" s="40">
         <f>U12*$D$6</f>
-        <v>182.44910284463887</v>
+        <v>222.5879054704594</v>
       </c>
       <c r="Z12" s="40">
         <f>$F12/(1-$D$4-$Z$9)</f>
-        <v>115.84070021881833</v>
+        <v>141.32565426695837</v>
       </c>
       <c r="AA12" s="41">
         <f>Z12*$D$4</f>
-        <v>40.544245076586414</v>
+        <v>49.463978993435425</v>
       </c>
       <c r="AB12" s="42">
         <f>Z12-$F12-AA12</f>
-        <v>23.168140043763664</v>
+        <v>28.265130853391675</v>
       </c>
       <c r="AC12" s="43">
         <f>AB12/Z12</f>
-        <v>0.19999999999999998</v>
+        <v>0.2</v>
       </c>
       <c r="AD12" s="40">
         <f>Z12*$D$6</f>
-        <v>162.17698030634565</v>
+        <v>197.8559159737417</v>
       </c>
       <c r="AE12" s="40">
         <f>$F12/(1-$D$4-$AE$9)</f>
-        <v>104.2566301969365</v>
+        <v>127.19308884026253</v>
       </c>
       <c r="AF12" s="41">
         <f>AE12*$D$4</f>
-        <v>36.48982056892777</v>
+        <v>44.51758109409188</v>
       </c>
       <c r="AG12" s="42">
         <f>AE12-$F12-AF12</f>
-        <v>15.63849452954048</v>
+        <v>19.078963326039386</v>
       </c>
       <c r="AH12" s="43">
         <f>AG12/AE12</f>
@@ -4842,7 +4883,10 @@
       </c>
       <c r="AI12" s="40">
         <f>AE12*$D$6</f>
-        <v>145.95928227571108</v>
+        <v>178.07032437636752</v>
+      </c>
+      <c r="AL12" s="24" t="n">
+        <v>1.018131154266958</v>
       </c>
     </row>
     <row r="13" ht="43.5" customHeight="1" s="71">
@@ -4862,80 +4906,81 @@
       <c r="D13" s="7" t="n">
         <v>113</v>
       </c>
-      <c r="E13" s="24" t="n">
-        <v>0.8823803336980306</v>
+      <c r="E13" s="24">
+        <f>AL13*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>1.0765040071115979</v>
       </c>
       <c r="F13" s="8">
         <f>IF(AND(ISNUMBER(E13),ISNUMBER($D$8)),E13*$D$3,NA())</f>
-        <v>45.17787308533919</v>
+        <v>55.11700516411381</v>
       </c>
       <c r="G13" s="9">
         <f>F13/$D$8</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="H13" s="10">
         <f>G13*$D$4</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="I13" s="11">
         <f>G13-F13-H13</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="J13" s="12">
         <f>I13/G13</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="K13" s="13">
         <f>G13*$D$6</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="L13" s="14">
         <f>F13/(1-$D$4)</f>
-        <v>69.50442013129107</v>
+        <v>84.79539256017509</v>
       </c>
       <c r="M13" s="14">
         <f>L13*$D$6</f>
-        <v>97.30618818380749</v>
+        <v>118.71354958424511</v>
       </c>
       <c r="N13" s="15">
         <f>G13-F13</f>
-        <v>55.21740043763679</v>
+        <v>67.36522853391688</v>
       </c>
       <c r="O13" s="16">
         <f>N13-H13</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="P13" s="40">
         <f>$F13/(1-$D$4-$P$9)</f>
-        <v>129.0796373866834</v>
+        <v>157.47715761175374</v>
       </c>
       <c r="Q13" s="41">
         <f>P13*$D$4</f>
-        <v>45.177873085339186</v>
+        <v>55.117005164113806</v>
       </c>
       <c r="R13" s="42">
         <f>P13-$F13-Q13</f>
-        <v>38.723891216005015</v>
+        <v>47.24314728352613</v>
       </c>
       <c r="S13" s="43">
         <f>R13/P13</f>
-        <v>0.29999999999999993</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T13" s="40">
         <f>P13*$D$6</f>
-        <v>180.71149234135675</v>
+        <v>220.46802065645522</v>
       </c>
       <c r="U13" s="40">
         <f>$F13/(1-$D$4-$U$9)</f>
-        <v>112.94468271334797</v>
+        <v>137.79251291028453</v>
       </c>
       <c r="V13" s="41">
         <f>U13*$D$4</f>
-        <v>39.53063894967179</v>
+        <v>48.227379518599584</v>
       </c>
       <c r="W13" s="42">
         <f>U13-$F13-V13</f>
-        <v>28.236170678336997</v>
+        <v>34.44812822757114</v>
       </c>
       <c r="X13" s="43">
         <f>W13/U13</f>
@@ -4943,47 +4988,50 @@
       </c>
       <c r="Y13" s="40">
         <f>U13*$D$6</f>
-        <v>158.12255579868716</v>
+        <v>192.90951807439833</v>
       </c>
       <c r="Z13" s="40">
         <f>$F13/(1-$D$4-$Z$9)</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="AA13" s="41">
         <f>Z13*$D$4</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="AB13" s="42">
         <f>Z13-$F13-AA13</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="AC13" s="43">
         <f>AB13/Z13</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="AD13" s="40">
         <f>Z13*$D$6</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="AE13" s="40">
         <f>$F13/(1-$D$4-$AE$9)</f>
-        <v>90.35574617067839</v>
+        <v>110.23401032822763</v>
       </c>
       <c r="AF13" s="41">
         <f>AE13*$D$4</f>
-        <v>31.624511159737434</v>
+        <v>38.581903614879664</v>
       </c>
       <c r="AG13" s="42">
         <f>AE13-$F13-AF13</f>
-        <v>13.55336192560176</v>
+        <v>16.53510154923415</v>
       </c>
       <c r="AH13" s="43">
         <f>AG13/AE13</f>
-        <v>0.15000000000000002</v>
+        <v>0.15000000000000005</v>
       </c>
       <c r="AI13" s="40">
         <f>AE13*$D$6</f>
-        <v>126.49804463894974</v>
+        <v>154.32761445951866</v>
+      </c>
+      <c r="AL13" s="24" t="n">
+        <v>0.8823803336980306</v>
       </c>
     </row>
     <row r="14" ht="43.5" customHeight="1" s="71">
@@ -5003,80 +5051,81 @@
       <c r="D14" s="25" t="n">
         <v>112.5</v>
       </c>
-      <c r="E14" s="24" t="n">
-        <v>0.8823803336980306</v>
+      <c r="E14" s="24">
+        <f>AL14*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>1.0765040071115979</v>
       </c>
       <c r="F14" s="8">
         <f>IF(AND(ISNUMBER(E14),ISNUMBER($D$8)),E14*$D$3,NA())</f>
-        <v>45.17787308533919</v>
+        <v>55.11700516411381</v>
       </c>
       <c r="G14" s="9">
         <f>F14/$D$8</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="H14" s="10">
         <f>G14*$D$4</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="I14" s="11">
         <f>G14-F14-H14</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="J14" s="12">
         <f>I14/G14</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="K14" s="13">
         <f>G14*$D$6</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="L14" s="14">
         <f>F14/(1-$D$4)</f>
-        <v>69.50442013129107</v>
+        <v>84.79539256017509</v>
       </c>
       <c r="M14" s="14">
         <f>L14*$D$6</f>
-        <v>97.30618818380749</v>
+        <v>118.71354958424511</v>
       </c>
       <c r="N14" s="15">
         <f>G14-F14</f>
-        <v>55.21740043763679</v>
+        <v>67.36522853391688</v>
       </c>
       <c r="O14" s="16">
         <f>N14-H14</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="P14" s="40">
         <f>$F14/(1-$D$4-$P$9)</f>
-        <v>129.0796373866834</v>
+        <v>157.47715761175374</v>
       </c>
       <c r="Q14" s="41">
         <f>P14*$D$4</f>
-        <v>45.177873085339186</v>
+        <v>55.117005164113806</v>
       </c>
       <c r="R14" s="42">
         <f>P14-$F14-Q14</f>
-        <v>38.723891216005015</v>
+        <v>47.24314728352613</v>
       </c>
       <c r="S14" s="43">
         <f>R14/P14</f>
-        <v>0.29999999999999993</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T14" s="40">
         <f>P14*$D$6</f>
-        <v>180.71149234135675</v>
+        <v>220.46802065645522</v>
       </c>
       <c r="U14" s="40">
         <f>$F14/(1-$D$4-$U$9)</f>
-        <v>112.94468271334797</v>
+        <v>137.79251291028453</v>
       </c>
       <c r="V14" s="41">
         <f>U14*$D$4</f>
-        <v>39.53063894967179</v>
+        <v>48.227379518599584</v>
       </c>
       <c r="W14" s="42">
         <f>U14-$F14-V14</f>
-        <v>28.236170678336997</v>
+        <v>34.44812822757114</v>
       </c>
       <c r="X14" s="43">
         <f>W14/U14</f>
@@ -5084,47 +5133,50 @@
       </c>
       <c r="Y14" s="40">
         <f>U14*$D$6</f>
-        <v>158.12255579868716</v>
+        <v>192.90951807439833</v>
       </c>
       <c r="Z14" s="40">
         <f>$F14/(1-$D$4-$Z$9)</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="AA14" s="41">
         <f>Z14*$D$4</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="AB14" s="42">
         <f>Z14-$F14-AA14</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="AC14" s="43">
         <f>AB14/Z14</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="AD14" s="40">
         <f>Z14*$D$6</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="AE14" s="40">
         <f>$F14/(1-$D$4-$AE$9)</f>
-        <v>90.35574617067839</v>
+        <v>110.23401032822763</v>
       </c>
       <c r="AF14" s="41">
         <f>AE14*$D$4</f>
-        <v>31.624511159737434</v>
+        <v>38.581903614879664</v>
       </c>
       <c r="AG14" s="42">
         <f>AE14-$F14-AF14</f>
-        <v>13.55336192560176</v>
+        <v>16.53510154923415</v>
       </c>
       <c r="AH14" s="43">
         <f>AG14/AE14</f>
-        <v>0.15000000000000002</v>
+        <v>0.15000000000000005</v>
       </c>
       <c r="AI14" s="40">
         <f>AE14*$D$6</f>
-        <v>126.49804463894974</v>
+        <v>154.32761445951866</v>
+      </c>
+      <c r="AL14" s="24" t="n">
+        <v>0.8823803336980306</v>
       </c>
     </row>
     <row r="15" ht="43.5" customHeight="1" s="71">
@@ -5144,80 +5196,81 @@
       <c r="D15" s="7" t="n">
         <v>113</v>
       </c>
-      <c r="E15" s="24" t="n">
-        <v>0.8823803336980306</v>
+      <c r="E15" s="24">
+        <f>AL15*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>1.0765040071115979</v>
       </c>
       <c r="F15" s="8">
         <f>IF(AND(ISNUMBER(E15),ISNUMBER($D$8)),E15*$D$3,NA())</f>
-        <v>45.17787308533919</v>
+        <v>55.11700516411381</v>
       </c>
       <c r="G15" s="9">
         <f>F15/$D$8</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="H15" s="10">
         <f>G15*$D$4</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="I15" s="11">
         <f>G15-F15-H15</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="J15" s="12">
         <f>I15/G15</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="K15" s="13">
         <f>G15*$D$6</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="L15" s="14">
         <f>F15/(1-$D$4)</f>
-        <v>69.50442013129107</v>
+        <v>84.79539256017509</v>
       </c>
       <c r="M15" s="14">
         <f>L15*$D$6</f>
-        <v>97.30618818380749</v>
+        <v>118.71354958424511</v>
       </c>
       <c r="N15" s="15">
         <f>G15-F15</f>
-        <v>55.21740043763679</v>
+        <v>67.36522853391688</v>
       </c>
       <c r="O15" s="16">
         <f>N15-H15</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="P15" s="40">
         <f>$F15/(1-$D$4-$P$9)</f>
-        <v>129.0796373866834</v>
+        <v>157.47715761175374</v>
       </c>
       <c r="Q15" s="41">
         <f>P15*$D$4</f>
-        <v>45.177873085339186</v>
+        <v>55.117005164113806</v>
       </c>
       <c r="R15" s="42">
         <f>P15-$F15-Q15</f>
-        <v>38.723891216005015</v>
+        <v>47.24314728352613</v>
       </c>
       <c r="S15" s="43">
         <f>R15/P15</f>
-        <v>0.29999999999999993</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T15" s="40">
         <f>P15*$D$6</f>
-        <v>180.71149234135675</v>
+        <v>220.46802065645522</v>
       </c>
       <c r="U15" s="40">
         <f>$F15/(1-$D$4-$U$9)</f>
-        <v>112.94468271334797</v>
+        <v>137.79251291028453</v>
       </c>
       <c r="V15" s="41">
         <f>U15*$D$4</f>
-        <v>39.53063894967179</v>
+        <v>48.227379518599584</v>
       </c>
       <c r="W15" s="42">
         <f>U15-$F15-V15</f>
-        <v>28.236170678336997</v>
+        <v>34.44812822757114</v>
       </c>
       <c r="X15" s="43">
         <f>W15/U15</f>
@@ -5225,47 +5278,50 @@
       </c>
       <c r="Y15" s="40">
         <f>U15*$D$6</f>
-        <v>158.12255579868716</v>
+        <v>192.90951807439833</v>
       </c>
       <c r="Z15" s="40">
         <f>$F15/(1-$D$4-$Z$9)</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="AA15" s="41">
         <f>Z15*$D$4</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="AB15" s="42">
         <f>Z15-$F15-AA15</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="AC15" s="43">
         <f>AB15/Z15</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="AD15" s="40">
         <f>Z15*$D$6</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="AE15" s="40">
         <f>$F15/(1-$D$4-$AE$9)</f>
-        <v>90.35574617067839</v>
+        <v>110.23401032822763</v>
       </c>
       <c r="AF15" s="41">
         <f>AE15*$D$4</f>
-        <v>31.624511159737434</v>
+        <v>38.581903614879664</v>
       </c>
       <c r="AG15" s="42">
         <f>AE15-$F15-AF15</f>
-        <v>13.55336192560176</v>
+        <v>16.53510154923415</v>
       </c>
       <c r="AH15" s="43">
         <f>AG15/AE15</f>
-        <v>0.15000000000000002</v>
+        <v>0.15000000000000005</v>
       </c>
       <c r="AI15" s="40">
         <f>AE15*$D$6</f>
-        <v>126.49804463894974</v>
+        <v>154.32761445951866</v>
+      </c>
+      <c r="AL15" s="24" t="n">
+        <v>0.8823803336980306</v>
       </c>
     </row>
     <row r="16" ht="43.5" customHeight="1" s="71">
@@ -5285,80 +5341,81 @@
       <c r="D16" s="7" t="n">
         <v>113</v>
       </c>
-      <c r="E16" s="24" t="n">
-        <v>0.8823803336980306</v>
+      <c r="E16" s="24">
+        <f>AL16*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>1.0765040071115979</v>
       </c>
       <c r="F16" s="8">
         <f>IF(AND(ISNUMBER(E16),ISNUMBER($D$8)),E16*$D$3,NA())</f>
-        <v>45.17787308533919</v>
+        <v>55.11700516411381</v>
       </c>
       <c r="G16" s="9">
         <f>F16/$D$8</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="H16" s="10">
         <f>G16*$D$4</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="I16" s="11">
         <f>G16-F16-H16</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="J16" s="12">
         <f>I16/G16</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="K16" s="13">
         <f>G16*$D$6</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="L16" s="14">
         <f>F16/(1-$D$4)</f>
-        <v>69.50442013129107</v>
+        <v>84.79539256017509</v>
       </c>
       <c r="M16" s="14">
         <f>L16*$D$6</f>
-        <v>97.30618818380749</v>
+        <v>118.71354958424511</v>
       </c>
       <c r="N16" s="15">
         <f>G16-F16</f>
-        <v>55.21740043763679</v>
+        <v>67.36522853391688</v>
       </c>
       <c r="O16" s="16">
         <f>N16-H16</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="P16" s="40">
         <f>$F16/(1-$D$4-$P$9)</f>
-        <v>129.0796373866834</v>
+        <v>157.47715761175374</v>
       </c>
       <c r="Q16" s="41">
         <f>P16*$D$4</f>
-        <v>45.177873085339186</v>
+        <v>55.117005164113806</v>
       </c>
       <c r="R16" s="42">
         <f>P16-$F16-Q16</f>
-        <v>38.723891216005015</v>
+        <v>47.24314728352613</v>
       </c>
       <c r="S16" s="43">
         <f>R16/P16</f>
-        <v>0.29999999999999993</v>
+        <v>0.30000000000000004</v>
       </c>
       <c r="T16" s="40">
         <f>P16*$D$6</f>
-        <v>180.71149234135675</v>
+        <v>220.46802065645522</v>
       </c>
       <c r="U16" s="40">
         <f>$F16/(1-$D$4-$U$9)</f>
-        <v>112.94468271334797</v>
+        <v>137.79251291028453</v>
       </c>
       <c r="V16" s="41">
         <f>U16*$D$4</f>
-        <v>39.53063894967179</v>
+        <v>48.227379518599584</v>
       </c>
       <c r="W16" s="42">
         <f>U16-$F16-V16</f>
-        <v>28.236170678336997</v>
+        <v>34.44812822757114</v>
       </c>
       <c r="X16" s="43">
         <f>W16/U16</f>
@@ -5366,47 +5423,50 @@
       </c>
       <c r="Y16" s="40">
         <f>U16*$D$6</f>
-        <v>158.12255579868716</v>
+        <v>192.90951807439833</v>
       </c>
       <c r="Z16" s="40">
         <f>$F16/(1-$D$4-$Z$9)</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="AA16" s="41">
         <f>Z16*$D$4</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="AB16" s="42">
         <f>Z16-$F16-AA16</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="AC16" s="43">
         <f>AB16/Z16</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="AD16" s="40">
         <f>Z16*$D$6</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="AE16" s="40">
         <f>$F16/(1-$D$4-$AE$9)</f>
-        <v>90.35574617067839</v>
+        <v>110.23401032822763</v>
       </c>
       <c r="AF16" s="41">
         <f>AE16*$D$4</f>
-        <v>31.624511159737434</v>
+        <v>38.581903614879664</v>
       </c>
       <c r="AG16" s="42">
         <f>AE16-$F16-AF16</f>
-        <v>13.55336192560176</v>
+        <v>16.53510154923415</v>
       </c>
       <c r="AH16" s="43">
         <f>AG16/AE16</f>
-        <v>0.15000000000000002</v>
+        <v>0.15000000000000005</v>
       </c>
       <c r="AI16" s="40">
         <f>AE16*$D$6</f>
-        <v>126.49804463894974</v>
+        <v>154.32761445951866</v>
+      </c>
+      <c r="AL16" s="24" t="n">
+        <v>0.8823803336980306</v>
       </c>
     </row>
     <row r="17"/>
@@ -5491,27 +5551,27 @@
       <c r="E22" s="65" t="n"/>
       <c r="F22" s="29">
         <f>E11</f>
-        <v>1.018131154266958</v>
+        <v>1.2421200082056887</v>
       </c>
       <c r="G22" s="29">
         <f>E12</f>
-        <v>1.018131154266958</v>
+        <v>1.2421200082056887</v>
       </c>
       <c r="H22" s="29">
         <f>E13</f>
-        <v>0.882380333698031</v>
+        <v>1.0765040071115979</v>
       </c>
       <c r="I22" s="29">
         <f>E14</f>
-        <v>0.882380333698031</v>
+        <v>1.0765040071115979</v>
       </c>
       <c r="J22" s="29">
         <f>E15</f>
-        <v>0.882380333698031</v>
+        <v>1.0765040071115979</v>
       </c>
       <c r="K22" s="29">
         <f>E16</f>
-        <v>0.882380333698031</v>
+        <v>1.0765040071115979</v>
       </c>
     </row>
     <row r="23" ht="31.05" customHeight="1" s="71">
@@ -5573,27 +5633,27 @@
       <c r="E24" s="65" t="n"/>
       <c r="F24" s="31">
         <f>F11</f>
-        <v>52.12831509846825</v>
+        <v>63.596544420131266</v>
       </c>
       <c r="G24" s="31">
         <f>F12</f>
-        <v>52.12831509846825</v>
+        <v>63.596544420131266</v>
       </c>
       <c r="H24" s="31">
         <f>F13</f>
-        <v>45.17787308533919</v>
+        <v>55.11700516411381</v>
       </c>
       <c r="I24" s="31">
         <f>F14</f>
-        <v>45.17787308533919</v>
+        <v>55.11700516411381</v>
       </c>
       <c r="J24" s="31">
         <f>F15</f>
-        <v>45.17787308533919</v>
+        <v>55.11700516411381</v>
       </c>
       <c r="K24" s="31">
         <f>F16</f>
-        <v>45.17787308533919</v>
+        <v>55.11700516411381</v>
       </c>
     </row>
     <row r="25" ht="31.05" customHeight="1" s="71">
@@ -5813,27 +5873,27 @@
       <c r="E30" s="65" t="n"/>
       <c r="F30" s="34">
         <f>G11</f>
-        <v>115.84070021881833</v>
+        <v>141.32565426695837</v>
       </c>
       <c r="G30" s="34">
         <f>G12</f>
-        <v>115.84070021881833</v>
+        <v>141.32565426695837</v>
       </c>
       <c r="H30" s="34">
         <f>G13</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="I30" s="34">
         <f>G14</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="J30" s="34">
         <f>G15</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
       <c r="K30" s="34">
         <f>G16</f>
-        <v>100.39527352297598</v>
+        <v>122.4822336980307</v>
       </c>
     </row>
     <row r="31" ht="31.05" customHeight="1" s="71">
@@ -5854,27 +5914,27 @@
       <c r="E31" s="65" t="n"/>
       <c r="F31" s="31">
         <f>N11</f>
-        <v>63.71238512035008</v>
+        <v>77.7291098468271</v>
       </c>
       <c r="G31" s="31">
         <f>N12</f>
-        <v>63.71238512035008</v>
+        <v>77.7291098468271</v>
       </c>
       <c r="H31" s="31">
         <f>N13</f>
-        <v>55.21740043763679</v>
+        <v>67.36522853391688</v>
       </c>
       <c r="I31" s="31">
         <f>N14</f>
-        <v>55.21740043763679</v>
+        <v>67.36522853391688</v>
       </c>
       <c r="J31" s="31">
         <f>N15</f>
-        <v>55.21740043763679</v>
+        <v>67.36522853391688</v>
       </c>
       <c r="K31" s="31">
         <f>N16</f>
-        <v>55.21740043763679</v>
+        <v>67.36522853391688</v>
       </c>
     </row>
     <row r="32" ht="31.05" customHeight="1" s="71">
@@ -5895,27 +5955,27 @@
       <c r="E32" s="65" t="n"/>
       <c r="F32" s="31">
         <f>H11</f>
-        <v>40.544245076586414</v>
+        <v>49.463978993435425</v>
       </c>
       <c r="G32" s="31">
         <f>H12</f>
-        <v>40.544245076586414</v>
+        <v>49.463978993435425</v>
       </c>
       <c r="H32" s="31">
         <f>H13</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="I32" s="31">
         <f>H14</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="J32" s="31">
         <f>H15</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
       <c r="K32" s="31">
         <f>H16</f>
-        <v>35.13834573304159</v>
+        <v>42.86878179431074</v>
       </c>
     </row>
     <row r="33" ht="31.05" customHeight="1" s="71">
@@ -5936,27 +5996,27 @@
       <c r="E33" s="65" t="n"/>
       <c r="F33" s="36">
         <f>I11</f>
-        <v>23.168140043763664</v>
+        <v>28.265130853391675</v>
       </c>
       <c r="G33" s="36">
         <f>I12</f>
-        <v>23.168140043763664</v>
+        <v>28.265130853391675</v>
       </c>
       <c r="H33" s="36">
         <f>I13</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="I33" s="36">
         <f>I14</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="J33" s="36">
         <f>I15</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
       <c r="K33" s="36">
         <f>I16</f>
-        <v>20.0790547045952</v>
+        <v>24.496446739606135</v>
       </c>
     </row>
     <row r="34" ht="31.05" customHeight="1" s="71">
@@ -5977,27 +6037,27 @@
       <c r="E34" s="65" t="n"/>
       <c r="F34" s="37">
         <f>J11</f>
-        <v>0.19999999999999998</v>
+        <v>0.2</v>
       </c>
       <c r="G34" s="37">
         <f>J12</f>
-        <v>0.19999999999999998</v>
+        <v>0.2</v>
       </c>
       <c r="H34" s="37">
         <f>J13</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="I34" s="37">
         <f>J14</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="J34" s="37">
         <f>J15</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="K34" s="37">
         <f>J16</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999996</v>
       </c>
     </row>
     <row r="35" ht="31.05" customHeight="1" s="71">
@@ -6100,27 +6160,27 @@
       <c r="E37" s="65" t="n"/>
       <c r="F37" s="34">
         <f>K11</f>
-        <v>162.17698030634565</v>
+        <v>197.8559159737417</v>
       </c>
       <c r="G37" s="34">
         <f>K12</f>
-        <v>162.17698030634565</v>
+        <v>197.8559159737417</v>
       </c>
       <c r="H37" s="34">
         <f>K13</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="I37" s="34">
         <f>K14</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="J37" s="34">
         <f>K15</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
       <c r="K37" s="34">
         <f>K16</f>
-        <v>140.55338293216636</v>
+        <v>171.47512717724297</v>
       </c>
     </row>
     <row r="38" ht="31.05" customHeight="1" s="71">
@@ -6141,27 +6201,27 @@
       <c r="E38" s="65" t="n"/>
       <c r="F38" s="31">
         <f>L11</f>
-        <v>80.19740784379731</v>
+        <v>97.84083756943271</v>
       </c>
       <c r="G38" s="31">
         <f>L12</f>
-        <v>80.19740784379731</v>
+        <v>97.84083756943271</v>
       </c>
       <c r="H38" s="31">
         <f>L13</f>
-        <v>69.50442013129107</v>
+        <v>84.79539256017509</v>
       </c>
       <c r="I38" s="31">
         <f>L14</f>
-        <v>69.50442013129107</v>
+        <v>84.79539256017509</v>
       </c>
       <c r="J38" s="31">
         <f>L15</f>
-        <v>69.50442013129107</v>
+        <v>84.79539256017509</v>
       </c>
       <c r="K38" s="31">
         <f>L16</f>
-        <v>69.50442013129107</v>
+        <v>84.79539256017509</v>
       </c>
     </row>
     <row r="39" ht="31.05" customHeight="1" s="71">
@@ -6182,27 +6242,27 @@
       <c r="E39" s="65" t="n"/>
       <c r="F39" s="31">
         <f>M11</f>
-        <v>112.27637098131622</v>
+        <v>136.9771725972058</v>
       </c>
       <c r="G39" s="31">
         <f>M12</f>
-        <v>112.27637098131622</v>
+        <v>136.9771725972058</v>
       </c>
       <c r="H39" s="31">
         <f>M13</f>
-        <v>97.30618818380749</v>
+        <v>118.71354958424511</v>
       </c>
       <c r="I39" s="31">
         <f>M14</f>
-        <v>97.30618818380749</v>
+        <v>118.71354958424511</v>
       </c>
       <c r="J39" s="31">
         <f>M15</f>
-        <v>97.30618818380749</v>
+        <v>118.71354958424511</v>
       </c>
       <c r="K39" s="31">
         <f>M16</f>
-        <v>97.30618818380749</v>
+        <v>118.71354958424511</v>
       </c>
     </row>
   </sheetData>
@@ -6839,7 +6899,7 @@
         </is>
       </c>
       <c r="B24" s="149">
-        <f>'Model 6 pallets'!E13</f>
+        <f>'Model 6 pallets'!AL13</f>
         <v>1.134046875</v>
       </c>
       <c r="C24" s="182">
@@ -6854,7 +6914,7 @@
         </is>
       </c>
       <c r="B25" s="149">
-        <f>'Model 6 pallets'!E11</f>
+        <f>'Model 6 pallets'!AL11</f>
         <v>1.308515625</v>
       </c>
       <c r="C25" s="182">
@@ -7435,7 +7495,7 @@
         </is>
       </c>
       <c r="B23" s="149">
-        <f>'Model 33 pallets'!E13</f>
+        <f>'Model 33 pallets'!AL13</f>
         <v>0.882380333698031</v>
       </c>
       <c r="C23" s="182">
@@ -7450,7 +7510,7 @@
         </is>
       </c>
       <c r="B24" s="149">
-        <f>'Model 33 pallets'!E11</f>
+        <f>'Model 33 pallets'!AL11</f>
         <v>1.018131154266958</v>
       </c>
       <c r="C24" s="182">

</xml_diff>

<commit_message>
Internal model: cost uplift 12.5 %, bonus 35 %, margin auto-offsets the uplift (ask and shelf unchanged)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
+++ b/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
@@ -793,7 +793,7 @@
     <xf numFmtId="0" fontId="11" fillId="19" borderId="10"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="10"/>
   </cellStyleXfs>
-  <cellXfs count="184">
+  <cellXfs count="185">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1294,6 +1294,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="184" fontId="8" fillId="18" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="172" fontId="36" fillId="23" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="176" fontId="22" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1696,11 +1699,11 @@
       </c>
       <c r="G6" s="176">
         <f>F6*'Price 120 UAH - 33 pallets'!G14</f>
-        <v>9.939132078774618</v>
+        <v>5.6472341356673965</v>
       </c>
       <c r="H6" s="177">
         <f>F6+G6</f>
-        <v>55.11700516411379</v>
+        <v>50.82510722100657</v>
       </c>
       <c r="I6" s="178">
         <f>ROUND(H6-'Price 120 UAH - 33 pallets'!C4,4)</f>
@@ -1732,11 +1735,11 @@
       </c>
       <c r="G7" s="176">
         <f>F7*'Price 120 UAH - 33 pallets'!G14</f>
-        <v>11.468229321663024</v>
+        <v>6.5160393873085365</v>
       </c>
       <c r="H7" s="177">
         <f>F7+G7</f>
-        <v>63.596544420131316</v>
+        <v>58.64435448577683</v>
       </c>
       <c r="I7" s="178">
         <f>ROUND(H7-'Price 120 UAH - 33 pallets'!C6,4)</f>
@@ -1752,7 +1755,7 @@
       </c>
       <c r="B8" s="179">
         <f>'Price 120 UAH - 33 pallets'!B19*'Price 120 UAH - 33 pallets'!F14</f>
-        <v>22.016000000000002</v>
+        <v>27.648000000000003</v>
       </c>
       <c r="C8" s="179">
         <f>('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16)/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18)*'Price 120 UAH - 33 pallets'!F14</f>
@@ -1760,23 +1763,23 @@
       </c>
       <c r="D8" s="179">
         <f>('Price 120 UAH - 33 pallets'!B19+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))*(1+'Price 120 UAH - 33 pallets'!D16)*'Price 120 UAH - 33 pallets'!B16*'Price 120 UAH - 33 pallets'!F14</f>
-        <v>4.905503030303031</v>
+        <v>6.031903030303031</v>
       </c>
       <c r="E8" s="179">
         <f>(B8+C8+D8+('Price 120 UAH - 33 pallets'!B19+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))*'Price 120 UAH - 33 pallets'!D16*'Price 120 UAH - 33 pallets'!F14)*'Price 120 UAH - 33 pallets'!C16</f>
-        <v>0.7707345454545456</v>
+        <v>0.9396945454545457</v>
       </c>
       <c r="F8" s="175">
         <f>SUM(B8:E8)</f>
-        <v>31.600116363636367</v>
+        <v>38.52747636363637</v>
       </c>
       <c r="G8" s="176">
         <f>F8*'Price 120 UAH - 33 pallets'!G14</f>
-        <v>6.952025600000001</v>
+        <v>4.815934545454546</v>
       </c>
       <c r="H8" s="177">
         <f>F8+G8</f>
-        <v>38.552141963636366</v>
+        <v>43.34341090909091</v>
       </c>
       <c r="I8" s="178">
         <f>ROUND(H8-'Price 120 UAH - 33 pallets'!C8,4)</f>
@@ -1862,11 +1865,11 @@
       </c>
       <c r="G12" s="176">
         <f>F12*'Price 120 UAH - 6 pallets'!G14</f>
-        <v>12.773904</v>
+        <v>7.2579</v>
       </c>
       <c r="H12" s="177">
         <f>F12+G12</f>
-        <v>70.837104</v>
+        <v>65.3211</v>
       </c>
       <c r="I12" s="178">
         <f>ROUND(H12-'Price 120 UAH - 6 pallets'!C4,4)</f>
@@ -1898,11 +1901,11 @@
       </c>
       <c r="G13" s="176">
         <f>F13*'Price 120 UAH - 6 pallets'!G14</f>
-        <v>14.739120000000002</v>
+        <v>8.374500000000001</v>
       </c>
       <c r="H13" s="177">
         <f>F13+G13</f>
-        <v>81.73512000000001</v>
+        <v>75.3705</v>
       </c>
       <c r="I13" s="178">
         <f>ROUND(H13-'Price 120 UAH - 6 pallets'!C6,4)</f>
@@ -1918,7 +1921,7 @@
       </c>
       <c r="B14" s="179">
         <f>'Price 120 UAH - 6 pallets'!B20*'Price 120 UAH - 6 pallets'!F14</f>
-        <v>10.752</v>
+        <v>16.384</v>
       </c>
       <c r="C14" s="179">
         <f>('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16)/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18)*'Price 120 UAH - 6 pallets'!F14</f>
@@ -1926,23 +1929,23 @@
       </c>
       <c r="D14" s="179">
         <f>('Price 120 UAH - 6 pallets'!B20+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))*(1+'Price 120 UAH - 6 pallets'!D16)*'Price 120 UAH - 6 pallets'!B16*'Price 120 UAH - 6 pallets'!F14</f>
-        <v>4.091733333333333</v>
+        <v>5.218133333333333</v>
       </c>
       <c r="E14" s="179">
         <f>(B14+C14+D14+('Price 120 UAH - 6 pallets'!B20+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))*'Price 120 UAH - 6 pallets'!D16*'Price 120 UAH - 6 pallets'!F14)*'Price 120 UAH - 6 pallets'!C16</f>
-        <v>0.7617600000000001</v>
+        <v>0.93072</v>
       </c>
       <c r="F14" s="175">
         <f>SUM(B14:E14)</f>
-        <v>31.23216</v>
+        <v>38.15952</v>
       </c>
       <c r="G14" s="176">
         <f>F14*'Price 120 UAH - 6 pallets'!G14</f>
-        <v>6.8710752</v>
+        <v>4.76994</v>
       </c>
       <c r="H14" s="177">
         <f>F14+G14</f>
-        <v>38.1032352</v>
+        <v>42.92946</v>
       </c>
       <c r="I14" s="178">
         <f>ROUND(H14-'Price 120 UAH - 6 pallets'!C8,4)</f>
@@ -2075,12 +2078,13 @@
         </is>
       </c>
       <c r="C5" s="63" t="n"/>
-      <c r="D5" s="18" t="n">
-        <v>0.2</v>
+      <c r="D5" s="18">
+        <f>'Price 120 UAH - 6 pallets'!C14</f>
+        <v>0.14375000000000004</v>
       </c>
       <c r="E5" s="68" t="str">
         <f>ROUND(D5*100,0)&amp;"% = (partner price − landed cost − bonus) / full partner price."</f>
-        <v>20% = (partner price − landed cost − bonus) / full partner price.</v>
+        <v>14% = (partner price − landed cost − bonus) / full partner price.</v>
       </c>
       <c r="F5" s="69" t="n"/>
       <c r="G5" s="69" t="n"/>
@@ -2144,11 +2148,11 @@
       <c r="C8" s="77" t="n"/>
       <c r="D8" s="23">
         <f>IF(AND(COUNT(D3:D6)=4,D3&gt;0,D4&gt;=0,D5&gt;=0,D4+D5&lt;1,D6&gt;0),1-D4-D5,NA())</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="E8" s="79" t="str">
         <f>"100% − bonus − margin. Current terms: 100% − "&amp;ROUND(D4*100,0)&amp;"% − "&amp;ROUND(D5*100,0)&amp;"% = "&amp;ROUND(D8*100,0)&amp;"%."</f>
-        <v>100% − bonus − margin. Current terms: 100% − 35% − 20% = 45%.</v>
+        <v>100% − bonus − margin. Current terms: 100% − 35% − 14% = 51%.</v>
       </c>
       <c r="F8" s="69" t="n"/>
       <c r="G8" s="69" t="n"/>
@@ -2427,127 +2431,127 @@
       </c>
       <c r="E11" s="24">
         <f>AL11*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
-        <v>1.5963890625000001</v>
+        <v>1.472080078125</v>
       </c>
       <c r="F11" s="8">
         <f>IF(AND(ISNUMBER(E11),ISNUMBER($D$8)),E11*$D$3,NA())</f>
-        <v>81.73512000000001</v>
+        <v>75.3705</v>
       </c>
       <c r="G11" s="9">
         <f>F11/$D$8</f>
-        <v>181.63360000000003</v>
+        <v>148.88000000000002</v>
       </c>
       <c r="H11" s="10">
         <f>G11*$D$4</f>
-        <v>63.571760000000005</v>
+        <v>52.108000000000004</v>
       </c>
       <c r="I11" s="11">
         <f>G11-F11-H11</f>
-        <v>36.326720000000016</v>
+        <v>21.401500000000013</v>
       </c>
       <c r="J11" s="12">
         <f>I11/G11</f>
-        <v>0.20000000000000007</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="K11" s="13">
         <f>G11*$D$6</f>
-        <v>254.28704000000002</v>
+        <v>208.43200000000002</v>
       </c>
       <c r="L11" s="14">
         <f>F11/(1-$D$4)</f>
-        <v>125.74633846153847</v>
+        <v>115.9546153846154</v>
       </c>
       <c r="M11" s="14">
         <f>L11*$D$6</f>
-        <v>176.04487384615385</v>
+        <v>162.33646153846155</v>
       </c>
       <c r="N11" s="15">
         <f>G11-F11</f>
-        <v>99.89848000000002</v>
+        <v>73.50950000000002</v>
       </c>
       <c r="O11" s="16">
         <f>N11-H11</f>
-        <v>36.326720000000016</v>
+        <v>21.401500000000013</v>
       </c>
       <c r="P11" s="40">
         <f>$F11/(1-$D$4-$P$9)</f>
-        <v>233.52891428571428</v>
+        <v>215.34428571428572</v>
       </c>
       <c r="Q11" s="41">
         <f>P11*$D$4</f>
-        <v>81.73512</v>
+        <v>75.37049999999999</v>
       </c>
       <c r="R11" s="42">
         <f>P11-$F11-Q11</f>
-        <v>70.05867428571429</v>
+        <v>64.60328571428573</v>
       </c>
       <c r="S11" s="43">
         <f>R11/P11</f>
-        <v>0.30000000000000004</v>
+        <v>0.3000000000000001</v>
       </c>
       <c r="T11" s="40">
         <f>P11*$D$6</f>
-        <v>326.94048</v>
+        <v>301.48199999999997</v>
       </c>
       <c r="U11" s="40">
         <f>$F11/(1-$D$4-$U$9)</f>
-        <v>204.33780000000002</v>
+        <v>188.42625</v>
       </c>
       <c r="V11" s="41">
         <f>U11*$D$4</f>
-        <v>71.51823</v>
+        <v>65.9491875</v>
       </c>
       <c r="W11" s="42">
         <f>U11-$F11-V11</f>
-        <v>51.084450000000004</v>
+        <v>47.10656250000001</v>
       </c>
       <c r="X11" s="43">
         <f>W11/U11</f>
-        <v>0.25</v>
+        <v>0.25000000000000006</v>
       </c>
       <c r="Y11" s="40">
         <f>U11*$D$6</f>
-        <v>286.07292</v>
+        <v>263.79675</v>
       </c>
       <c r="Z11" s="40">
         <f>$F11/(1-$D$4-$Z$9)</f>
-        <v>181.63360000000003</v>
+        <v>167.49</v>
       </c>
       <c r="AA11" s="41">
         <f>Z11*$D$4</f>
-        <v>63.571760000000005</v>
+        <v>58.6215</v>
       </c>
       <c r="AB11" s="42">
         <f>Z11-$F11-AA11</f>
-        <v>36.326720000000016</v>
+        <v>33.498000000000005</v>
       </c>
       <c r="AC11" s="43">
         <f>AB11/Z11</f>
-        <v>0.20000000000000007</v>
+        <v>0.2</v>
       </c>
       <c r="AD11" s="40">
         <f>Z11*$D$6</f>
-        <v>254.28704000000002</v>
+        <v>234.486</v>
       </c>
       <c r="AE11" s="40">
         <f>$F11/(1-$D$4-$AE$9)</f>
-        <v>163.47024000000002</v>
+        <v>150.741</v>
       </c>
       <c r="AF11" s="41">
         <f>AE11*$D$4</f>
-        <v>57.214584</v>
+        <v>52.759350000000005</v>
       </c>
       <c r="AG11" s="42">
         <f>AE11-$F11-AF11</f>
-        <v>24.520536000000007</v>
+        <v>22.611150000000002</v>
       </c>
       <c r="AH11" s="43">
         <f>AG11/AE11</f>
-        <v>0.15000000000000002</v>
+        <v>0.15</v>
       </c>
       <c r="AI11" s="40">
         <f>AE11*$D$6</f>
-        <v>228.858336</v>
+        <v>211.03740000000002</v>
       </c>
       <c r="AL11" s="24" t="n">
         <v>1.308515625</v>
@@ -2572,127 +2576,127 @@
       </c>
       <c r="E12" s="24">
         <f>AL12*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
-        <v>1.5963890625000001</v>
+        <v>1.472080078125</v>
       </c>
       <c r="F12" s="8">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER($D$8)),E12*$D$3,NA())</f>
-        <v>81.73512000000001</v>
+        <v>75.3705</v>
       </c>
       <c r="G12" s="9">
         <f>F12/$D$8</f>
-        <v>181.63360000000003</v>
+        <v>148.88000000000002</v>
       </c>
       <c r="H12" s="10">
         <f>G12*$D$4</f>
-        <v>63.571760000000005</v>
+        <v>52.108000000000004</v>
       </c>
       <c r="I12" s="11">
         <f>G12-F12-H12</f>
-        <v>36.326720000000016</v>
+        <v>21.401500000000013</v>
       </c>
       <c r="J12" s="12">
         <f>I12/G12</f>
-        <v>0.20000000000000007</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="K12" s="13">
         <f>G12*$D$6</f>
-        <v>254.28704000000002</v>
+        <v>208.43200000000002</v>
       </c>
       <c r="L12" s="14">
         <f>F12/(1-$D$4)</f>
-        <v>125.74633846153847</v>
+        <v>115.9546153846154</v>
       </c>
       <c r="M12" s="14">
         <f>L12*$D$6</f>
-        <v>176.04487384615385</v>
+        <v>162.33646153846155</v>
       </c>
       <c r="N12" s="15">
         <f>G12-F12</f>
-        <v>99.89848000000002</v>
+        <v>73.50950000000002</v>
       </c>
       <c r="O12" s="16">
         <f>N12-H12</f>
-        <v>36.326720000000016</v>
+        <v>21.401500000000013</v>
       </c>
       <c r="P12" s="40">
         <f>$F12/(1-$D$4-$P$9)</f>
-        <v>233.52891428571428</v>
+        <v>215.34428571428572</v>
       </c>
       <c r="Q12" s="41">
         <f>P12*$D$4</f>
-        <v>81.73512</v>
+        <v>75.37049999999999</v>
       </c>
       <c r="R12" s="42">
         <f>P12-$F12-Q12</f>
-        <v>70.05867428571429</v>
+        <v>64.60328571428573</v>
       </c>
       <c r="S12" s="43">
         <f>R12/P12</f>
-        <v>0.30000000000000004</v>
+        <v>0.3000000000000001</v>
       </c>
       <c r="T12" s="40">
         <f>P12*$D$6</f>
-        <v>326.94048</v>
+        <v>301.48199999999997</v>
       </c>
       <c r="U12" s="40">
         <f>$F12/(1-$D$4-$U$9)</f>
-        <v>204.33780000000002</v>
+        <v>188.42625</v>
       </c>
       <c r="V12" s="41">
         <f>U12*$D$4</f>
-        <v>71.51823</v>
+        <v>65.9491875</v>
       </c>
       <c r="W12" s="42">
         <f>U12-$F12-V12</f>
-        <v>51.084450000000004</v>
+        <v>47.10656250000001</v>
       </c>
       <c r="X12" s="43">
         <f>W12/U12</f>
-        <v>0.25</v>
+        <v>0.25000000000000006</v>
       </c>
       <c r="Y12" s="40">
         <f>U12*$D$6</f>
-        <v>286.07292</v>
+        <v>263.79675</v>
       </c>
       <c r="Z12" s="40">
         <f>$F12/(1-$D$4-$Z$9)</f>
-        <v>181.63360000000003</v>
+        <v>167.49</v>
       </c>
       <c r="AA12" s="41">
         <f>Z12*$D$4</f>
-        <v>63.571760000000005</v>
+        <v>58.6215</v>
       </c>
       <c r="AB12" s="42">
         <f>Z12-$F12-AA12</f>
-        <v>36.326720000000016</v>
+        <v>33.498000000000005</v>
       </c>
       <c r="AC12" s="43">
         <f>AB12/Z12</f>
-        <v>0.20000000000000007</v>
+        <v>0.2</v>
       </c>
       <c r="AD12" s="40">
         <f>Z12*$D$6</f>
-        <v>254.28704000000002</v>
+        <v>234.486</v>
       </c>
       <c r="AE12" s="40">
         <f>$F12/(1-$D$4-$AE$9)</f>
-        <v>163.47024000000002</v>
+        <v>150.741</v>
       </c>
       <c r="AF12" s="41">
         <f>AE12*$D$4</f>
-        <v>57.214584</v>
+        <v>52.759350000000005</v>
       </c>
       <c r="AG12" s="42">
         <f>AE12-$F12-AF12</f>
-        <v>24.520536000000007</v>
+        <v>22.611150000000002</v>
       </c>
       <c r="AH12" s="43">
         <f>AG12/AE12</f>
-        <v>0.15000000000000002</v>
+        <v>0.15</v>
       </c>
       <c r="AI12" s="40">
         <f>AE12*$D$6</f>
-        <v>228.858336</v>
+        <v>211.03740000000002</v>
       </c>
       <c r="AL12" s="24" t="n">
         <v>1.308515625</v>
@@ -2717,127 +2721,127 @@
       </c>
       <c r="E13" s="24">
         <f>AL13*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
-        <v>1.3835371874999998</v>
+        <v>1.2758027343749998</v>
       </c>
       <c r="F13" s="8">
         <f>IF(AND(ISNUMBER(E13),ISNUMBER($D$8)),E13*$D$3,NA())</f>
-        <v>70.837104</v>
+        <v>65.32109999999999</v>
       </c>
       <c r="G13" s="9">
         <f>F13/$D$8</f>
-        <v>157.41578666666666</v>
+        <v>129.0293333333333</v>
       </c>
       <c r="H13" s="10">
         <f>G13*$D$4</f>
-        <v>55.09552533333333</v>
+        <v>45.16026666666666</v>
       </c>
       <c r="I13" s="11">
         <f>G13-F13-H13</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="J13" s="12">
         <f>I13/G13</f>
-        <v>0.20000000000000004</v>
+        <v>0.14375000000000002</v>
       </c>
       <c r="K13" s="13">
         <f>G13*$D$6</f>
-        <v>220.3821013333333</v>
+        <v>180.64106666666663</v>
       </c>
       <c r="L13" s="14">
         <f>F13/(1-$D$4)</f>
-        <v>108.98016</v>
+        <v>100.49399999999997</v>
       </c>
       <c r="M13" s="14">
         <f>L13*$D$6</f>
-        <v>152.57222399999998</v>
+        <v>140.69159999999994</v>
       </c>
       <c r="N13" s="15">
         <f>G13-F13</f>
-        <v>86.57868266666667</v>
+        <v>63.708233333333325</v>
       </c>
       <c r="O13" s="16">
         <f>N13-H13</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="P13" s="40">
         <f>$F13/(1-$D$4-$P$9)</f>
-        <v>202.39172571428568</v>
+        <v>186.63171428571422</v>
       </c>
       <c r="Q13" s="41">
         <f>P13*$D$4</f>
-        <v>70.83710399999998</v>
+        <v>65.32109999999997</v>
       </c>
       <c r="R13" s="42">
         <f>P13-$F13-Q13</f>
-        <v>60.71751771428572</v>
+        <v>55.989514285714264</v>
       </c>
       <c r="S13" s="43">
         <f>R13/P13</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T13" s="40">
         <f>P13*$D$6</f>
-        <v>283.34841599999993</v>
+        <v>261.2843999999999</v>
       </c>
       <c r="U13" s="40">
         <f>$F13/(1-$D$4-$U$9)</f>
-        <v>177.09275999999997</v>
+        <v>163.30274999999995</v>
       </c>
       <c r="V13" s="41">
         <f>U13*$D$4</f>
-        <v>61.98246599999999</v>
+        <v>57.15596249999998</v>
       </c>
       <c r="W13" s="42">
         <f>U13-$F13-V13</f>
-        <v>44.273189999999985</v>
+        <v>40.82568749999998</v>
       </c>
       <c r="X13" s="43">
         <f>W13/U13</f>
-        <v>0.24999999999999997</v>
+        <v>0.24999999999999994</v>
       </c>
       <c r="Y13" s="40">
         <f>U13*$D$6</f>
-        <v>247.92986399999995</v>
+        <v>228.62384999999992</v>
       </c>
       <c r="Z13" s="40">
         <f>$F13/(1-$D$4-$Z$9)</f>
-        <v>157.41578666666666</v>
+        <v>145.15799999999996</v>
       </c>
       <c r="AA13" s="41">
         <f>Z13*$D$4</f>
-        <v>55.09552533333333</v>
+        <v>50.80529999999998</v>
       </c>
       <c r="AB13" s="42">
         <f>Z13-$F13-AA13</f>
-        <v>31.483157333333338</v>
+        <v>29.03159999999999</v>
       </c>
       <c r="AC13" s="43">
         <f>AB13/Z13</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="AD13" s="40">
         <f>Z13*$D$6</f>
-        <v>220.3821013333333</v>
+        <v>203.22119999999993</v>
       </c>
       <c r="AE13" s="40">
         <f>$F13/(1-$D$4-$AE$9)</f>
-        <v>141.674208</v>
+        <v>130.64219999999997</v>
       </c>
       <c r="AF13" s="41">
         <f>AE13*$D$4</f>
-        <v>49.58597279999999</v>
+        <v>45.724769999999985</v>
       </c>
       <c r="AG13" s="42">
         <f>AE13-$F13-AF13</f>
-        <v>21.251131200000003</v>
+        <v>19.596330000000002</v>
       </c>
       <c r="AH13" s="43">
         <f>AG13/AE13</f>
-        <v>0.15000000000000002</v>
+        <v>0.15000000000000005</v>
       </c>
       <c r="AI13" s="40">
         <f>AE13*$D$6</f>
-        <v>198.34389119999997</v>
+        <v>182.89907999999994</v>
       </c>
       <c r="AL13" s="24" t="n">
         <v>1.134046875</v>
@@ -2862,127 +2866,127 @@
       </c>
       <c r="E14" s="24">
         <f>AL14*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
-        <v>1.3835371874999998</v>
+        <v>1.2758027343749998</v>
       </c>
       <c r="F14" s="8">
         <f>IF(AND(ISNUMBER(E14),ISNUMBER($D$8)),E14*$D$3,NA())</f>
-        <v>70.837104</v>
+        <v>65.32109999999999</v>
       </c>
       <c r="G14" s="9">
         <f>F14/$D$8</f>
-        <v>157.41578666666666</v>
+        <v>129.0293333333333</v>
       </c>
       <c r="H14" s="10">
         <f>G14*$D$4</f>
-        <v>55.09552533333333</v>
+        <v>45.16026666666666</v>
       </c>
       <c r="I14" s="11">
         <f>G14-F14-H14</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="J14" s="12">
         <f>I14/G14</f>
-        <v>0.20000000000000004</v>
+        <v>0.14375000000000002</v>
       </c>
       <c r="K14" s="13">
         <f>G14*$D$6</f>
-        <v>220.3821013333333</v>
+        <v>180.64106666666663</v>
       </c>
       <c r="L14" s="14">
         <f>F14/(1-$D$4)</f>
-        <v>108.98016</v>
+        <v>100.49399999999997</v>
       </c>
       <c r="M14" s="14">
         <f>L14*$D$6</f>
-        <v>152.57222399999998</v>
+        <v>140.69159999999994</v>
       </c>
       <c r="N14" s="15">
         <f>G14-F14</f>
-        <v>86.57868266666667</v>
+        <v>63.708233333333325</v>
       </c>
       <c r="O14" s="16">
         <f>N14-H14</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="P14" s="40">
         <f>$F14/(1-$D$4-$P$9)</f>
-        <v>202.39172571428568</v>
+        <v>186.63171428571422</v>
       </c>
       <c r="Q14" s="41">
         <f>P14*$D$4</f>
-        <v>70.83710399999998</v>
+        <v>65.32109999999997</v>
       </c>
       <c r="R14" s="42">
         <f>P14-$F14-Q14</f>
-        <v>60.71751771428572</v>
+        <v>55.989514285714264</v>
       </c>
       <c r="S14" s="43">
         <f>R14/P14</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T14" s="40">
         <f>P14*$D$6</f>
-        <v>283.34841599999993</v>
+        <v>261.2843999999999</v>
       </c>
       <c r="U14" s="40">
         <f>$F14/(1-$D$4-$U$9)</f>
-        <v>177.09275999999997</v>
+        <v>163.30274999999995</v>
       </c>
       <c r="V14" s="41">
         <f>U14*$D$4</f>
-        <v>61.98246599999999</v>
+        <v>57.15596249999998</v>
       </c>
       <c r="W14" s="42">
         <f>U14-$F14-V14</f>
-        <v>44.273189999999985</v>
+        <v>40.82568749999998</v>
       </c>
       <c r="X14" s="43">
         <f>W14/U14</f>
-        <v>0.24999999999999997</v>
+        <v>0.24999999999999994</v>
       </c>
       <c r="Y14" s="40">
         <f>U14*$D$6</f>
-        <v>247.92986399999995</v>
+        <v>228.62384999999992</v>
       </c>
       <c r="Z14" s="40">
         <f>$F14/(1-$D$4-$Z$9)</f>
-        <v>157.41578666666666</v>
+        <v>145.15799999999996</v>
       </c>
       <c r="AA14" s="41">
         <f>Z14*$D$4</f>
-        <v>55.09552533333333</v>
+        <v>50.80529999999998</v>
       </c>
       <c r="AB14" s="42">
         <f>Z14-$F14-AA14</f>
-        <v>31.483157333333338</v>
+        <v>29.03159999999999</v>
       </c>
       <c r="AC14" s="43">
         <f>AB14/Z14</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="AD14" s="40">
         <f>Z14*$D$6</f>
-        <v>220.3821013333333</v>
+        <v>203.22119999999993</v>
       </c>
       <c r="AE14" s="40">
         <f>$F14/(1-$D$4-$AE$9)</f>
-        <v>141.674208</v>
+        <v>130.64219999999997</v>
       </c>
       <c r="AF14" s="41">
         <f>AE14*$D$4</f>
-        <v>49.58597279999999</v>
+        <v>45.724769999999985</v>
       </c>
       <c r="AG14" s="42">
         <f>AE14-$F14-AF14</f>
-        <v>21.251131200000003</v>
+        <v>19.596330000000002</v>
       </c>
       <c r="AH14" s="43">
         <f>AG14/AE14</f>
-        <v>0.15000000000000002</v>
+        <v>0.15000000000000005</v>
       </c>
       <c r="AI14" s="40">
         <f>AE14*$D$6</f>
-        <v>198.34389119999997</v>
+        <v>182.89907999999994</v>
       </c>
       <c r="AL14" s="24" t="n">
         <v>1.134046875</v>
@@ -3007,127 +3011,127 @@
       </c>
       <c r="E15" s="24">
         <f>AL15*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
-        <v>1.3835371874999998</v>
+        <v>1.2758027343749998</v>
       </c>
       <c r="F15" s="8">
         <f>IF(AND(ISNUMBER(E15),ISNUMBER($D$8)),E15*$D$3,NA())</f>
-        <v>70.837104</v>
+        <v>65.32109999999999</v>
       </c>
       <c r="G15" s="9">
         <f>F15/$D$8</f>
-        <v>157.41578666666666</v>
+        <v>129.0293333333333</v>
       </c>
       <c r="H15" s="10">
         <f>G15*$D$4</f>
-        <v>55.09552533333333</v>
+        <v>45.16026666666666</v>
       </c>
       <c r="I15" s="11">
         <f>G15-F15-H15</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="J15" s="12">
         <f>I15/G15</f>
-        <v>0.20000000000000004</v>
+        <v>0.14375000000000002</v>
       </c>
       <c r="K15" s="13">
         <f>G15*$D$6</f>
-        <v>220.3821013333333</v>
+        <v>180.64106666666663</v>
       </c>
       <c r="L15" s="14">
         <f>F15/(1-$D$4)</f>
-        <v>108.98016</v>
+        <v>100.49399999999997</v>
       </c>
       <c r="M15" s="14">
         <f>L15*$D$6</f>
-        <v>152.57222399999998</v>
+        <v>140.69159999999994</v>
       </c>
       <c r="N15" s="15">
         <f>G15-F15</f>
-        <v>86.57868266666667</v>
+        <v>63.708233333333325</v>
       </c>
       <c r="O15" s="16">
         <f>N15-H15</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="P15" s="40">
         <f>$F15/(1-$D$4-$P$9)</f>
-        <v>202.39172571428568</v>
+        <v>186.63171428571422</v>
       </c>
       <c r="Q15" s="41">
         <f>P15*$D$4</f>
-        <v>70.83710399999998</v>
+        <v>65.32109999999997</v>
       </c>
       <c r="R15" s="42">
         <f>P15-$F15-Q15</f>
-        <v>60.71751771428572</v>
+        <v>55.989514285714264</v>
       </c>
       <c r="S15" s="43">
         <f>R15/P15</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T15" s="40">
         <f>P15*$D$6</f>
-        <v>283.34841599999993</v>
+        <v>261.2843999999999</v>
       </c>
       <c r="U15" s="40">
         <f>$F15/(1-$D$4-$U$9)</f>
-        <v>177.09275999999997</v>
+        <v>163.30274999999995</v>
       </c>
       <c r="V15" s="41">
         <f>U15*$D$4</f>
-        <v>61.98246599999999</v>
+        <v>57.15596249999998</v>
       </c>
       <c r="W15" s="42">
         <f>U15-$F15-V15</f>
-        <v>44.273189999999985</v>
+        <v>40.82568749999998</v>
       </c>
       <c r="X15" s="43">
         <f>W15/U15</f>
-        <v>0.24999999999999997</v>
+        <v>0.24999999999999994</v>
       </c>
       <c r="Y15" s="40">
         <f>U15*$D$6</f>
-        <v>247.92986399999995</v>
+        <v>228.62384999999992</v>
       </c>
       <c r="Z15" s="40">
         <f>$F15/(1-$D$4-$Z$9)</f>
-        <v>157.41578666666666</v>
+        <v>145.15799999999996</v>
       </c>
       <c r="AA15" s="41">
         <f>Z15*$D$4</f>
-        <v>55.09552533333333</v>
+        <v>50.80529999999998</v>
       </c>
       <c r="AB15" s="42">
         <f>Z15-$F15-AA15</f>
-        <v>31.483157333333338</v>
+        <v>29.03159999999999</v>
       </c>
       <c r="AC15" s="43">
         <f>AB15/Z15</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="AD15" s="40">
         <f>Z15*$D$6</f>
-        <v>220.3821013333333</v>
+        <v>203.22119999999993</v>
       </c>
       <c r="AE15" s="40">
         <f>$F15/(1-$D$4-$AE$9)</f>
-        <v>141.674208</v>
+        <v>130.64219999999997</v>
       </c>
       <c r="AF15" s="41">
         <f>AE15*$D$4</f>
-        <v>49.58597279999999</v>
+        <v>45.724769999999985</v>
       </c>
       <c r="AG15" s="42">
         <f>AE15-$F15-AF15</f>
-        <v>21.251131200000003</v>
+        <v>19.596330000000002</v>
       </c>
       <c r="AH15" s="43">
         <f>AG15/AE15</f>
-        <v>0.15000000000000002</v>
+        <v>0.15000000000000005</v>
       </c>
       <c r="AI15" s="40">
         <f>AE15*$D$6</f>
-        <v>198.34389119999997</v>
+        <v>182.89907999999994</v>
       </c>
       <c r="AL15" s="24" t="n">
         <v>1.134046875</v>
@@ -3152,127 +3156,127 @@
       </c>
       <c r="E16" s="24">
         <f>AL16*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
-        <v>1.3835371874999998</v>
+        <v>1.2758027343749998</v>
       </c>
       <c r="F16" s="8">
         <f>IF(AND(ISNUMBER(E16),ISNUMBER($D$8)),E16*$D$3,NA())</f>
-        <v>70.837104</v>
+        <v>65.32109999999999</v>
       </c>
       <c r="G16" s="9">
         <f>F16/$D$8</f>
-        <v>157.41578666666666</v>
+        <v>129.0293333333333</v>
       </c>
       <c r="H16" s="10">
         <f>G16*$D$4</f>
-        <v>55.09552533333333</v>
+        <v>45.16026666666666</v>
       </c>
       <c r="I16" s="11">
         <f>G16-F16-H16</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="J16" s="12">
         <f>I16/G16</f>
-        <v>0.20000000000000004</v>
+        <v>0.14375000000000002</v>
       </c>
       <c r="K16" s="13">
         <f>G16*$D$6</f>
-        <v>220.3821013333333</v>
+        <v>180.64106666666663</v>
       </c>
       <c r="L16" s="14">
         <f>F16/(1-$D$4)</f>
-        <v>108.98016</v>
+        <v>100.49399999999997</v>
       </c>
       <c r="M16" s="14">
         <f>L16*$D$6</f>
-        <v>152.57222399999998</v>
+        <v>140.69159999999994</v>
       </c>
       <c r="N16" s="15">
         <f>G16-F16</f>
-        <v>86.57868266666667</v>
+        <v>63.708233333333325</v>
       </c>
       <c r="O16" s="16">
         <f>N16-H16</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="P16" s="40">
         <f>$F16/(1-$D$4-$P$9)</f>
-        <v>202.39172571428568</v>
+        <v>186.63171428571422</v>
       </c>
       <c r="Q16" s="41">
         <f>P16*$D$4</f>
-        <v>70.83710399999998</v>
+        <v>65.32109999999997</v>
       </c>
       <c r="R16" s="42">
         <f>P16-$F16-Q16</f>
-        <v>60.71751771428572</v>
+        <v>55.989514285714264</v>
       </c>
       <c r="S16" s="43">
         <f>R16/P16</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T16" s="40">
         <f>P16*$D$6</f>
-        <v>283.34841599999993</v>
+        <v>261.2843999999999</v>
       </c>
       <c r="U16" s="40">
         <f>$F16/(1-$D$4-$U$9)</f>
-        <v>177.09275999999997</v>
+        <v>163.30274999999995</v>
       </c>
       <c r="V16" s="41">
         <f>U16*$D$4</f>
-        <v>61.98246599999999</v>
+        <v>57.15596249999998</v>
       </c>
       <c r="W16" s="42">
         <f>U16-$F16-V16</f>
-        <v>44.273189999999985</v>
+        <v>40.82568749999998</v>
       </c>
       <c r="X16" s="43">
         <f>W16/U16</f>
-        <v>0.24999999999999997</v>
+        <v>0.24999999999999994</v>
       </c>
       <c r="Y16" s="40">
         <f>U16*$D$6</f>
-        <v>247.92986399999995</v>
+        <v>228.62384999999992</v>
       </c>
       <c r="Z16" s="40">
         <f>$F16/(1-$D$4-$Z$9)</f>
-        <v>157.41578666666666</v>
+        <v>145.15799999999996</v>
       </c>
       <c r="AA16" s="41">
         <f>Z16*$D$4</f>
-        <v>55.09552533333333</v>
+        <v>50.80529999999998</v>
       </c>
       <c r="AB16" s="42">
         <f>Z16-$F16-AA16</f>
-        <v>31.483157333333338</v>
+        <v>29.03159999999999</v>
       </c>
       <c r="AC16" s="43">
         <f>AB16/Z16</f>
-        <v>0.20000000000000004</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="AD16" s="40">
         <f>Z16*$D$6</f>
-        <v>220.3821013333333</v>
+        <v>203.22119999999993</v>
       </c>
       <c r="AE16" s="40">
         <f>$F16/(1-$D$4-$AE$9)</f>
-        <v>141.674208</v>
+        <v>130.64219999999997</v>
       </c>
       <c r="AF16" s="41">
         <f>AE16*$D$4</f>
-        <v>49.58597279999999</v>
+        <v>45.724769999999985</v>
       </c>
       <c r="AG16" s="42">
         <f>AE16-$F16-AF16</f>
-        <v>21.251131200000003</v>
+        <v>19.596330000000002</v>
       </c>
       <c r="AH16" s="43">
         <f>AG16/AE16</f>
-        <v>0.15000000000000002</v>
+        <v>0.15000000000000005</v>
       </c>
       <c r="AI16" s="40">
         <f>AE16*$D$6</f>
-        <v>198.34389119999997</v>
+        <v>182.89907999999994</v>
       </c>
       <c r="AL16" s="24" t="n">
         <v>1.134046875</v>
@@ -3360,27 +3364,27 @@
       <c r="E22" s="65" t="n"/>
       <c r="F22" s="29">
         <f>E11</f>
-        <v>1.5963890625000001</v>
+        <v>1.472080078125</v>
       </c>
       <c r="G22" s="29">
         <f>E12</f>
-        <v>1.5963890625000001</v>
+        <v>1.472080078125</v>
       </c>
       <c r="H22" s="29">
         <f>E13</f>
-        <v>1.3835371874999998</v>
+        <v>1.2758027343749998</v>
       </c>
       <c r="I22" s="29">
         <f>E14</f>
-        <v>1.3835371874999998</v>
+        <v>1.2758027343749998</v>
       </c>
       <c r="J22" s="29">
         <f>E15</f>
-        <v>1.3835371874999998</v>
+        <v>1.2758027343749998</v>
       </c>
       <c r="K22" s="29">
         <f>E16</f>
-        <v>1.3835371874999998</v>
+        <v>1.2758027343749998</v>
       </c>
     </row>
     <row r="23" ht="31.05" customHeight="1" s="71">
@@ -3442,27 +3446,27 @@
       <c r="E24" s="65" t="n"/>
       <c r="F24" s="31">
         <f>F11</f>
-        <v>81.73512000000001</v>
+        <v>75.3705</v>
       </c>
       <c r="G24" s="31">
         <f>F12</f>
-        <v>81.73512000000001</v>
+        <v>75.3705</v>
       </c>
       <c r="H24" s="31">
         <f>F13</f>
-        <v>70.837104</v>
+        <v>65.32109999999999</v>
       </c>
       <c r="I24" s="31">
         <f>F14</f>
-        <v>70.837104</v>
+        <v>65.32109999999999</v>
       </c>
       <c r="J24" s="31">
         <f>F15</f>
-        <v>70.837104</v>
+        <v>65.32109999999999</v>
       </c>
       <c r="K24" s="31">
         <f>F16</f>
-        <v>70.837104</v>
+        <v>65.32109999999999</v>
       </c>
     </row>
     <row r="25" ht="31.05" customHeight="1" s="71">
@@ -3600,27 +3604,27 @@
       <c r="E28" s="65" t="n"/>
       <c r="F28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="G28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="H28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="I28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="J28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="K28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
     </row>
     <row r="29" ht="31.05" customHeight="1" s="71">
@@ -3641,27 +3645,27 @@
       <c r="E29" s="65" t="n"/>
       <c r="F29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="G29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="H29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="I29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="J29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="K29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
     </row>
     <row r="30" ht="31.05" customHeight="1" s="71">
@@ -3682,27 +3686,27 @@
       <c r="E30" s="65" t="n"/>
       <c r="F30" s="34">
         <f>G11</f>
-        <v>181.63360000000003</v>
+        <v>148.88000000000002</v>
       </c>
       <c r="G30" s="34">
         <f>G12</f>
-        <v>181.63360000000003</v>
+        <v>148.88000000000002</v>
       </c>
       <c r="H30" s="34">
         <f>G13</f>
-        <v>157.41578666666666</v>
+        <v>129.0293333333333</v>
       </c>
       <c r="I30" s="34">
         <f>G14</f>
-        <v>157.41578666666666</v>
+        <v>129.0293333333333</v>
       </c>
       <c r="J30" s="34">
         <f>G15</f>
-        <v>157.41578666666666</v>
+        <v>129.0293333333333</v>
       </c>
       <c r="K30" s="34">
         <f>G16</f>
-        <v>157.41578666666666</v>
+        <v>129.0293333333333</v>
       </c>
     </row>
     <row r="31" ht="31.05" customHeight="1" s="71">
@@ -3723,27 +3727,27 @@
       <c r="E31" s="65" t="n"/>
       <c r="F31" s="31">
         <f>N11</f>
-        <v>99.89848000000002</v>
+        <v>73.50950000000002</v>
       </c>
       <c r="G31" s="31">
         <f>N12</f>
-        <v>99.89848000000002</v>
+        <v>73.50950000000002</v>
       </c>
       <c r="H31" s="31">
         <f>N13</f>
-        <v>86.57868266666667</v>
+        <v>63.708233333333325</v>
       </c>
       <c r="I31" s="31">
         <f>N14</f>
-        <v>86.57868266666667</v>
+        <v>63.708233333333325</v>
       </c>
       <c r="J31" s="31">
         <f>N15</f>
-        <v>86.57868266666667</v>
+        <v>63.708233333333325</v>
       </c>
       <c r="K31" s="31">
         <f>N16</f>
-        <v>86.57868266666667</v>
+        <v>63.708233333333325</v>
       </c>
     </row>
     <row r="32" ht="31.05" customHeight="1" s="71">
@@ -3764,27 +3768,27 @@
       <c r="E32" s="65" t="n"/>
       <c r="F32" s="31">
         <f>H11</f>
-        <v>63.571760000000005</v>
+        <v>52.108000000000004</v>
       </c>
       <c r="G32" s="31">
         <f>H12</f>
-        <v>63.571760000000005</v>
+        <v>52.108000000000004</v>
       </c>
       <c r="H32" s="31">
         <f>H13</f>
-        <v>55.09552533333333</v>
+        <v>45.16026666666666</v>
       </c>
       <c r="I32" s="31">
         <f>H14</f>
-        <v>55.09552533333333</v>
+        <v>45.16026666666666</v>
       </c>
       <c r="J32" s="31">
         <f>H15</f>
-        <v>55.09552533333333</v>
+        <v>45.16026666666666</v>
       </c>
       <c r="K32" s="31">
         <f>H16</f>
-        <v>55.09552533333333</v>
+        <v>45.16026666666666</v>
       </c>
     </row>
     <row r="33" ht="31.05" customHeight="1" s="71">
@@ -3805,27 +3809,27 @@
       <c r="E33" s="65" t="n"/>
       <c r="F33" s="36">
         <f>I11</f>
-        <v>36.326720000000016</v>
+        <v>21.401500000000013</v>
       </c>
       <c r="G33" s="36">
         <f>I12</f>
-        <v>36.326720000000016</v>
+        <v>21.401500000000013</v>
       </c>
       <c r="H33" s="36">
         <f>I13</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="I33" s="36">
         <f>I14</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="J33" s="36">
         <f>I15</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
       <c r="K33" s="36">
         <f>I16</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666667</v>
       </c>
     </row>
     <row r="34" ht="31.05" customHeight="1" s="71">
@@ -3846,27 +3850,27 @@
       <c r="E34" s="65" t="n"/>
       <c r="F34" s="37">
         <f>J11</f>
-        <v>0.20000000000000007</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="G34" s="37">
         <f>J12</f>
-        <v>0.20000000000000007</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="H34" s="37">
         <f>J13</f>
-        <v>0.20000000000000004</v>
+        <v>0.14375000000000002</v>
       </c>
       <c r="I34" s="37">
         <f>J14</f>
-        <v>0.20000000000000004</v>
+        <v>0.14375000000000002</v>
       </c>
       <c r="J34" s="37">
         <f>J15</f>
-        <v>0.20000000000000004</v>
+        <v>0.14375000000000002</v>
       </c>
       <c r="K34" s="37">
         <f>J16</f>
-        <v>0.20000000000000004</v>
+        <v>0.14375000000000002</v>
       </c>
     </row>
     <row r="35" ht="31.05" customHeight="1" s="71">
@@ -3969,27 +3973,27 @@
       <c r="E37" s="65" t="n"/>
       <c r="F37" s="34">
         <f>K11</f>
-        <v>254.28704000000002</v>
+        <v>208.43200000000002</v>
       </c>
       <c r="G37" s="34">
         <f>K12</f>
-        <v>254.28704000000002</v>
+        <v>208.43200000000002</v>
       </c>
       <c r="H37" s="34">
         <f>K13</f>
-        <v>220.3821013333333</v>
+        <v>180.64106666666663</v>
       </c>
       <c r="I37" s="34">
         <f>K14</f>
-        <v>220.3821013333333</v>
+        <v>180.64106666666663</v>
       </c>
       <c r="J37" s="34">
         <f>K15</f>
-        <v>220.3821013333333</v>
+        <v>180.64106666666663</v>
       </c>
       <c r="K37" s="34">
         <f>K16</f>
-        <v>220.3821013333333</v>
+        <v>180.64106666666663</v>
       </c>
     </row>
     <row r="38" ht="31.05" customHeight="1" s="71">
@@ -4010,27 +4014,27 @@
       <c r="E38" s="65" t="n"/>
       <c r="F38" s="31">
         <f>L11</f>
-        <v>125.74633846153847</v>
+        <v>115.9546153846154</v>
       </c>
       <c r="G38" s="31">
         <f>L12</f>
-        <v>125.74633846153847</v>
+        <v>115.9546153846154</v>
       </c>
       <c r="H38" s="31">
         <f>L13</f>
-        <v>108.98016</v>
+        <v>100.49399999999997</v>
       </c>
       <c r="I38" s="31">
         <f>L14</f>
-        <v>108.98016</v>
+        <v>100.49399999999997</v>
       </c>
       <c r="J38" s="31">
         <f>L15</f>
-        <v>108.98016</v>
+        <v>100.49399999999997</v>
       </c>
       <c r="K38" s="31">
         <f>L16</f>
-        <v>108.98016</v>
+        <v>100.49399999999997</v>
       </c>
     </row>
     <row r="39" ht="31.05" customHeight="1" s="71">
@@ -4051,27 +4055,27 @@
       <c r="E39" s="65" t="n"/>
       <c r="F39" s="31">
         <f>M11</f>
-        <v>176.04487384615385</v>
+        <v>162.33646153846155</v>
       </c>
       <c r="G39" s="31">
         <f>M12</f>
-        <v>176.04487384615385</v>
+        <v>162.33646153846155</v>
       </c>
       <c r="H39" s="31">
         <f>M13</f>
-        <v>152.57222399999998</v>
+        <v>140.69159999999994</v>
       </c>
       <c r="I39" s="31">
         <f>M14</f>
-        <v>152.57222399999998</v>
+        <v>140.69159999999994</v>
       </c>
       <c r="J39" s="31">
         <f>M15</f>
-        <v>152.57222399999998</v>
+        <v>140.69159999999994</v>
       </c>
       <c r="K39" s="31">
         <f>M16</f>
-        <v>152.57222399999998</v>
+        <v>140.69159999999994</v>
       </c>
     </row>
   </sheetData>
@@ -4266,12 +4270,13 @@
         </is>
       </c>
       <c r="C5" s="63" t="n"/>
-      <c r="D5" s="18" t="n">
-        <v>0.2</v>
+      <c r="D5" s="18">
+        <f>'Price 120 UAH - 33 pallets'!C14</f>
+        <v>0.14375000000000004</v>
       </c>
       <c r="E5" s="68" t="str">
         <f>ROUND(D5*100,0)&amp;"% = (partner price − landed cost − bonus) / full partner price."</f>
-        <v>20% = (partner price − landed cost − bonus) / full partner price.</v>
+        <v>14% = (partner price − landed cost − bonus) / full partner price.</v>
       </c>
       <c r="F5" s="69" t="n"/>
       <c r="G5" s="69" t="n"/>
@@ -4335,11 +4340,11 @@
       <c r="C8" s="77" t="n"/>
       <c r="D8" s="23">
         <f>IF(AND(COUNT(D3:D6)=4,D3&gt;0,D4&gt;=0,D5&gt;=0,D4+D5&lt;1,D6&gt;0),1-D4-D5,NA())</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="E8" s="79" t="str">
         <f>"100% − bonus − margin. Current terms: 100% − "&amp;ROUND(D4*100,0)&amp;"% − "&amp;ROUND(D5*100,0)&amp;"% = "&amp;ROUND(D8*100,0)&amp;"%."</f>
-        <v>100% − bonus − margin. Current terms: 100% − 35% − 20% = 45%.</v>
+        <v>100% − bonus − margin. Current terms: 100% − 35% − 14% = 51%.</v>
       </c>
       <c r="F8" s="69" t="n"/>
       <c r="G8" s="69" t="n"/>
@@ -4618,79 +4623,79 @@
       </c>
       <c r="E11" s="24">
         <f>AL11*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
-        <v>1.2421200082056887</v>
+        <v>1.1453975485503278</v>
       </c>
       <c r="F11" s="8">
         <f>IF(AND(ISNUMBER(E11),ISNUMBER($D$8)),E11*$D$3,NA())</f>
-        <v>63.596544420131266</v>
+        <v>58.64435448577679</v>
       </c>
       <c r="G11" s="9">
         <f>F11/$D$8</f>
-        <v>141.32565426695837</v>
+        <v>115.84070021881836</v>
       </c>
       <c r="H11" s="10">
         <f>G11*$D$4</f>
-        <v>49.463978993435425</v>
+        <v>40.54424507658642</v>
       </c>
       <c r="I11" s="11">
         <f>G11-F11-H11</f>
-        <v>28.265130853391675</v>
+        <v>16.652100656455147</v>
       </c>
       <c r="J11" s="12">
         <f>I11/G11</f>
-        <v>0.2</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="K11" s="13">
         <f>G11*$D$6</f>
-        <v>197.8559159737417</v>
+        <v>162.17698030634568</v>
       </c>
       <c r="L11" s="14">
         <f>F11/(1-$D$4)</f>
-        <v>97.84083756943271</v>
+        <v>90.22208382427198</v>
       </c>
       <c r="M11" s="14">
         <f>L11*$D$6</f>
-        <v>136.9771725972058</v>
+        <v>126.31091735398076</v>
       </c>
       <c r="N11" s="15">
         <f>G11-F11</f>
-        <v>77.7291098468271</v>
+        <v>57.19634573304157</v>
       </c>
       <c r="O11" s="16">
         <f>N11-H11</f>
-        <v>28.265130853391675</v>
+        <v>16.652100656455147</v>
       </c>
       <c r="P11" s="40">
         <f>$F11/(1-$D$4-$P$9)</f>
-        <v>181.70441262894647</v>
+        <v>167.5552985307908</v>
       </c>
       <c r="Q11" s="41">
         <f>P11*$D$4</f>
-        <v>63.59654442013126</v>
+        <v>58.64435448577677</v>
       </c>
       <c r="R11" s="42">
         <f>P11-$F11-Q11</f>
-        <v>54.511323788683946</v>
+        <v>50.26658955923723</v>
       </c>
       <c r="S11" s="43">
         <f>R11/P11</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T11" s="40">
         <f>P11*$D$6</f>
-        <v>254.38617768052504</v>
+        <v>234.5774179431071</v>
       </c>
       <c r="U11" s="40">
         <f>$F11/(1-$D$4-$U$9)</f>
-        <v>158.99136105032815</v>
+        <v>146.61088621444196</v>
       </c>
       <c r="V11" s="41">
         <f>U11*$D$4</f>
-        <v>55.64697636761485</v>
+        <v>51.313810175054684</v>
       </c>
       <c r="W11" s="42">
         <f>U11-$F11-V11</f>
-        <v>39.74784026258204</v>
+        <v>36.65272155361049</v>
       </c>
       <c r="X11" s="43">
         <f>W11/U11</f>
@@ -4698,39 +4703,39 @@
       </c>
       <c r="Y11" s="40">
         <f>U11*$D$6</f>
-        <v>222.5879054704594</v>
+        <v>205.25524070021874</v>
       </c>
       <c r="Z11" s="40">
         <f>$F11/(1-$D$4-$Z$9)</f>
-        <v>141.32565426695837</v>
+        <v>130.32078774617062</v>
       </c>
       <c r="AA11" s="41">
         <f>Z11*$D$4</f>
-        <v>49.463978993435425</v>
+        <v>45.61227571115972</v>
       </c>
       <c r="AB11" s="42">
         <f>Z11-$F11-AA11</f>
-        <v>28.265130853391675</v>
+        <v>26.064157549234118</v>
       </c>
       <c r="AC11" s="43">
         <f>AB11/Z11</f>
-        <v>0.2</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="AD11" s="40">
         <f>Z11*$D$6</f>
-        <v>197.8559159737417</v>
+        <v>182.44910284463887</v>
       </c>
       <c r="AE11" s="40">
         <f>$F11/(1-$D$4-$AE$9)</f>
-        <v>127.19308884026253</v>
+        <v>117.28870897155358</v>
       </c>
       <c r="AF11" s="41">
         <f>AE11*$D$4</f>
-        <v>44.51758109409188</v>
+        <v>41.05104814004375</v>
       </c>
       <c r="AG11" s="42">
         <f>AE11-$F11-AF11</f>
-        <v>19.078963326039386</v>
+        <v>17.59330634573304</v>
       </c>
       <c r="AH11" s="43">
         <f>AG11/AE11</f>
@@ -4738,7 +4743,7 @@
       </c>
       <c r="AI11" s="40">
         <f>AE11*$D$6</f>
-        <v>178.07032437636752</v>
+        <v>164.204192560175</v>
       </c>
       <c r="AL11" s="24" t="n">
         <v>1.018131154266958</v>
@@ -4763,79 +4768,79 @@
       </c>
       <c r="E12" s="24">
         <f>AL12*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
-        <v>1.2421200082056887</v>
+        <v>1.1453975485503278</v>
       </c>
       <c r="F12" s="8">
         <f>IF(AND(ISNUMBER(E12),ISNUMBER($D$8)),E12*$D$3,NA())</f>
-        <v>63.596544420131266</v>
+        <v>58.64435448577679</v>
       </c>
       <c r="G12" s="9">
         <f>F12/$D$8</f>
-        <v>141.32565426695837</v>
+        <v>115.84070021881836</v>
       </c>
       <c r="H12" s="10">
         <f>G12*$D$4</f>
-        <v>49.463978993435425</v>
+        <v>40.54424507658642</v>
       </c>
       <c r="I12" s="11">
         <f>G12-F12-H12</f>
-        <v>28.265130853391675</v>
+        <v>16.652100656455147</v>
       </c>
       <c r="J12" s="12">
         <f>I12/G12</f>
-        <v>0.2</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="K12" s="13">
         <f>G12*$D$6</f>
-        <v>197.8559159737417</v>
+        <v>162.17698030634568</v>
       </c>
       <c r="L12" s="14">
         <f>F12/(1-$D$4)</f>
-        <v>97.84083756943271</v>
+        <v>90.22208382427198</v>
       </c>
       <c r="M12" s="14">
         <f>L12*$D$6</f>
-        <v>136.9771725972058</v>
+        <v>126.31091735398076</v>
       </c>
       <c r="N12" s="15">
         <f>G12-F12</f>
-        <v>77.7291098468271</v>
+        <v>57.19634573304157</v>
       </c>
       <c r="O12" s="16">
         <f>N12-H12</f>
-        <v>28.265130853391675</v>
+        <v>16.652100656455147</v>
       </c>
       <c r="P12" s="40">
         <f>$F12/(1-$D$4-$P$9)</f>
-        <v>181.70441262894647</v>
+        <v>167.5552985307908</v>
       </c>
       <c r="Q12" s="41">
         <f>P12*$D$4</f>
-        <v>63.59654442013126</v>
+        <v>58.64435448577677</v>
       </c>
       <c r="R12" s="42">
         <f>P12-$F12-Q12</f>
-        <v>54.511323788683946</v>
+        <v>50.26658955923723</v>
       </c>
       <c r="S12" s="43">
         <f>R12/P12</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T12" s="40">
         <f>P12*$D$6</f>
-        <v>254.38617768052504</v>
+        <v>234.5774179431071</v>
       </c>
       <c r="U12" s="40">
         <f>$F12/(1-$D$4-$U$9)</f>
-        <v>158.99136105032815</v>
+        <v>146.61088621444196</v>
       </c>
       <c r="V12" s="41">
         <f>U12*$D$4</f>
-        <v>55.64697636761485</v>
+        <v>51.313810175054684</v>
       </c>
       <c r="W12" s="42">
         <f>U12-$F12-V12</f>
-        <v>39.74784026258204</v>
+        <v>36.65272155361049</v>
       </c>
       <c r="X12" s="43">
         <f>W12/U12</f>
@@ -4843,39 +4848,39 @@
       </c>
       <c r="Y12" s="40">
         <f>U12*$D$6</f>
-        <v>222.5879054704594</v>
+        <v>205.25524070021874</v>
       </c>
       <c r="Z12" s="40">
         <f>$F12/(1-$D$4-$Z$9)</f>
-        <v>141.32565426695837</v>
+        <v>130.32078774617062</v>
       </c>
       <c r="AA12" s="41">
         <f>Z12*$D$4</f>
-        <v>49.463978993435425</v>
+        <v>45.61227571115972</v>
       </c>
       <c r="AB12" s="42">
         <f>Z12-$F12-AA12</f>
-        <v>28.265130853391675</v>
+        <v>26.064157549234118</v>
       </c>
       <c r="AC12" s="43">
         <f>AB12/Z12</f>
-        <v>0.2</v>
+        <v>0.19999999999999996</v>
       </c>
       <c r="AD12" s="40">
         <f>Z12*$D$6</f>
-        <v>197.8559159737417</v>
+        <v>182.44910284463887</v>
       </c>
       <c r="AE12" s="40">
         <f>$F12/(1-$D$4-$AE$9)</f>
-        <v>127.19308884026253</v>
+        <v>117.28870897155358</v>
       </c>
       <c r="AF12" s="41">
         <f>AE12*$D$4</f>
-        <v>44.51758109409188</v>
+        <v>41.05104814004375</v>
       </c>
       <c r="AG12" s="42">
         <f>AE12-$F12-AF12</f>
-        <v>19.078963326039386</v>
+        <v>17.59330634573304</v>
       </c>
       <c r="AH12" s="43">
         <f>AG12/AE12</f>
@@ -4883,7 +4888,7 @@
       </c>
       <c r="AI12" s="40">
         <f>AE12*$D$6</f>
-        <v>178.07032437636752</v>
+        <v>164.204192560175</v>
       </c>
       <c r="AL12" s="24" t="n">
         <v>1.018131154266958</v>
@@ -4908,127 +4913,127 @@
       </c>
       <c r="E13" s="24">
         <f>AL13*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
       <c r="F13" s="8">
         <f>IF(AND(ISNUMBER(E13),ISNUMBER($D$8)),E13*$D$3,NA())</f>
-        <v>55.11700516411381</v>
+        <v>50.82510722100659</v>
       </c>
       <c r="G13" s="9">
         <f>F13/$D$8</f>
-        <v>122.4822336980307</v>
+        <v>100.39527352297598</v>
       </c>
       <c r="H13" s="10">
         <f>G13*$D$4</f>
-        <v>42.86878179431074</v>
+        <v>35.13834573304159</v>
       </c>
       <c r="I13" s="11">
         <f>G13-F13-H13</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="J13" s="12">
         <f>I13/G13</f>
-        <v>0.19999999999999996</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="K13" s="13">
         <f>G13*$D$6</f>
-        <v>171.47512717724297</v>
+        <v>140.55338293216636</v>
       </c>
       <c r="L13" s="14">
         <f>F13/(1-$D$4)</f>
-        <v>84.79539256017509</v>
+        <v>78.19247264770244</v>
       </c>
       <c r="M13" s="14">
         <f>L13*$D$6</f>
-        <v>118.71354958424511</v>
+        <v>109.46946170678342</v>
       </c>
       <c r="N13" s="15">
         <f>G13-F13</f>
-        <v>67.36522853391688</v>
+        <v>49.570166301969394</v>
       </c>
       <c r="O13" s="16">
         <f>N13-H13</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="P13" s="40">
         <f>$F13/(1-$D$4-$P$9)</f>
-        <v>157.47715761175374</v>
+        <v>145.21459206001882</v>
       </c>
       <c r="Q13" s="41">
         <f>P13*$D$4</f>
-        <v>55.117005164113806</v>
+        <v>50.82510722100658</v>
       </c>
       <c r="R13" s="42">
         <f>P13-$F13-Q13</f>
-        <v>47.24314728352613</v>
+        <v>43.56437761800564</v>
       </c>
       <c r="S13" s="43">
         <f>R13/P13</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T13" s="40">
         <f>P13*$D$6</f>
-        <v>220.46802065645522</v>
+        <v>203.30042888402633</v>
       </c>
       <c r="U13" s="40">
         <f>$F13/(1-$D$4-$U$9)</f>
-        <v>137.79251291028453</v>
+        <v>127.06276805251647</v>
       </c>
       <c r="V13" s="41">
         <f>U13*$D$4</f>
-        <v>48.227379518599584</v>
+        <v>44.471968818380766</v>
       </c>
       <c r="W13" s="42">
         <f>U13-$F13-V13</f>
-        <v>34.44812822757114</v>
+        <v>31.76569201312912</v>
       </c>
       <c r="X13" s="43">
         <f>W13/U13</f>
-        <v>0.25000000000000006</v>
+        <v>0.25</v>
       </c>
       <c r="Y13" s="40">
         <f>U13*$D$6</f>
-        <v>192.90951807439833</v>
+        <v>177.88787527352306</v>
       </c>
       <c r="Z13" s="40">
         <f>$F13/(1-$D$4-$Z$9)</f>
-        <v>122.4822336980307</v>
+        <v>112.94468271334797</v>
       </c>
       <c r="AA13" s="41">
         <f>Z13*$D$4</f>
-        <v>42.86878179431074</v>
+        <v>39.53063894967179</v>
       </c>
       <c r="AB13" s="42">
         <f>Z13-$F13-AA13</f>
-        <v>24.496446739606135</v>
+        <v>22.588936542669593</v>
       </c>
       <c r="AC13" s="43">
         <f>AB13/Z13</f>
-        <v>0.19999999999999996</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="AD13" s="40">
         <f>Z13*$D$6</f>
-        <v>171.47512717724297</v>
+        <v>158.12255579868716</v>
       </c>
       <c r="AE13" s="40">
         <f>$F13/(1-$D$4-$AE$9)</f>
-        <v>110.23401032822763</v>
+        <v>101.65021444201318</v>
       </c>
       <c r="AF13" s="41">
         <f>AE13*$D$4</f>
-        <v>38.581903614879664</v>
+        <v>35.57757505470461</v>
       </c>
       <c r="AG13" s="42">
         <f>AE13-$F13-AF13</f>
-        <v>16.53510154923415</v>
+        <v>15.24753216630198</v>
       </c>
       <c r="AH13" s="43">
         <f>AG13/AE13</f>
-        <v>0.15000000000000005</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="AI13" s="40">
         <f>AE13*$D$6</f>
-        <v>154.32761445951866</v>
+        <v>142.31030021881844</v>
       </c>
       <c r="AL13" s="24" t="n">
         <v>0.8823803336980306</v>
@@ -5053,127 +5058,127 @@
       </c>
       <c r="E14" s="24">
         <f>AL14*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
       <c r="F14" s="8">
         <f>IF(AND(ISNUMBER(E14),ISNUMBER($D$8)),E14*$D$3,NA())</f>
-        <v>55.11700516411381</v>
+        <v>50.82510722100659</v>
       </c>
       <c r="G14" s="9">
         <f>F14/$D$8</f>
-        <v>122.4822336980307</v>
+        <v>100.39527352297598</v>
       </c>
       <c r="H14" s="10">
         <f>G14*$D$4</f>
-        <v>42.86878179431074</v>
+        <v>35.13834573304159</v>
       </c>
       <c r="I14" s="11">
         <f>G14-F14-H14</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="J14" s="12">
         <f>I14/G14</f>
-        <v>0.19999999999999996</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="K14" s="13">
         <f>G14*$D$6</f>
-        <v>171.47512717724297</v>
+        <v>140.55338293216636</v>
       </c>
       <c r="L14" s="14">
         <f>F14/(1-$D$4)</f>
-        <v>84.79539256017509</v>
+        <v>78.19247264770244</v>
       </c>
       <c r="M14" s="14">
         <f>L14*$D$6</f>
-        <v>118.71354958424511</v>
+        <v>109.46946170678342</v>
       </c>
       <c r="N14" s="15">
         <f>G14-F14</f>
-        <v>67.36522853391688</v>
+        <v>49.570166301969394</v>
       </c>
       <c r="O14" s="16">
         <f>N14-H14</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="P14" s="40">
         <f>$F14/(1-$D$4-$P$9)</f>
-        <v>157.47715761175374</v>
+        <v>145.21459206001882</v>
       </c>
       <c r="Q14" s="41">
         <f>P14*$D$4</f>
-        <v>55.117005164113806</v>
+        <v>50.82510722100658</v>
       </c>
       <c r="R14" s="42">
         <f>P14-$F14-Q14</f>
-        <v>47.24314728352613</v>
+        <v>43.56437761800564</v>
       </c>
       <c r="S14" s="43">
         <f>R14/P14</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T14" s="40">
         <f>P14*$D$6</f>
-        <v>220.46802065645522</v>
+        <v>203.30042888402633</v>
       </c>
       <c r="U14" s="40">
         <f>$F14/(1-$D$4-$U$9)</f>
-        <v>137.79251291028453</v>
+        <v>127.06276805251647</v>
       </c>
       <c r="V14" s="41">
         <f>U14*$D$4</f>
-        <v>48.227379518599584</v>
+        <v>44.471968818380766</v>
       </c>
       <c r="W14" s="42">
         <f>U14-$F14-V14</f>
-        <v>34.44812822757114</v>
+        <v>31.76569201312912</v>
       </c>
       <c r="X14" s="43">
         <f>W14/U14</f>
-        <v>0.25000000000000006</v>
+        <v>0.25</v>
       </c>
       <c r="Y14" s="40">
         <f>U14*$D$6</f>
-        <v>192.90951807439833</v>
+        <v>177.88787527352306</v>
       </c>
       <c r="Z14" s="40">
         <f>$F14/(1-$D$4-$Z$9)</f>
-        <v>122.4822336980307</v>
+        <v>112.94468271334797</v>
       </c>
       <c r="AA14" s="41">
         <f>Z14*$D$4</f>
-        <v>42.86878179431074</v>
+        <v>39.53063894967179</v>
       </c>
       <c r="AB14" s="42">
         <f>Z14-$F14-AA14</f>
-        <v>24.496446739606135</v>
+        <v>22.588936542669593</v>
       </c>
       <c r="AC14" s="43">
         <f>AB14/Z14</f>
-        <v>0.19999999999999996</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="AD14" s="40">
         <f>Z14*$D$6</f>
-        <v>171.47512717724297</v>
+        <v>158.12255579868716</v>
       </c>
       <c r="AE14" s="40">
         <f>$F14/(1-$D$4-$AE$9)</f>
-        <v>110.23401032822763</v>
+        <v>101.65021444201318</v>
       </c>
       <c r="AF14" s="41">
         <f>AE14*$D$4</f>
-        <v>38.581903614879664</v>
+        <v>35.57757505470461</v>
       </c>
       <c r="AG14" s="42">
         <f>AE14-$F14-AF14</f>
-        <v>16.53510154923415</v>
+        <v>15.24753216630198</v>
       </c>
       <c r="AH14" s="43">
         <f>AG14/AE14</f>
-        <v>0.15000000000000005</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="AI14" s="40">
         <f>AE14*$D$6</f>
-        <v>154.32761445951866</v>
+        <v>142.31030021881844</v>
       </c>
       <c r="AL14" s="24" t="n">
         <v>0.8823803336980306</v>
@@ -5198,127 +5203,127 @@
       </c>
       <c r="E15" s="24">
         <f>AL15*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
       <c r="F15" s="8">
         <f>IF(AND(ISNUMBER(E15),ISNUMBER($D$8)),E15*$D$3,NA())</f>
-        <v>55.11700516411381</v>
+        <v>50.82510722100659</v>
       </c>
       <c r="G15" s="9">
         <f>F15/$D$8</f>
-        <v>122.4822336980307</v>
+        <v>100.39527352297598</v>
       </c>
       <c r="H15" s="10">
         <f>G15*$D$4</f>
-        <v>42.86878179431074</v>
+        <v>35.13834573304159</v>
       </c>
       <c r="I15" s="11">
         <f>G15-F15-H15</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="J15" s="12">
         <f>I15/G15</f>
-        <v>0.19999999999999996</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="K15" s="13">
         <f>G15*$D$6</f>
-        <v>171.47512717724297</v>
+        <v>140.55338293216636</v>
       </c>
       <c r="L15" s="14">
         <f>F15/(1-$D$4)</f>
-        <v>84.79539256017509</v>
+        <v>78.19247264770244</v>
       </c>
       <c r="M15" s="14">
         <f>L15*$D$6</f>
-        <v>118.71354958424511</v>
+        <v>109.46946170678342</v>
       </c>
       <c r="N15" s="15">
         <f>G15-F15</f>
-        <v>67.36522853391688</v>
+        <v>49.570166301969394</v>
       </c>
       <c r="O15" s="16">
         <f>N15-H15</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="P15" s="40">
         <f>$F15/(1-$D$4-$P$9)</f>
-        <v>157.47715761175374</v>
+        <v>145.21459206001882</v>
       </c>
       <c r="Q15" s="41">
         <f>P15*$D$4</f>
-        <v>55.117005164113806</v>
+        <v>50.82510722100658</v>
       </c>
       <c r="R15" s="42">
         <f>P15-$F15-Q15</f>
-        <v>47.24314728352613</v>
+        <v>43.56437761800564</v>
       </c>
       <c r="S15" s="43">
         <f>R15/P15</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T15" s="40">
         <f>P15*$D$6</f>
-        <v>220.46802065645522</v>
+        <v>203.30042888402633</v>
       </c>
       <c r="U15" s="40">
         <f>$F15/(1-$D$4-$U$9)</f>
-        <v>137.79251291028453</v>
+        <v>127.06276805251647</v>
       </c>
       <c r="V15" s="41">
         <f>U15*$D$4</f>
-        <v>48.227379518599584</v>
+        <v>44.471968818380766</v>
       </c>
       <c r="W15" s="42">
         <f>U15-$F15-V15</f>
-        <v>34.44812822757114</v>
+        <v>31.76569201312912</v>
       </c>
       <c r="X15" s="43">
         <f>W15/U15</f>
-        <v>0.25000000000000006</v>
+        <v>0.25</v>
       </c>
       <c r="Y15" s="40">
         <f>U15*$D$6</f>
-        <v>192.90951807439833</v>
+        <v>177.88787527352306</v>
       </c>
       <c r="Z15" s="40">
         <f>$F15/(1-$D$4-$Z$9)</f>
-        <v>122.4822336980307</v>
+        <v>112.94468271334797</v>
       </c>
       <c r="AA15" s="41">
         <f>Z15*$D$4</f>
-        <v>42.86878179431074</v>
+        <v>39.53063894967179</v>
       </c>
       <c r="AB15" s="42">
         <f>Z15-$F15-AA15</f>
-        <v>24.496446739606135</v>
+        <v>22.588936542669593</v>
       </c>
       <c r="AC15" s="43">
         <f>AB15/Z15</f>
-        <v>0.19999999999999996</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="AD15" s="40">
         <f>Z15*$D$6</f>
-        <v>171.47512717724297</v>
+        <v>158.12255579868716</v>
       </c>
       <c r="AE15" s="40">
         <f>$F15/(1-$D$4-$AE$9)</f>
-        <v>110.23401032822763</v>
+        <v>101.65021444201318</v>
       </c>
       <c r="AF15" s="41">
         <f>AE15*$D$4</f>
-        <v>38.581903614879664</v>
+        <v>35.57757505470461</v>
       </c>
       <c r="AG15" s="42">
         <f>AE15-$F15-AF15</f>
-        <v>16.53510154923415</v>
+        <v>15.24753216630198</v>
       </c>
       <c r="AH15" s="43">
         <f>AG15/AE15</f>
-        <v>0.15000000000000005</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="AI15" s="40">
         <f>AE15*$D$6</f>
-        <v>154.32761445951866</v>
+        <v>142.31030021881844</v>
       </c>
       <c r="AL15" s="24" t="n">
         <v>0.8823803336980306</v>
@@ -5343,127 +5348,127 @@
       </c>
       <c r="E16" s="24">
         <f>AL16*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
       <c r="F16" s="8">
         <f>IF(AND(ISNUMBER(E16),ISNUMBER($D$8)),E16*$D$3,NA())</f>
-        <v>55.11700516411381</v>
+        <v>50.82510722100659</v>
       </c>
       <c r="G16" s="9">
         <f>F16/$D$8</f>
-        <v>122.4822336980307</v>
+        <v>100.39527352297598</v>
       </c>
       <c r="H16" s="10">
         <f>G16*$D$4</f>
-        <v>42.86878179431074</v>
+        <v>35.13834573304159</v>
       </c>
       <c r="I16" s="11">
         <f>G16-F16-H16</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="J16" s="12">
         <f>I16/G16</f>
-        <v>0.19999999999999996</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="K16" s="13">
         <f>G16*$D$6</f>
-        <v>171.47512717724297</v>
+        <v>140.55338293216636</v>
       </c>
       <c r="L16" s="14">
         <f>F16/(1-$D$4)</f>
-        <v>84.79539256017509</v>
+        <v>78.19247264770244</v>
       </c>
       <c r="M16" s="14">
         <f>L16*$D$6</f>
-        <v>118.71354958424511</v>
+        <v>109.46946170678342</v>
       </c>
       <c r="N16" s="15">
         <f>G16-F16</f>
-        <v>67.36522853391688</v>
+        <v>49.570166301969394</v>
       </c>
       <c r="O16" s="16">
         <f>N16-H16</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="P16" s="40">
         <f>$F16/(1-$D$4-$P$9)</f>
-        <v>157.47715761175374</v>
+        <v>145.21459206001882</v>
       </c>
       <c r="Q16" s="41">
         <f>P16*$D$4</f>
-        <v>55.117005164113806</v>
+        <v>50.82510722100658</v>
       </c>
       <c r="R16" s="42">
         <f>P16-$F16-Q16</f>
-        <v>47.24314728352613</v>
+        <v>43.56437761800564</v>
       </c>
       <c r="S16" s="43">
         <f>R16/P16</f>
-        <v>0.30000000000000004</v>
+        <v>0.3</v>
       </c>
       <c r="T16" s="40">
         <f>P16*$D$6</f>
-        <v>220.46802065645522</v>
+        <v>203.30042888402633</v>
       </c>
       <c r="U16" s="40">
         <f>$F16/(1-$D$4-$U$9)</f>
-        <v>137.79251291028453</v>
+        <v>127.06276805251647</v>
       </c>
       <c r="V16" s="41">
         <f>U16*$D$4</f>
-        <v>48.227379518599584</v>
+        <v>44.471968818380766</v>
       </c>
       <c r="W16" s="42">
         <f>U16-$F16-V16</f>
-        <v>34.44812822757114</v>
+        <v>31.76569201312912</v>
       </c>
       <c r="X16" s="43">
         <f>W16/U16</f>
-        <v>0.25000000000000006</v>
+        <v>0.25</v>
       </c>
       <c r="Y16" s="40">
         <f>U16*$D$6</f>
-        <v>192.90951807439833</v>
+        <v>177.88787527352306</v>
       </c>
       <c r="Z16" s="40">
         <f>$F16/(1-$D$4-$Z$9)</f>
-        <v>122.4822336980307</v>
+        <v>112.94468271334797</v>
       </c>
       <c r="AA16" s="41">
         <f>Z16*$D$4</f>
-        <v>42.86878179431074</v>
+        <v>39.53063894967179</v>
       </c>
       <c r="AB16" s="42">
         <f>Z16-$F16-AA16</f>
-        <v>24.496446739606135</v>
+        <v>22.588936542669593</v>
       </c>
       <c r="AC16" s="43">
         <f>AB16/Z16</f>
-        <v>0.19999999999999996</v>
+        <v>0.19999999999999998</v>
       </c>
       <c r="AD16" s="40">
         <f>Z16*$D$6</f>
-        <v>171.47512717724297</v>
+        <v>158.12255579868716</v>
       </c>
       <c r="AE16" s="40">
         <f>$F16/(1-$D$4-$AE$9)</f>
-        <v>110.23401032822763</v>
+        <v>101.65021444201318</v>
       </c>
       <c r="AF16" s="41">
         <f>AE16*$D$4</f>
-        <v>38.581903614879664</v>
+        <v>35.57757505470461</v>
       </c>
       <c r="AG16" s="42">
         <f>AE16-$F16-AF16</f>
-        <v>16.53510154923415</v>
+        <v>15.24753216630198</v>
       </c>
       <c r="AH16" s="43">
         <f>AG16/AE16</f>
-        <v>0.15000000000000005</v>
+        <v>0.15000000000000002</v>
       </c>
       <c r="AI16" s="40">
         <f>AE16*$D$6</f>
-        <v>154.32761445951866</v>
+        <v>142.31030021881844</v>
       </c>
       <c r="AL16" s="24" t="n">
         <v>0.8823803336980306</v>
@@ -5551,27 +5556,27 @@
       <c r="E22" s="65" t="n"/>
       <c r="F22" s="29">
         <f>E11</f>
-        <v>1.2421200082056887</v>
+        <v>1.1453975485503278</v>
       </c>
       <c r="G22" s="29">
         <f>E12</f>
-        <v>1.2421200082056887</v>
+        <v>1.1453975485503278</v>
       </c>
       <c r="H22" s="29">
         <f>E13</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
       <c r="I22" s="29">
         <f>E14</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
       <c r="J22" s="29">
         <f>E15</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
       <c r="K22" s="29">
         <f>E16</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
     </row>
     <row r="23" ht="31.05" customHeight="1" s="71">
@@ -5633,27 +5638,27 @@
       <c r="E24" s="65" t="n"/>
       <c r="F24" s="31">
         <f>F11</f>
-        <v>63.596544420131266</v>
+        <v>58.64435448577679</v>
       </c>
       <c r="G24" s="31">
         <f>F12</f>
-        <v>63.596544420131266</v>
+        <v>58.64435448577679</v>
       </c>
       <c r="H24" s="31">
         <f>F13</f>
-        <v>55.11700516411381</v>
+        <v>50.82510722100659</v>
       </c>
       <c r="I24" s="31">
         <f>F14</f>
-        <v>55.11700516411381</v>
+        <v>50.82510722100659</v>
       </c>
       <c r="J24" s="31">
         <f>F15</f>
-        <v>55.11700516411381</v>
+        <v>50.82510722100659</v>
       </c>
       <c r="K24" s="31">
         <f>F16</f>
-        <v>55.11700516411381</v>
+        <v>50.82510722100659</v>
       </c>
     </row>
     <row r="25" ht="31.05" customHeight="1" s="71">
@@ -5791,27 +5796,27 @@
       <c r="E28" s="65" t="n"/>
       <c r="F28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="G28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="H28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="I28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="J28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
       <c r="K28" s="32">
         <f>$D$5</f>
-        <v>0.2</v>
+        <v>0.14375000000000004</v>
       </c>
     </row>
     <row r="29" ht="31.05" customHeight="1" s="71">
@@ -5832,27 +5837,27 @@
       <c r="E29" s="65" t="n"/>
       <c r="F29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="G29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="H29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="I29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="J29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
       <c r="K29" s="32">
         <f>$D$8</f>
-        <v>0.45</v>
+        <v>0.50625</v>
       </c>
     </row>
     <row r="30" ht="31.05" customHeight="1" s="71">
@@ -5873,27 +5878,27 @@
       <c r="E30" s="65" t="n"/>
       <c r="F30" s="34">
         <f>G11</f>
-        <v>141.32565426695837</v>
+        <v>115.84070021881836</v>
       </c>
       <c r="G30" s="34">
         <f>G12</f>
-        <v>141.32565426695837</v>
+        <v>115.84070021881836</v>
       </c>
       <c r="H30" s="34">
         <f>G13</f>
-        <v>122.4822336980307</v>
+        <v>100.39527352297598</v>
       </c>
       <c r="I30" s="34">
         <f>G14</f>
-        <v>122.4822336980307</v>
+        <v>100.39527352297598</v>
       </c>
       <c r="J30" s="34">
         <f>G15</f>
-        <v>122.4822336980307</v>
+        <v>100.39527352297598</v>
       </c>
       <c r="K30" s="34">
         <f>G16</f>
-        <v>122.4822336980307</v>
+        <v>100.39527352297598</v>
       </c>
     </row>
     <row r="31" ht="31.05" customHeight="1" s="71">
@@ -5914,27 +5919,27 @@
       <c r="E31" s="65" t="n"/>
       <c r="F31" s="31">
         <f>N11</f>
-        <v>77.7291098468271</v>
+        <v>57.19634573304157</v>
       </c>
       <c r="G31" s="31">
         <f>N12</f>
-        <v>77.7291098468271</v>
+        <v>57.19634573304157</v>
       </c>
       <c r="H31" s="31">
         <f>N13</f>
-        <v>67.36522853391688</v>
+        <v>49.570166301969394</v>
       </c>
       <c r="I31" s="31">
         <f>N14</f>
-        <v>67.36522853391688</v>
+        <v>49.570166301969394</v>
       </c>
       <c r="J31" s="31">
         <f>N15</f>
-        <v>67.36522853391688</v>
+        <v>49.570166301969394</v>
       </c>
       <c r="K31" s="31">
         <f>N16</f>
-        <v>67.36522853391688</v>
+        <v>49.570166301969394</v>
       </c>
     </row>
     <row r="32" ht="31.05" customHeight="1" s="71">
@@ -5955,27 +5960,27 @@
       <c r="E32" s="65" t="n"/>
       <c r="F32" s="31">
         <f>H11</f>
-        <v>49.463978993435425</v>
+        <v>40.54424507658642</v>
       </c>
       <c r="G32" s="31">
         <f>H12</f>
-        <v>49.463978993435425</v>
+        <v>40.54424507658642</v>
       </c>
       <c r="H32" s="31">
         <f>H13</f>
-        <v>42.86878179431074</v>
+        <v>35.13834573304159</v>
       </c>
       <c r="I32" s="31">
         <f>H14</f>
-        <v>42.86878179431074</v>
+        <v>35.13834573304159</v>
       </c>
       <c r="J32" s="31">
         <f>H15</f>
-        <v>42.86878179431074</v>
+        <v>35.13834573304159</v>
       </c>
       <c r="K32" s="31">
         <f>H16</f>
-        <v>42.86878179431074</v>
+        <v>35.13834573304159</v>
       </c>
     </row>
     <row r="33" ht="31.05" customHeight="1" s="71">
@@ -5996,27 +6001,27 @@
       <c r="E33" s="65" t="n"/>
       <c r="F33" s="36">
         <f>I11</f>
-        <v>28.265130853391675</v>
+        <v>16.652100656455147</v>
       </c>
       <c r="G33" s="36">
         <f>I12</f>
-        <v>28.265130853391675</v>
+        <v>16.652100656455147</v>
       </c>
       <c r="H33" s="36">
         <f>I13</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="I33" s="36">
         <f>I14</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="J33" s="36">
         <f>I15</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="K33" s="36">
         <f>I16</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
     </row>
     <row r="34" ht="31.05" customHeight="1" s="71">
@@ -6037,27 +6042,27 @@
       <c r="E34" s="65" t="n"/>
       <c r="F34" s="37">
         <f>J11</f>
-        <v>0.2</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="G34" s="37">
         <f>J12</f>
-        <v>0.2</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="H34" s="37">
         <f>J13</f>
-        <v>0.19999999999999996</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="I34" s="37">
         <f>J14</f>
-        <v>0.19999999999999996</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="J34" s="37">
         <f>J15</f>
-        <v>0.19999999999999996</v>
+        <v>0.14375000000000007</v>
       </c>
       <c r="K34" s="37">
         <f>J16</f>
-        <v>0.19999999999999996</v>
+        <v>0.14375000000000007</v>
       </c>
     </row>
     <row r="35" ht="31.05" customHeight="1" s="71">
@@ -6160,27 +6165,27 @@
       <c r="E37" s="65" t="n"/>
       <c r="F37" s="34">
         <f>K11</f>
-        <v>197.8559159737417</v>
+        <v>162.17698030634568</v>
       </c>
       <c r="G37" s="34">
         <f>K12</f>
-        <v>197.8559159737417</v>
+        <v>162.17698030634568</v>
       </c>
       <c r="H37" s="34">
         <f>K13</f>
-        <v>171.47512717724297</v>
+        <v>140.55338293216636</v>
       </c>
       <c r="I37" s="34">
         <f>K14</f>
-        <v>171.47512717724297</v>
+        <v>140.55338293216636</v>
       </c>
       <c r="J37" s="34">
         <f>K15</f>
-        <v>171.47512717724297</v>
+        <v>140.55338293216636</v>
       </c>
       <c r="K37" s="34">
         <f>K16</f>
-        <v>171.47512717724297</v>
+        <v>140.55338293216636</v>
       </c>
     </row>
     <row r="38" ht="31.05" customHeight="1" s="71">
@@ -6201,27 +6206,27 @@
       <c r="E38" s="65" t="n"/>
       <c r="F38" s="31">
         <f>L11</f>
-        <v>97.84083756943271</v>
+        <v>90.22208382427198</v>
       </c>
       <c r="G38" s="31">
         <f>L12</f>
-        <v>97.84083756943271</v>
+        <v>90.22208382427198</v>
       </c>
       <c r="H38" s="31">
         <f>L13</f>
-        <v>84.79539256017509</v>
+        <v>78.19247264770244</v>
       </c>
       <c r="I38" s="31">
         <f>L14</f>
-        <v>84.79539256017509</v>
+        <v>78.19247264770244</v>
       </c>
       <c r="J38" s="31">
         <f>L15</f>
-        <v>84.79539256017509</v>
+        <v>78.19247264770244</v>
       </c>
       <c r="K38" s="31">
         <f>L16</f>
-        <v>84.79539256017509</v>
+        <v>78.19247264770244</v>
       </c>
     </row>
     <row r="39" ht="31.05" customHeight="1" s="71">
@@ -6242,27 +6247,27 @@
       <c r="E39" s="65" t="n"/>
       <c r="F39" s="31">
         <f>M11</f>
-        <v>136.9771725972058</v>
+        <v>126.31091735398076</v>
       </c>
       <c r="G39" s="31">
         <f>M12</f>
-        <v>136.9771725972058</v>
+        <v>126.31091735398076</v>
       </c>
       <c r="H39" s="31">
         <f>M13</f>
-        <v>118.71354958424511</v>
+        <v>109.46946170678342</v>
       </c>
       <c r="I39" s="31">
         <f>M14</f>
-        <v>118.71354958424511</v>
+        <v>109.46946170678342</v>
       </c>
       <c r="J39" s="31">
         <f>M15</f>
-        <v>118.71354958424511</v>
+        <v>109.46946170678342</v>
       </c>
       <c r="K39" s="31">
         <f>M16</f>
-        <v>118.71354958424511</v>
+        <v>109.46946170678342</v>
       </c>
     </row>
   </sheetData>
@@ -6347,14 +6352,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="38" customWidth="1" style="71" min="1" max="1"/>
     <col width="17" customWidth="1" style="71" min="2" max="2"/>
     <col width="23.88671875" customWidth="1" style="71" min="3" max="3"/>
     <col width="17" customWidth="1" style="71" min="4" max="8"/>
-    <col width="17" customWidth="1" style="71" min="8" max="8"/>
+    <col width="22" customWidth="1" style="71" min="8" max="8"/>
     <col width="2" customWidth="1" style="71" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -6373,7 +6378,7 @@
       </c>
       <c r="B2" s="135">
         <f>B20</f>
-        <v>0.21</v>
+        <v>0.32</v>
       </c>
       <c r="C2" s="63" t="n"/>
       <c r="D2" s="129" t="str">
@@ -6383,7 +6388,7 @@
       <c r="E2" s="63" t="n"/>
       <c r="F2" s="128" t="str">
         <f>"reduction −"&amp;ROUND((1-B20/B5)*100,0)&amp;" % / −"&amp;ROUND((1-B20/B7)*100,0)&amp;" %"</f>
-        <v>reduction −68 % / −72 %</v>
+        <v>reduction −51 % / −57 %</v>
       </c>
       <c r="G2" s="63" t="n"/>
       <c r="H2" s="129" t="inlineStr">
@@ -6407,7 +6412,7 @@
       <c r="C3" s="99" t="str">
         <f>"Landed cost in Ukraine"&amp;CHAR(10)&amp;"product + costs in Ukraine"&amp;IF(G14&gt;0," + "&amp;ROUND(G14*100,1)&amp;" % uplift","")</f>
         <v>Landed cost in Ukraine
-product + costs in Ukraine + 22 % uplift</v>
+product + costs in Ukraine + 12.5 % uplift</v>
       </c>
       <c r="D3" s="99" t="inlineStr">
         <is>
@@ -6423,7 +6428,7 @@
       <c r="F3" s="99" t="str">
         <f>"Our profit"&amp;CHAR(10)&amp;ROUND(C14*100,0)&amp;" % of partner price"</f>
         <v>Our profit
-20 % of partner price</v>
+14 % of partner price</v>
       </c>
       <c r="G3" s="99" t="inlineStr">
         <is>
@@ -6451,27 +6456,27 @@
       </c>
       <c r="C4" s="101">
         <f>$B$24*F14*(1+$G$14)</f>
-        <v>70.837104</v>
+        <v>65.3211</v>
       </c>
       <c r="D4" s="101">
         <f>C4/(1-D14-C14)</f>
-        <v>157.41578666666666</v>
+        <v>129.02933333333334</v>
       </c>
       <c r="E4" s="102">
         <f>D4*D14</f>
-        <v>55.09552533333333</v>
+        <v>45.160266666666665</v>
       </c>
       <c r="F4" s="102">
         <f>D4-C4-E4</f>
-        <v>31.483157333333338</v>
+        <v>18.547966666666674</v>
       </c>
       <c r="G4" s="102">
         <f>D4*(E14-1)</f>
-        <v>62.96631466666665</v>
+        <v>51.611733333333326</v>
       </c>
       <c r="H4" s="103">
         <f>D4*E14</f>
-        <v>220.3821013333333</v>
+        <v>180.64106666666666</v>
       </c>
     </row>
     <row r="5" ht="19.95" customHeight="1" s="71">
@@ -6481,27 +6486,27 @@
       </c>
       <c r="C5" s="138">
         <f>C4/F14</f>
-        <v>1.3835371874999998</v>
+        <v>1.275802734375</v>
       </c>
       <c r="D5" s="139">
         <f>D4/F14</f>
-        <v>3.074527083333333</v>
+        <v>2.5201041666666666</v>
       </c>
       <c r="E5" s="139">
         <f>E4/F14</f>
-        <v>1.0760844791666664</v>
+        <v>0.8820364583333332</v>
       </c>
       <c r="F5" s="139">
         <f>F4/F14</f>
-        <v>0.6149054166666668</v>
+        <v>0.36226497395833346</v>
       </c>
       <c r="G5" s="139">
         <f>G4/F14</f>
-        <v>1.2298108333333329</v>
+        <v>1.0080416666666665</v>
       </c>
       <c r="H5" s="139">
         <f>H4/F14</f>
-        <v>4.3043379166666655</v>
+        <v>3.528145833333333</v>
       </c>
     </row>
     <row r="6" ht="25.95" customHeight="1" s="71">
@@ -6517,27 +6522,27 @@
       </c>
       <c r="C6" s="109">
         <f>$B$25*F14*(1+$G$14)</f>
-        <v>81.73512000000001</v>
+        <v>75.3705</v>
       </c>
       <c r="D6" s="109">
         <f>C6/(1-D14-C14)</f>
-        <v>181.63360000000003</v>
+        <v>148.88000000000002</v>
       </c>
       <c r="E6" s="110">
         <f>D6*D14</f>
-        <v>63.571760000000005</v>
+        <v>52.108000000000004</v>
       </c>
       <c r="F6" s="110">
         <f>D6-C6-E6</f>
-        <v>36.326720000000016</v>
+        <v>21.401500000000013</v>
       </c>
       <c r="G6" s="110">
         <f>D6*(E14-1)</f>
-        <v>72.65343999999999</v>
+        <v>59.552</v>
       </c>
       <c r="H6" s="111">
         <f>D6*E14</f>
-        <v>254.28704000000002</v>
+        <v>208.43200000000002</v>
       </c>
     </row>
     <row r="7" ht="19.95" customHeight="1" s="71">
@@ -6547,27 +6552,27 @@
       </c>
       <c r="C7" s="138">
         <f>C6/F14</f>
-        <v>1.5963890625000001</v>
+        <v>1.472080078125</v>
       </c>
       <c r="D7" s="140">
         <f>D6/F14</f>
-        <v>3.5475312500000005</v>
+        <v>2.9078125000000004</v>
       </c>
       <c r="E7" s="140">
         <f>E6/F14</f>
-        <v>1.2416359375000001</v>
+        <v>1.017734375</v>
       </c>
       <c r="F7" s="140">
         <f>F6/F14</f>
-        <v>0.7095062500000002</v>
+        <v>0.41799804687500025</v>
       </c>
       <c r="G7" s="140">
         <f>G6/F14</f>
-        <v>1.4190124999999998</v>
+        <v>1.163125</v>
       </c>
       <c r="H7" s="140">
         <f>H6/F14</f>
-        <v>4.9665437500000005</v>
+        <v>4.0709375</v>
       </c>
     </row>
     <row r="8" ht="25.95" customHeight="1" s="71">
@@ -6579,62 +6584,62 @@
       </c>
       <c r="B8" s="115">
         <f>B9*F14</f>
-        <v>10.752</v>
+        <v>16.384</v>
       </c>
       <c r="C8" s="115">
         <f>B22</f>
-        <v>38.1032352</v>
+        <v>42.92945999999999</v>
       </c>
       <c r="D8" s="115">
         <f>C8/(1-D14-C14)</f>
-        <v>84.673856</v>
+        <v>84.79893333333332</v>
       </c>
       <c r="E8" s="116">
         <f>D8*D14</f>
-        <v>29.635849599999997</v>
+        <v>29.67962666666666</v>
       </c>
       <c r="F8" s="116">
         <f>D8-C8-E8</f>
-        <v>16.934771200000004</v>
+        <v>12.189846666666671</v>
       </c>
       <c r="G8" s="116">
         <f>D8*(E14-1)</f>
-        <v>33.86954239999999</v>
+        <v>33.919573333333325</v>
       </c>
       <c r="H8" s="117">
         <f>D8*E14</f>
-        <v>118.54339839999999</v>
+        <v>118.71850666666664</v>
       </c>
     </row>
     <row r="9" ht="19.95" customHeight="1" s="71">
       <c r="A9" s="136" t="n"/>
       <c r="B9" s="141">
         <f>B20</f>
-        <v>0.21</v>
+        <v>0.32</v>
       </c>
       <c r="C9" s="142">
         <f>C8/F14</f>
-        <v>0.7442038125</v>
+        <v>0.8384660156249998</v>
       </c>
       <c r="D9" s="142">
         <f>D8/F14</f>
-        <v>1.65378625</v>
+        <v>1.6562291666666664</v>
       </c>
       <c r="E9" s="142">
         <f>E8/F14</f>
-        <v>0.5788251874999999</v>
+        <v>0.5796802083333332</v>
       </c>
       <c r="F9" s="142">
         <f>F8/F14</f>
-        <v>0.33075725000000006</v>
+        <v>0.2380829427083334</v>
       </c>
       <c r="G9" s="142">
         <f>G8/F14</f>
-        <v>0.6615144999999998</v>
+        <v>0.6624916666666665</v>
       </c>
       <c r="H9" s="142">
         <f>H8/F14</f>
-        <v>2.3153007499999996</v>
+        <v>2.318720833333333</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" s="71">
@@ -6645,62 +6650,62 @@
       </c>
       <c r="B10" s="143">
         <f>B8-B4</f>
-        <v>-22.528</v>
+        <v>-16.896</v>
       </c>
       <c r="C10" s="143">
         <f>C8-C4</f>
-        <v>-32.733868799999996</v>
+        <v>-22.39164000000001</v>
       </c>
       <c r="D10" s="143">
         <f>D8-D4</f>
-        <v>-72.74193066666666</v>
+        <v>-44.23040000000002</v>
       </c>
       <c r="E10" s="143">
         <f>E8-E4</f>
-        <v>-25.45967573333333</v>
+        <v>-15.480640000000005</v>
       </c>
       <c r="F10" s="143">
         <f>F8-F4</f>
-        <v>-14.548386133333334</v>
+        <v>-6.358120000000003</v>
       </c>
       <c r="G10" s="143">
         <f>G8-G4</f>
-        <v>-29.096772266666655</v>
+        <v>-17.69216</v>
       </c>
       <c r="H10" s="143">
         <f>H8-H4</f>
-        <v>-101.83870293333332</v>
+        <v>-61.92256000000002</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="71">
       <c r="A11" s="136" t="n"/>
       <c r="B11" s="144">
         <f>B9-B5</f>
-        <v>-0.44000000000000006</v>
+        <v>-0.33</v>
       </c>
       <c r="C11" s="144">
         <f>C9-C5</f>
-        <v>-0.6393333749999998</v>
+        <v>-0.43733671875000024</v>
       </c>
       <c r="D11" s="144">
         <f>D9-D5</f>
-        <v>-1.420740833333333</v>
+        <v>-0.8638750000000002</v>
       </c>
       <c r="E11" s="144">
         <f>E9-E5</f>
-        <v>-0.4972592916666665</v>
+        <v>-0.30235625</v>
       </c>
       <c r="F11" s="144">
         <f>F9-F5</f>
-        <v>-0.2841481666666667</v>
+        <v>-0.12418203125000005</v>
       </c>
       <c r="G11" s="144">
         <f>G9-G5</f>
-        <v>-0.5682963333333331</v>
+        <v>-0.34555</v>
       </c>
       <c r="H11" s="144">
         <f>H9-H5</f>
-        <v>-1.989037166666666</v>
+        <v>-1.209425</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="71" thickBot="1">
@@ -6725,7 +6730,7 @@
       </c>
       <c r="C13" s="45" t="inlineStr">
         <is>
-          <t>Our margin</t>
+          <t>Margin shown (auto: offsets the cost uplift)</t>
         </is>
       </c>
       <c r="D13" s="45" t="inlineStr">
@@ -6746,6 +6751,11 @@
       <c r="G13" s="45" t="inlineStr">
         <is>
           <t>Cost uplift, % of landed cost (assumption)</t>
+        </is>
+      </c>
+      <c r="H13" s="45" t="inlineStr">
+        <is>
+          <t>Base share of price for cost (real model: 1 − 25 % − 30 %)</t>
         </is>
       </c>
     </row>
@@ -6758,8 +6768,9 @@
       <c r="B14" s="47" t="n">
         <v>120</v>
       </c>
-      <c r="C14" s="145" t="n">
-        <v>0.2</v>
+      <c r="C14" s="182">
+        <f>1-D14-H14*(1+G14)</f>
+        <v>0.14375000000000004</v>
       </c>
       <c r="D14" s="146">
         <f>'Model 6 pallets'!D4</f>
@@ -6774,7 +6785,10 @@
         <v>51.2</v>
       </c>
       <c r="G14" s="145" t="n">
-        <v>0.22</v>
+        <v>0.125</v>
+      </c>
+      <c r="H14" s="145" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="15">
@@ -6866,7 +6880,7 @@
       </c>
       <c r="B20" s="147">
         <f>ROUNDDOWN(((B14/E14*(1-D14-C14)/(1+G14))/F14/(1+C16)-(E16+F16+G16+E16*B18*(D16+B16*(1+D16)))/(C18*D18))/((1+D16)*(1+B16)),2)</f>
-        <v>0.21</v>
+        <v>0.32</v>
       </c>
     </row>
     <row r="21">
@@ -6877,7 +6891,7 @@
       </c>
       <c r="B21" s="148">
         <f>((B14/E14*(1-D14-C14)/(1+G14))/F14/(1+C16)-(E16+F16+G16+E16*B18*(D16+B16*(1+D16)))/(C18*D18))/((1+D16)*(1+B16))</f>
-        <v>0.216093830325013</v>
+        <v>0.3265407229965157</v>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1" s="71">
@@ -6888,7 +6902,7 @@
       </c>
       <c r="B22" s="57">
         <f>(B20*F14+(E16+F16+G16)/(C18*D18)*F14+(B20+E16*B18/(C18*D18))*D16*F14+(B20+E16*B18/(C18*D18))*(1+D16)*B16*F14)*(1+C16)*(1+G14)</f>
-        <v>38.1032352</v>
+        <v>42.92945999999999</v>
       </c>
     </row>
     <row r="23"/>
@@ -6902,9 +6916,9 @@
         <f>'Model 6 pallets'!AL13</f>
         <v>1.134046875</v>
       </c>
-      <c r="C24" s="182">
+      <c r="C24" s="183">
         <f>B24*(1+$G$14)</f>
-        <v>1.3835371874999998</v>
+        <v>1.2758027343749998</v>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1" s="71">
@@ -6917,9 +6931,9 @@
         <f>'Model 6 pallets'!AL11</f>
         <v>1.308515625</v>
       </c>
-      <c r="C25" s="182">
+      <c r="C25" s="183">
         <f>B25*(1+$G$14)</f>
-        <v>1.5963890625000001</v>
+        <v>1.472080078125</v>
       </c>
     </row>
   </sheetData>
@@ -6946,12 +6960,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I24"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="38" customWidth="1" style="71" min="1" max="1"/>
     <col width="17" customWidth="1" style="71" min="2" max="8"/>
-    <col width="17" customWidth="1" style="71" min="8" max="8"/>
+    <col width="22" customWidth="1" style="71" min="8" max="8"/>
     <col width="2" customWidth="1" style="71" min="9" max="9"/>
   </cols>
   <sheetData>
@@ -6970,7 +6984,7 @@
       </c>
       <c r="B2" s="151">
         <f>B19</f>
-        <v>0.43</v>
+        <v>0.54</v>
       </c>
       <c r="C2" s="152" t="n"/>
       <c r="D2" s="98" t="str">
@@ -6980,7 +6994,7 @@
       <c r="E2" s="152" t="n"/>
       <c r="F2" s="97" t="str">
         <f>"reduction −"&amp;ROUND((1-B19/B5)*100,0)&amp;" % / −"&amp;ROUND((1-B19/B7)*100,0)&amp;" %"</f>
-        <v>reduction −34 % / −43 %</v>
+        <v>reduction −17 % / −28 %</v>
       </c>
       <c r="G2" s="152" t="n"/>
       <c r="H2" s="98" t="inlineStr">
@@ -7004,7 +7018,7 @@
       <c r="C3" s="99" t="str">
         <f>"Landed cost in Ukraine"&amp;CHAR(10)&amp;"product + costs in Ukraine"&amp;IF(G14&gt;0," + "&amp;ROUND(G14*100,1)&amp;" % uplift","")</f>
         <v>Landed cost in Ukraine
-product + costs in Ukraine + 22 % uplift</v>
+product + costs in Ukraine + 12.5 % uplift</v>
       </c>
       <c r="D3" s="99" t="inlineStr">
         <is>
@@ -7020,7 +7034,7 @@
       <c r="F3" s="99" t="str">
         <f>"Our profit"&amp;CHAR(10)&amp;ROUND(C14*100,0)&amp;" % of partner price"</f>
         <v>Our profit
-20 % of partner price</v>
+14 % of partner price</v>
       </c>
       <c r="G3" s="99" t="inlineStr">
         <is>
@@ -7048,27 +7062,27 @@
       </c>
       <c r="C4" s="101">
         <f>$B$23*F14*(1+$G$14)</f>
-        <v>55.11700516411381</v>
+        <v>50.82510722100659</v>
       </c>
       <c r="D4" s="101">
         <f>C4/(1-D14-C14)</f>
-        <v>122.4822336980307</v>
+        <v>100.39527352297598</v>
       </c>
       <c r="E4" s="102">
         <f>D4*D14</f>
-        <v>42.86878179431074</v>
+        <v>35.13834573304159</v>
       </c>
       <c r="F4" s="102">
         <f>D4-C4-E4</f>
-        <v>24.496446739606135</v>
+        <v>14.431820568927805</v>
       </c>
       <c r="G4" s="102">
         <f>D4*(E14-1)</f>
-        <v>48.99289347921227</v>
+        <v>40.15810940919039</v>
       </c>
       <c r="H4" s="103">
         <f>D4*E14</f>
-        <v>171.47512717724297</v>
+        <v>140.55338293216636</v>
       </c>
     </row>
     <row r="5">
@@ -7078,27 +7092,27 @@
       </c>
       <c r="C5" s="138">
         <f>C4/F14</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
       <c r="D5" s="139">
         <f>D4/F14</f>
-        <v>2.392231126914662</v>
+        <v>1.9608451859956246</v>
       </c>
       <c r="E5" s="139">
         <f>E4/F14</f>
-        <v>0.8372808944201316</v>
+        <v>0.6862958150984685</v>
       </c>
       <c r="F5" s="139">
         <f>F4/F14</f>
-        <v>0.4784462253829323</v>
+        <v>0.2818714954868712</v>
       </c>
       <c r="G5" s="139">
         <f>G4/F14</f>
-        <v>0.9568924507658646</v>
+        <v>0.7843380743982498</v>
       </c>
       <c r="H5" s="139">
         <f>H4/F14</f>
-        <v>3.3491235776805266</v>
+        <v>2.745183260393874</v>
       </c>
     </row>
     <row r="6" ht="25.95" customHeight="1" s="71">
@@ -7114,27 +7128,27 @@
       </c>
       <c r="C6" s="109">
         <f>$B$24*F14*(1+$G$14)</f>
-        <v>63.59654442013126</v>
+        <v>58.64435448577678</v>
       </c>
       <c r="D6" s="109">
         <f>C6/(1-D14-C14)</f>
-        <v>141.32565426695834</v>
+        <v>115.84070021881834</v>
       </c>
       <c r="E6" s="110">
         <f>D6*D14</f>
-        <v>49.46397899343542</v>
+        <v>40.544245076586414</v>
       </c>
       <c r="F6" s="110">
         <f>D6-C6-E6</f>
-        <v>28.265130853391653</v>
+        <v>16.652100656455147</v>
       </c>
       <c r="G6" s="110">
         <f>D6*(E14-1)</f>
-        <v>56.53026170678332</v>
+        <v>46.33628008752733</v>
       </c>
       <c r="H6" s="111">
         <f>D6*E14</f>
-        <v>197.85591597374167</v>
+        <v>162.17698030634565</v>
       </c>
     </row>
     <row r="7" ht="19.95" customHeight="1" s="71">
@@ -7144,27 +7158,27 @@
       </c>
       <c r="C7" s="138">
         <f>C6/F14</f>
-        <v>1.2421200082056887</v>
+        <v>1.1453975485503276</v>
       </c>
       <c r="D7" s="140">
         <f>D6/F14</f>
-        <v>2.76026668490153</v>
+        <v>2.2625136761487954</v>
       </c>
       <c r="E7" s="140">
         <f>E6/F14</f>
-        <v>0.9660933397155355</v>
+        <v>0.7918797866520784</v>
       </c>
       <c r="F7" s="140">
         <f>F6/F14</f>
-        <v>0.5520533369803057</v>
+        <v>0.3252363409463896</v>
       </c>
       <c r="G7" s="140">
         <f>G6/F14</f>
-        <v>1.1041066739606116</v>
+        <v>0.9050054704595181</v>
       </c>
       <c r="H7" s="140">
         <f>H6/F14</f>
-        <v>3.864373358862142</v>
+        <v>3.1675191466083135</v>
       </c>
     </row>
     <row r="8" ht="25.95" customHeight="1" s="71">
@@ -7176,62 +7190,62 @@
       </c>
       <c r="B8" s="115">
         <f>B9*F14</f>
-        <v>22.016000000000002</v>
+        <v>27.648000000000003</v>
       </c>
       <c r="C8" s="115">
         <f>B21</f>
-        <v>38.552141963636366</v>
+        <v>43.34341090909091</v>
       </c>
       <c r="D8" s="115">
         <f>C8/(1-D14-C14)</f>
-        <v>85.67142658585858</v>
+        <v>85.61661414141415</v>
       </c>
       <c r="E8" s="116">
         <f>D8*D14</f>
-        <v>29.9849993050505</v>
+        <v>29.96581494949495</v>
       </c>
       <c r="F8" s="116">
         <f>D8-C8-E8</f>
-        <v>17.134285317171717</v>
+        <v>12.307388282828285</v>
       </c>
       <c r="G8" s="116">
         <f>D8*(E14-1)</f>
-        <v>34.268570634343426</v>
+        <v>34.246645656565654</v>
       </c>
       <c r="H8" s="117">
         <f>D8*E14</f>
-        <v>119.939997220202</v>
+        <v>119.8632597979798</v>
       </c>
     </row>
     <row r="9" ht="19.95" customHeight="1" s="71">
       <c r="A9" s="136" t="n"/>
       <c r="B9" s="141">
         <f>B19</f>
-        <v>0.43</v>
+        <v>0.54</v>
       </c>
       <c r="C9" s="142">
         <f>C8/F14</f>
-        <v>0.7529715227272727</v>
+        <v>0.8465509943181818</v>
       </c>
       <c r="D9" s="142">
         <f>D8/F14</f>
-        <v>1.6732700505050504</v>
+        <v>1.672199494949495</v>
       </c>
       <c r="E9" s="142">
         <f>E8/F14</f>
-        <v>0.5856445176767675</v>
+        <v>0.5852698232323231</v>
       </c>
       <c r="F9" s="142">
         <f>F8/F14</f>
-        <v>0.3346540101010101</v>
+        <v>0.24037867739898994</v>
       </c>
       <c r="G9" s="142">
         <f>G8/F14</f>
-        <v>0.66930802020202</v>
+        <v>0.6688797979797979</v>
       </c>
       <c r="H9" s="142">
         <f>H8/F14</f>
-        <v>2.34257807070707</v>
+        <v>2.3410792929292925</v>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1" s="71">
@@ -7242,62 +7256,62 @@
       </c>
       <c r="B10" s="143">
         <f>B8-B4</f>
-        <v>-11.264</v>
+        <v>-5.631999999999998</v>
       </c>
       <c r="C10" s="143">
         <f>C8-C4</f>
-        <v>-16.564863200477447</v>
+        <v>-7.481696311915677</v>
       </c>
       <c r="D10" s="143">
         <f>D8-D4</f>
-        <v>-36.810807112172114</v>
+        <v>-14.778659381561837</v>
       </c>
       <c r="E10" s="143">
         <f>E8-E4</f>
-        <v>-12.883782489260241</v>
+        <v>-5.172530783546641</v>
       </c>
       <c r="F10" s="143">
         <f>F8-F4</f>
-        <v>-7.3621614224344185</v>
+        <v>-2.1244322860995197</v>
       </c>
       <c r="G10" s="143">
         <f>G8-G4</f>
-        <v>-14.724322844868844</v>
+        <v>-5.911463752624734</v>
       </c>
       <c r="H10" s="143">
         <f>H8-H4</f>
-        <v>-51.535129957040965</v>
+        <v>-20.690123134186564</v>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="71">
       <c r="A11" s="136" t="n"/>
       <c r="B11" s="144">
         <f>B9-B5</f>
-        <v>-0.22000000000000003</v>
+        <v>-0.10999999999999999</v>
       </c>
       <c r="C11" s="144">
         <f>C9-C5</f>
-        <v>-0.32353248438432514</v>
+        <v>-0.14612688109210314</v>
       </c>
       <c r="D11" s="144">
         <f>D9-D5</f>
-        <v>-0.7189610764096117</v>
+        <v>-0.2886456910461297</v>
       </c>
       <c r="E11" s="144">
         <f>E9-E5</f>
-        <v>-0.25163637674336414</v>
+        <v>-0.10102599186614536</v>
       </c>
       <c r="F11" s="144">
         <f>F9-F5</f>
-        <v>-0.1437922152819222</v>
+        <v>-0.041492818087881245</v>
       </c>
       <c r="G11" s="144">
         <f>G9-G5</f>
-        <v>-0.28758443056384464</v>
+        <v>-0.11545827641845186</v>
       </c>
       <c r="H11" s="144">
         <f>H9-H5</f>
-        <v>-1.0065455069734566</v>
+        <v>-0.40410396746458144</v>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="71" thickBot="1">
@@ -7322,7 +7336,7 @@
       </c>
       <c r="C13" s="45" t="inlineStr">
         <is>
-          <t>Our margin</t>
+          <t>Margin shown (auto: offsets the cost uplift)</t>
         </is>
       </c>
       <c r="D13" s="45" t="inlineStr">
@@ -7343,6 +7357,11 @@
       <c r="G13" s="45" t="inlineStr">
         <is>
           <t>Cost uplift, % of landed cost (assumption)</t>
+        </is>
+      </c>
+      <c r="H13" s="45" t="inlineStr">
+        <is>
+          <t>Base share of price for cost (real model: 1 − 25 % − 30 %)</t>
         </is>
       </c>
     </row>
@@ -7355,8 +7374,9 @@
       <c r="B14" s="47" t="n">
         <v>120</v>
       </c>
-      <c r="C14" s="145" t="n">
-        <v>0.2</v>
+      <c r="C14" s="182">
+        <f>1-D14-H14*(1+G14)</f>
+        <v>0.14375000000000004</v>
       </c>
       <c r="D14" s="146">
         <f>'Model 33 pallets'!D4</f>
@@ -7371,7 +7391,10 @@
         <v>51.2</v>
       </c>
       <c r="G14" s="145" t="n">
-        <v>0.22</v>
+        <v>0.125</v>
+      </c>
+      <c r="H14" s="145" t="n">
+        <v>0.45</v>
       </c>
     </row>
     <row r="15">
@@ -7462,7 +7485,7 @@
       </c>
       <c r="B19" s="147">
         <f>ROUNDDOWN(((B14/E14*(1-D14-C14)/(1+G14))/F14/(1+C16)-(E16+F16+G16+E16*B18*(D16+B16*(1+D16)))/(C18*D18))/((1+D16)*(1+B16)),2)</f>
-        <v>0.43</v>
+        <v>0.54</v>
       </c>
     </row>
     <row r="20">
@@ -7473,7 +7496,7 @@
       </c>
       <c r="B20" s="148">
         <f>((B14/E14*(1-D14-C14)/(1+G14))/F14/(1+C16)-(E16+F16+G16+E16*B18*(D16+B16*(1+D16)))/(C18*D18))/((1+D16)*(1+B16))</f>
-        <v>0.43025102729470993</v>
+        <v>0.5406979199662126</v>
       </c>
     </row>
     <row r="21" ht="30" customHeight="1" s="71">
@@ -7484,7 +7507,7 @@
       </c>
       <c r="B21" s="57">
         <f>(B19*F14+(E16+F16+G16)/(C18*D18)*F14+(B19+E16*B18/(C18*D18))*D16*F14+(B19+E16*B18/(C18*D18))*(1+D16)*B16*F14)*(1+C16)*(1+G14)</f>
-        <v>38.552141963636366</v>
+        <v>43.34341090909091</v>
       </c>
     </row>
     <row r="22"/>
@@ -7498,9 +7521,9 @@
         <f>'Model 33 pallets'!AL13</f>
         <v>0.882380333698031</v>
       </c>
-      <c r="C23" s="182">
+      <c r="C23" s="183">
         <f>B23*(1+$G$14)</f>
-        <v>1.0765040071115979</v>
+        <v>0.992677875410285</v>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1" s="71">
@@ -7513,9 +7536,9 @@
         <f>'Model 33 pallets'!AL11</f>
         <v>1.018131154266958</v>
       </c>
-      <c r="C24" s="182">
+      <c r="C24" s="183">
         <f>B24*(1+$G$14)</f>
-        <v>1.2421200082056887</v>
+        <v>1.1453975485503278</v>
       </c>
     </row>
   </sheetData>
@@ -7760,7 +7783,7 @@
         <f>ROUNDDOWN((($H9/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K9" s="183">
+      <c r="K9" s="184">
         <f>J9/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7772,7 +7795,7 @@
         <f>ROUNDDOWN((($H9/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N9" s="183">
+      <c r="N9" s="184">
         <f>M9/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -7823,7 +7846,7 @@
         <f>ROUNDDOWN((($H11/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K11" s="183">
+      <c r="K11" s="184">
         <f>J11/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7835,7 +7858,7 @@
         <f>ROUNDDOWN((($H11/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N11" s="183">
+      <c r="N11" s="184">
         <f>M11/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -7879,7 +7902,7 @@
         <f>ROUNDDOWN((($H12/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K12" s="183">
+      <c r="K12" s="184">
         <f>J12/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7891,7 +7914,7 @@
         <f>ROUNDDOWN((($H12/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N12" s="183">
+      <c r="N12" s="184">
         <f>M12/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -7936,7 +7959,7 @@
         <f>ROUNDDOWN((($H13/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K13" s="183">
+      <c r="K13" s="184">
         <f>J13/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -7948,7 +7971,7 @@
         <f>ROUNDDOWN((($H13/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N13" s="183">
+      <c r="N13" s="184">
         <f>M13/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -7993,7 +8016,7 @@
         <f>ROUNDDOWN((($H14/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K14" s="183">
+      <c r="K14" s="184">
         <f>J14/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -8005,7 +8028,7 @@
         <f>ROUNDDOWN((($H14/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.32</v>
       </c>
-      <c r="N14" s="183">
+      <c r="N14" s="184">
         <f>M14/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
@@ -8056,7 +8079,7 @@
         <f>ROUNDDOWN((($H16/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.6</v>
       </c>
-      <c r="K16" s="183">
+      <c r="K16" s="184">
         <f>J16/0.65-1</f>
         <v>-0.07692307692307698</v>
       </c>
@@ -8068,7 +8091,7 @@
         <f>ROUNDDOWN((($H16/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.39</v>
       </c>
-      <c r="N16" s="183">
+      <c r="N16" s="184">
         <f>M16/0.65-1</f>
         <v>-0.4</v>
       </c>
@@ -8112,7 +8135,7 @@
         <f>ROUNDDOWN((($H17/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.54</v>
       </c>
-      <c r="K17" s="183">
+      <c r="K17" s="184">
         <f>J17/0.65-1</f>
         <v>-0.16923076923076918</v>
       </c>
@@ -8124,7 +8147,7 @@
         <f>ROUNDDOWN((($H17/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.33</v>
       </c>
-      <c r="N17" s="183">
+      <c r="N17" s="184">
         <f>M17/0.65-1</f>
         <v>-0.49230769230769234</v>
       </c>
@@ -8168,7 +8191,7 @@
         <f>ROUNDDOWN((($H18/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.48</v>
       </c>
-      <c r="K18" s="183">
+      <c r="K18" s="184">
         <f>J18/0.65-1</f>
         <v>-0.2615384615384616</v>
       </c>
@@ -8180,7 +8203,7 @@
         <f>ROUNDDOWN((($H18/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.27</v>
       </c>
-      <c r="N18" s="183">
+      <c r="N18" s="184">
         <f>M18/0.65-1</f>
         <v>-0.5846153846153845</v>
       </c>
@@ -8224,7 +8247,7 @@
         <f>ROUNDDOWN((($H19/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.42</v>
       </c>
-      <c r="K19" s="183">
+      <c r="K19" s="184">
         <f>J19/0.65-1</f>
         <v>-0.3538461538461539</v>
       </c>
@@ -8236,7 +8259,7 @@
         <f>ROUNDDOWN((($H19/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.2</v>
       </c>
-      <c r="N19" s="183">
+      <c r="N19" s="184">
         <f>M19/0.65-1</f>
         <v>-0.6923076923076923</v>
       </c>
@@ -8287,7 +8310,7 @@
         <f>ROUNDDOWN((($H21/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.47</v>
       </c>
-      <c r="K21" s="183">
+      <c r="K21" s="184">
         <f>J21/0.65-1</f>
         <v>-0.27692307692307694</v>
       </c>
@@ -8299,7 +8322,7 @@
         <f>ROUNDDOWN((($H21/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.25</v>
       </c>
-      <c r="N21" s="183">
+      <c r="N21" s="184">
         <f>M21/0.65-1</f>
         <v>-0.6153846153846154</v>
       </c>
@@ -8343,7 +8366,7 @@
         <f>ROUNDDOWN((($H22/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.4</v>
       </c>
-      <c r="K22" s="183">
+      <c r="K22" s="184">
         <f>J22/0.65-1</f>
         <v>-0.3846153846153846</v>
       </c>
@@ -8355,7 +8378,7 @@
         <f>ROUNDDOWN((($H22/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.19</v>
       </c>
-      <c r="N22" s="183">
+      <c r="N22" s="184">
         <f>M22/0.65-1</f>
         <v>-0.7076923076923076</v>
       </c>
@@ -8406,7 +8429,7 @@
         <f>ROUNDDOWN((($H24/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.6</v>
       </c>
-      <c r="K24" s="183">
+      <c r="K24" s="184">
         <f>J24/0.65-1</f>
         <v>-0.07692307692307698</v>
       </c>
@@ -8418,7 +8441,7 @@
         <f>ROUNDDOWN((($H24/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.39</v>
       </c>
-      <c r="N24" s="183">
+      <c r="N24" s="184">
         <f>M24/0.65-1</f>
         <v>-0.4</v>
       </c>
@@ -8462,7 +8485,7 @@
         <f>ROUNDDOWN((($H25/$D$5/(1+$C$5)-('Price 120 UAH - 33 pallets'!E16+'Price 120 UAH - 33 pallets'!F16+'Price 120 UAH - 33 pallets'!G16+'Price 120 UAH - 33 pallets'!E16*'Price 120 UAH - 33 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 33 pallets'!C18*'Price 120 UAH - 33 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.67</v>
       </c>
-      <c r="K25" s="183">
+      <c r="K25" s="184">
         <f>J25/0.65-1</f>
         <v>0.030769230769230882</v>
       </c>
@@ -8474,7 +8497,7 @@
         <f>ROUNDDOWN((($H25/$D$5/(1+$C$5)-('Price 120 UAH - 6 pallets'!E16+'Price 120 UAH - 6 pallets'!F16+'Price 120 UAH - 6 pallets'!G16+'Price 120 UAH - 6 pallets'!E16*'Price 120 UAH - 6 pallets'!B18*($G$5+$F$5*(1+$G$5)))/('Price 120 UAH - 6 pallets'!C18*'Price 120 UAH - 6 pallets'!D18))/((1+$G$5)*(1+$F$5))),2)</f>
         <v>0.46</v>
       </c>
-      <c r="N25" s="183">
+      <c r="N25" s="184">
         <f>M25/0.65-1</f>
         <v>-0.29230769230769227</v>
       </c>

</xml_diff>

<commit_message>
Model sheets: BEFORE -> AFTER shelf-price block in both models (built on user-edited files)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
+++ b/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
@@ -20,7 +20,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="22">
+  <numFmts count="24">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00&quot; ₴&quot;_-;\-* #,##0.00&quot; ₴&quot;_-;_-* \-??&quot; ₴&quot;_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ [$₴-422]_-;\-* #,##0.00\ [$₴-422]_-;_-* \-??\ [$₴-422]_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="0.0000&quot; €&quot;"/>
@@ -37,14 +37,16 @@
     <numFmt numFmtId="177" formatCode="\+#,##0.00&quot; ₴&quot;;\-#,##0.00&quot; ₴&quot;"/>
     <numFmt numFmtId="178" formatCode="\+&quot;€&quot;0.000;\-&quot;€&quot;0.000"/>
     <numFmt numFmtId="179" formatCode="+0%;-0%;0%"/>
-    <numFmt numFmtId="180" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
-    <numFmt numFmtId="181" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-_);_(@_)"/>
-    <numFmt numFmtId="182" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
-    <numFmt numFmtId="183" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
-    <numFmt numFmtId="184" formatCode="&quot;MARGIN &quot;0%"/>
-    <numFmt numFmtId="185" formatCode="0.00;-0.00;&quot;OK&quot;"/>
+    <numFmt numFmtId="180" formatCode="0.00;-0.00;&quot;OK&quot;"/>
+    <numFmt numFmtId="181" formatCode="&quot;MARGIN &quot;0%"/>
+    <numFmt numFmtId="182" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
+    <numFmt numFmtId="183" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-_);_(@_)"/>
+    <numFmt numFmtId="184" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
+    <numFmt numFmtId="185" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
+    <numFmt numFmtId="186" formatCode="+#,##0.00&quot; ₴&quot;;-#,##0.00&quot; ₴&quot;"/>
+    <numFmt numFmtId="187" formatCode="+0.0%;-0.0%"/>
   </numFmts>
-  <fonts count="42">
+  <fonts count="45">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -283,8 +285,25 @@
       <color rgb="FFB03A3A"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF203864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF203864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFA33A3A"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="31">
+  <fills count="38">
     <fill>
       <patternFill/>
     </fill>
@@ -432,6 +451,41 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FDE8E8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB07A12"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA33A3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9A441"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC26A6A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F8FC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFEF4DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFBE9E9"/>
       </patternFill>
     </fill>
   </fills>
@@ -786,14 +840,14 @@
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="11" fillId="19" borderId="10"/>
-    <xf numFmtId="180" fontId="1" fillId="19" borderId="10"/>
-    <xf numFmtId="181" fontId="1" fillId="19" borderId="10"/>
     <xf numFmtId="182" fontId="1" fillId="19" borderId="10"/>
     <xf numFmtId="183" fontId="1" fillId="19" borderId="10"/>
+    <xf numFmtId="184" fontId="1" fillId="19" borderId="10"/>
+    <xf numFmtId="185" fontId="1" fillId="19" borderId="10"/>
     <xf numFmtId="0" fontId="11" fillId="19" borderId="10"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="10"/>
   </cellStyleXfs>
-  <cellXfs count="185">
+  <cellXfs count="207">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1284,16 +1338,16 @@
     <xf numFmtId="171" fontId="24" fillId="29" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="185" fontId="30" fillId="25" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="180" fontId="30" fillId="25" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="171" fontId="37" fillId="29" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="184" fontId="8" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="184" fontId="8" fillId="18" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="181" fontId="8" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="8" fillId="18" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="172" fontId="36" fillId="23" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1303,6 +1357,72 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="179" fontId="38" fillId="25" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="180" fontId="30" fillId="25" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="8" fillId="15" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="181" fontId="8" fillId="18" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="18" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="31" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="32" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="6" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="42" fillId="23" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="43" fillId="23" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="35" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="10" fillId="35" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="9" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="10" fillId="36" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="10" fillId="36" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="21" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="186" fontId="44" fillId="37" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="187" fontId="44" fillId="37" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1705,7 +1825,7 @@
         <f>F6+G6</f>
         <v>50.82510722100657</v>
       </c>
-      <c r="I6" s="178">
+      <c r="I6" s="185">
         <f>ROUND(H6-'Price 120 UAH - 33 pallets'!C4,4)</f>
         <v>0</v>
       </c>
@@ -1741,7 +1861,7 @@
         <f>F7+G7</f>
         <v>58.64435448577683</v>
       </c>
-      <c r="I7" s="178">
+      <c r="I7" s="185">
         <f>ROUND(H7-'Price 120 UAH - 33 pallets'!C6,4)</f>
         <v>0</v>
       </c>
@@ -1781,7 +1901,7 @@
         <f>F8+G8</f>
         <v>43.34341090909091</v>
       </c>
-      <c r="I8" s="178">
+      <c r="I8" s="185">
         <f>ROUND(H8-'Price 120 UAH - 33 pallets'!C8,4)</f>
         <v>0</v>
       </c>
@@ -1871,7 +1991,7 @@
         <f>F12+G12</f>
         <v>65.3211</v>
       </c>
-      <c r="I12" s="178">
+      <c r="I12" s="185">
         <f>ROUND(H12-'Price 120 UAH - 6 pallets'!C4,4)</f>
         <v>0</v>
       </c>
@@ -1907,7 +2027,7 @@
         <f>F13+G13</f>
         <v>75.3705</v>
       </c>
-      <c r="I13" s="178">
+      <c r="I13" s="185">
         <f>ROUND(H13-'Price 120 UAH - 6 pallets'!C6,4)</f>
         <v>0</v>
       </c>
@@ -1947,7 +2067,7 @@
         <f>F14+G14</f>
         <v>42.92946</v>
       </c>
-      <c r="I14" s="178">
+      <c r="I14" s="185">
         <f>ROUND(H14-'Price 120 UAH - 6 pallets'!C8,4)</f>
         <v>0</v>
       </c>
@@ -1970,7 +2090,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL39"/>
+  <dimension ref="A1:AL53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="4" customWidth="1" style="71" min="1" max="1"/>
@@ -2204,28 +2324,28 @@
         </is>
       </c>
       <c r="O9" s="63" t="n"/>
-      <c r="P9" s="180" t="n">
+      <c r="P9" s="186" t="n">
         <v>0.3</v>
       </c>
       <c r="Q9" s="59" t="n"/>
       <c r="R9" s="59" t="n"/>
       <c r="S9" s="59" t="n"/>
       <c r="T9" s="60" t="n"/>
-      <c r="U9" s="181" t="n">
+      <c r="U9" s="187" t="n">
         <v>0.25</v>
       </c>
       <c r="V9" s="59" t="n"/>
       <c r="W9" s="59" t="n"/>
       <c r="X9" s="59" t="n"/>
       <c r="Y9" s="60" t="n"/>
-      <c r="Z9" s="180" t="n">
+      <c r="Z9" s="186" t="n">
         <v>0.2</v>
       </c>
       <c r="AA9" s="59" t="n"/>
       <c r="AB9" s="59" t="n"/>
       <c r="AC9" s="59" t="n"/>
       <c r="AD9" s="60" t="n"/>
-      <c r="AE9" s="181" t="n">
+      <c r="AE9" s="187" t="n">
         <v>0.15</v>
       </c>
       <c r="AF9" s="59" t="n"/>
@@ -3285,8 +3405,6 @@
         <v>1.134046875</v>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
     <row r="19" ht="28.05" customHeight="1" s="71">
       <c r="A19" s="26" t="n"/>
       <c r="B19" s="88" t="inlineStr">
@@ -4081,13 +4199,598 @@
         <v>140.69159999999994</v>
       </c>
     </row>
+    <row r="42" ht="26" customHeight="1" s="71">
+      <c r="B42" s="188" t="inlineStr">
+        <is>
+          <t>BEFORE → AFTER · shelf price at the current purchase price and at the SIAS request</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1" s="71">
+      <c r="B43" s="189" t="str">
+        <f>"Chain bonus "&amp;ROUND('Price 120 UAH - 6 pallets'!D14*100,0)&amp;" % · margin "&amp;ROUND('Price 120 UAH - 6 pallets'!C14*100,0)&amp;" % · markup ×"&amp;'Price 120 UAH - 6 pallets'!E14</f>
+        <v>Chain bonus 35 % · margin 14 % · markup ×1.4</v>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1" s="71">
+      <c r="E44" s="190" t="inlineStr">
+        <is>
+          <t>BEFORE · current SIAS purchase price</t>
+        </is>
+      </c>
+      <c r="F44" s="190" t="n"/>
+      <c r="G44" s="190" t="n"/>
+      <c r="H44" s="190" t="n"/>
+      <c r="I44" s="190" t="n"/>
+      <c r="J44" s="190" t="n"/>
+      <c r="K44" s="191" t="inlineStr">
+        <is>
+          <t>AFTER · SIAS request (one price for all 6 SKUs)</t>
+        </is>
+      </c>
+      <c r="L44" s="191" t="n"/>
+      <c r="M44" s="191" t="n"/>
+      <c r="N44" s="191" t="n"/>
+      <c r="O44" s="191" t="n"/>
+      <c r="P44" s="191" t="n"/>
+      <c r="Q44" s="192" t="inlineStr">
+        <is>
+          <t>CHANGE</t>
+        </is>
+      </c>
+      <c r="R44" s="192" t="n"/>
+    </row>
+    <row r="45" ht="42" customHeight="1" s="71">
+      <c r="A45" s="193" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B45" s="193" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C45" s="193" t="inlineStr">
+        <is>
+          <t>SIAS purchase: before → after</t>
+        </is>
+      </c>
+      <c r="D45" s="193" t="inlineStr">
+        <is>
+          <t>Weight, g</t>
+        </is>
+      </c>
+      <c r="E45" s="194" t="inlineStr">
+        <is>
+          <t>Purchase, €/pack</t>
+        </is>
+      </c>
+      <c r="F45" s="194" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴/pack</t>
+        </is>
+      </c>
+      <c r="G45" s="194" t="inlineStr">
+        <is>
+          <t>Partner price, ₴</t>
+        </is>
+      </c>
+      <c r="H45" s="194" t="inlineStr">
+        <is>
+          <t>Chain bonus, ₴</t>
+        </is>
+      </c>
+      <c r="I45" s="194" t="inlineStr">
+        <is>
+          <t>Left after bonus, ₴</t>
+        </is>
+      </c>
+      <c r="J45" s="194" t="inlineStr">
+        <is>
+          <t>Shelf price incl. VAT, ₴</t>
+        </is>
+      </c>
+      <c r="K45" s="195" t="inlineStr">
+        <is>
+          <t>Purchase, €/pack</t>
+        </is>
+      </c>
+      <c r="L45" s="195" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴/pack</t>
+        </is>
+      </c>
+      <c r="M45" s="195" t="inlineStr">
+        <is>
+          <t>Partner price, ₴</t>
+        </is>
+      </c>
+      <c r="N45" s="195" t="inlineStr">
+        <is>
+          <t>Chain bonus, ₴</t>
+        </is>
+      </c>
+      <c r="O45" s="195" t="inlineStr">
+        <is>
+          <t>Left after bonus, ₴</t>
+        </is>
+      </c>
+      <c r="P45" s="195" t="inlineStr">
+        <is>
+          <t>Shelf price incl. VAT, ₴</t>
+        </is>
+      </c>
+      <c r="Q45" s="196" t="inlineStr">
+        <is>
+          <t>Δ shelf, ₴</t>
+        </is>
+      </c>
+      <c r="R45" s="196" t="inlineStr">
+        <is>
+          <t>Δ shelf, %</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1" s="71">
+      <c r="A46" s="197">
+        <f>A11</f>
+        <v>1</v>
+      </c>
+      <c r="B46" s="198" t="str">
+        <f>C11</f>
+        <v>Gouda Cheese 123 g</v>
+      </c>
+      <c r="C46" s="197" t="str">
+        <f>"€"&amp;ROUND(E46,2)&amp;" → €"&amp;ROUND(K46,2)</f>
+        <v>€0.75 → €0.32</v>
+      </c>
+      <c r="D46" s="197">
+        <f>D11</f>
+        <v>123</v>
+      </c>
+      <c r="E46" s="199">
+        <f>'Price 120 UAH - 6 pallets'!$B$7</f>
+        <v>0.75</v>
+      </c>
+      <c r="F46" s="200">
+        <f>F11</f>
+        <v>75.3705</v>
+      </c>
+      <c r="G46" s="200">
+        <f>G11</f>
+        <v>148.88000000000002</v>
+      </c>
+      <c r="H46" s="200">
+        <f>H11</f>
+        <v>52.108000000000004</v>
+      </c>
+      <c r="I46" s="200">
+        <f>I11</f>
+        <v>21.401500000000013</v>
+      </c>
+      <c r="J46" s="201">
+        <f>K11</f>
+        <v>208.43200000000002</v>
+      </c>
+      <c r="K46" s="202">
+        <f>'Price 120 UAH - 6 pallets'!$B$20</f>
+        <v>0.32</v>
+      </c>
+      <c r="L46" s="203">
+        <f>'Price 120 UAH - 6 pallets'!$C$8</f>
+        <v>42.92945999999999</v>
+      </c>
+      <c r="M46" s="203">
+        <f>L46/(1-$D$4-$D$5)</f>
+        <v>84.79893333333332</v>
+      </c>
+      <c r="N46" s="203">
+        <f>M46*$D$4</f>
+        <v>29.67962666666666</v>
+      </c>
+      <c r="O46" s="203">
+        <f>M46-L46-N46</f>
+        <v>12.189846666666671</v>
+      </c>
+      <c r="P46" s="204">
+        <f>M46*$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
+      <c r="Q46" s="205">
+        <f>P46-J46</f>
+        <v>-89.71349333333337</v>
+      </c>
+      <c r="R46" s="206">
+        <f>Q46/J46</f>
+        <v>-0.4304209206519794</v>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1" s="71">
+      <c r="A47" s="197">
+        <f>A12</f>
+        <v>2</v>
+      </c>
+      <c r="B47" s="198" t="str">
+        <f>C12</f>
+        <v>Carbonara Spicy 131 g</v>
+      </c>
+      <c r="C47" s="197" t="str">
+        <f>"€"&amp;ROUND(E47,2)&amp;" → €"&amp;ROUND(K47,2)</f>
+        <v>€0.75 → €0.32</v>
+      </c>
+      <c r="D47" s="197">
+        <f>D12</f>
+        <v>131</v>
+      </c>
+      <c r="E47" s="199">
+        <f>'Price 120 UAH - 6 pallets'!$B$7</f>
+        <v>0.75</v>
+      </c>
+      <c r="F47" s="200">
+        <f>F12</f>
+        <v>75.3705</v>
+      </c>
+      <c r="G47" s="200">
+        <f>G12</f>
+        <v>148.88000000000002</v>
+      </c>
+      <c r="H47" s="200">
+        <f>H12</f>
+        <v>52.108000000000004</v>
+      </c>
+      <c r="I47" s="200">
+        <f>I12</f>
+        <v>21.401500000000013</v>
+      </c>
+      <c r="J47" s="201">
+        <f>K12</f>
+        <v>208.43200000000002</v>
+      </c>
+      <c r="K47" s="202">
+        <f>'Price 120 UAH - 6 pallets'!$B$20</f>
+        <v>0.32</v>
+      </c>
+      <c r="L47" s="203">
+        <f>'Price 120 UAH - 6 pallets'!$C$8</f>
+        <v>42.92945999999999</v>
+      </c>
+      <c r="M47" s="203">
+        <f>L47/(1-$D$4-$D$5)</f>
+        <v>84.79893333333332</v>
+      </c>
+      <c r="N47" s="203">
+        <f>M47*$D$4</f>
+        <v>29.67962666666666</v>
+      </c>
+      <c r="O47" s="203">
+        <f>M47-L47-N47</f>
+        <v>12.189846666666671</v>
+      </c>
+      <c r="P47" s="204">
+        <f>M47*$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
+      <c r="Q47" s="205">
+        <f>P47-J47</f>
+        <v>-89.71349333333337</v>
+      </c>
+      <c r="R47" s="206">
+        <f>Q47/J47</f>
+        <v>-0.4304209206519794</v>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1" s="71">
+      <c r="A48" s="197">
+        <f>A13</f>
+        <v>3</v>
+      </c>
+      <c r="B48" s="198" t="str">
+        <f>C13</f>
+        <v>Vegetable Flavor 113 g</v>
+      </c>
+      <c r="C48" s="197" t="str">
+        <f>"€"&amp;ROUND(E48,2)&amp;" → €"&amp;ROUND(K48,2)</f>
+        <v>€0.65 → €0.32</v>
+      </c>
+      <c r="D48" s="197">
+        <f>D13</f>
+        <v>113</v>
+      </c>
+      <c r="E48" s="199">
+        <f>'Price 120 UAH - 6 pallets'!$B$5</f>
+        <v>0.65</v>
+      </c>
+      <c r="F48" s="200">
+        <f>F13</f>
+        <v>65.32109999999999</v>
+      </c>
+      <c r="G48" s="200">
+        <f>G13</f>
+        <v>129.0293333333333</v>
+      </c>
+      <c r="H48" s="200">
+        <f>H13</f>
+        <v>45.16026666666666</v>
+      </c>
+      <c r="I48" s="200">
+        <f>I13</f>
+        <v>18.547966666666667</v>
+      </c>
+      <c r="J48" s="201">
+        <f>K13</f>
+        <v>180.64106666666663</v>
+      </c>
+      <c r="K48" s="202">
+        <f>'Price 120 UAH - 6 pallets'!$B$20</f>
+        <v>0.32</v>
+      </c>
+      <c r="L48" s="203">
+        <f>'Price 120 UAH - 6 pallets'!$C$8</f>
+        <v>42.92945999999999</v>
+      </c>
+      <c r="M48" s="203">
+        <f>L48/(1-$D$4-$D$5)</f>
+        <v>84.79893333333332</v>
+      </c>
+      <c r="N48" s="203">
+        <f>M48*$D$4</f>
+        <v>29.67962666666666</v>
+      </c>
+      <c r="O48" s="203">
+        <f>M48-L48-N48</f>
+        <v>12.189846666666671</v>
+      </c>
+      <c r="P48" s="204">
+        <f>M48*$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
+      <c r="Q48" s="205">
+        <f>P48-J48</f>
+        <v>-61.92255999999999</v>
+      </c>
+      <c r="R48" s="206">
+        <f>Q48/J48</f>
+        <v>-0.342793369983053</v>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1" s="71">
+      <c r="A49" s="197">
+        <f>A14</f>
+        <v>4</v>
+      </c>
+      <c r="B49" s="198" t="str">
+        <f>C14</f>
+        <v>Spicy Flavor 112.5 g</v>
+      </c>
+      <c r="C49" s="197" t="str">
+        <f>"€"&amp;ROUND(E49,2)&amp;" → €"&amp;ROUND(K49,2)</f>
+        <v>€0.65 → €0.32</v>
+      </c>
+      <c r="D49" s="197">
+        <f>D14</f>
+        <v>112.5</v>
+      </c>
+      <c r="E49" s="199">
+        <f>'Price 120 UAH - 6 pallets'!$B$5</f>
+        <v>0.65</v>
+      </c>
+      <c r="F49" s="200">
+        <f>F14</f>
+        <v>65.32109999999999</v>
+      </c>
+      <c r="G49" s="200">
+        <f>G14</f>
+        <v>129.0293333333333</v>
+      </c>
+      <c r="H49" s="200">
+        <f>H14</f>
+        <v>45.16026666666666</v>
+      </c>
+      <c r="I49" s="200">
+        <f>I14</f>
+        <v>18.547966666666667</v>
+      </c>
+      <c r="J49" s="201">
+        <f>K14</f>
+        <v>180.64106666666663</v>
+      </c>
+      <c r="K49" s="202">
+        <f>'Price 120 UAH - 6 pallets'!$B$20</f>
+        <v>0.32</v>
+      </c>
+      <c r="L49" s="203">
+        <f>'Price 120 UAH - 6 pallets'!$C$8</f>
+        <v>42.92945999999999</v>
+      </c>
+      <c r="M49" s="203">
+        <f>L49/(1-$D$4-$D$5)</f>
+        <v>84.79893333333332</v>
+      </c>
+      <c r="N49" s="203">
+        <f>M49*$D$4</f>
+        <v>29.67962666666666</v>
+      </c>
+      <c r="O49" s="203">
+        <f>M49-L49-N49</f>
+        <v>12.189846666666671</v>
+      </c>
+      <c r="P49" s="204">
+        <f>M49*$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
+      <c r="Q49" s="205">
+        <f>P49-J49</f>
+        <v>-61.92255999999999</v>
+      </c>
+      <c r="R49" s="206">
+        <f>Q49/J49</f>
+        <v>-0.342793369983053</v>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1" s="71">
+      <c r="A50" s="197">
+        <f>A15</f>
+        <v>5</v>
+      </c>
+      <c r="B50" s="198" t="str">
+        <f>C15</f>
+        <v>Beef Flavor 113 g</v>
+      </c>
+      <c r="C50" s="197" t="str">
+        <f>"€"&amp;ROUND(E50,2)&amp;" → €"&amp;ROUND(K50,2)</f>
+        <v>€0.65 → €0.32</v>
+      </c>
+      <c r="D50" s="197">
+        <f>D15</f>
+        <v>113</v>
+      </c>
+      <c r="E50" s="199">
+        <f>'Price 120 UAH - 6 pallets'!$B$5</f>
+        <v>0.65</v>
+      </c>
+      <c r="F50" s="200">
+        <f>F15</f>
+        <v>65.32109999999999</v>
+      </c>
+      <c r="G50" s="200">
+        <f>G15</f>
+        <v>129.0293333333333</v>
+      </c>
+      <c r="H50" s="200">
+        <f>H15</f>
+        <v>45.16026666666666</v>
+      </c>
+      <c r="I50" s="200">
+        <f>I15</f>
+        <v>18.547966666666667</v>
+      </c>
+      <c r="J50" s="201">
+        <f>K15</f>
+        <v>180.64106666666663</v>
+      </c>
+      <c r="K50" s="202">
+        <f>'Price 120 UAH - 6 pallets'!$B$20</f>
+        <v>0.32</v>
+      </c>
+      <c r="L50" s="203">
+        <f>'Price 120 UAH - 6 pallets'!$C$8</f>
+        <v>42.92945999999999</v>
+      </c>
+      <c r="M50" s="203">
+        <f>L50/(1-$D$4-$D$5)</f>
+        <v>84.79893333333332</v>
+      </c>
+      <c r="N50" s="203">
+        <f>M50*$D$4</f>
+        <v>29.67962666666666</v>
+      </c>
+      <c r="O50" s="203">
+        <f>M50-L50-N50</f>
+        <v>12.189846666666671</v>
+      </c>
+      <c r="P50" s="204">
+        <f>M50*$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
+      <c r="Q50" s="205">
+        <f>P50-J50</f>
+        <v>-61.92255999999999</v>
+      </c>
+      <c r="R50" s="206">
+        <f>Q50/J50</f>
+        <v>-0.342793369983053</v>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1" s="71">
+      <c r="A51" s="197">
+        <f>A16</f>
+        <v>6</v>
+      </c>
+      <c r="B51" s="198" t="str">
+        <f>C16</f>
+        <v>Chicken Flavor 113 g</v>
+      </c>
+      <c r="C51" s="197" t="str">
+        <f>"€"&amp;ROUND(E51,2)&amp;" → €"&amp;ROUND(K51,2)</f>
+        <v>€0.65 → €0.32</v>
+      </c>
+      <c r="D51" s="197">
+        <f>D16</f>
+        <v>113</v>
+      </c>
+      <c r="E51" s="199">
+        <f>'Price 120 UAH - 6 pallets'!$B$5</f>
+        <v>0.65</v>
+      </c>
+      <c r="F51" s="200">
+        <f>F16</f>
+        <v>65.32109999999999</v>
+      </c>
+      <c r="G51" s="200">
+        <f>G16</f>
+        <v>129.0293333333333</v>
+      </c>
+      <c r="H51" s="200">
+        <f>H16</f>
+        <v>45.16026666666666</v>
+      </c>
+      <c r="I51" s="200">
+        <f>I16</f>
+        <v>18.547966666666667</v>
+      </c>
+      <c r="J51" s="201">
+        <f>K16</f>
+        <v>180.64106666666663</v>
+      </c>
+      <c r="K51" s="202">
+        <f>'Price 120 UAH - 6 pallets'!$B$20</f>
+        <v>0.32</v>
+      </c>
+      <c r="L51" s="203">
+        <f>'Price 120 UAH - 6 pallets'!$C$8</f>
+        <v>42.92945999999999</v>
+      </c>
+      <c r="M51" s="203">
+        <f>L51/(1-$D$4-$D$5)</f>
+        <v>84.79893333333332</v>
+      </c>
+      <c r="N51" s="203">
+        <f>M51*$D$4</f>
+        <v>29.67962666666666</v>
+      </c>
+      <c r="O51" s="203">
+        <f>M51-L51-N51</f>
+        <v>12.189846666666671</v>
+      </c>
+      <c r="P51" s="204">
+        <f>M51*$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
+      <c r="Q51" s="205">
+        <f>P51-J51</f>
+        <v>-61.92255999999999</v>
+      </c>
+      <c r="R51" s="206">
+        <f>Q51/J51</f>
+        <v>-0.342793369983053</v>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1" s="71">
+      <c r="B53" s="171" t="inlineStr">
+        <is>
+          <t>"Before" landed cost per Self-Cost (incl. the uplift from G14 on the "Price 120 UAH" sheets); "after" is calculated at the SIAS request (logistics spread evenly per pack). Bonus, margin and markup come from the "Price 120 UAH" sheets.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="63">
+  <mergeCells count="69">
     <mergeCell ref="U9:Y9"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="D34:E34"/>
+    <mergeCell ref="K44:P44"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="B31:C31"/>
@@ -4103,22 +4806,27 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="G9:J9"/>
+    <mergeCell ref="B43:R43"/>
     <mergeCell ref="E3:K3"/>
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="D32:E32"/>
+    <mergeCell ref="B42:R42"/>
+    <mergeCell ref="E44:J44"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="E5:K5"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="E8:K8"/>
     <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B53:R53"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="D37:E37"/>
     <mergeCell ref="E4:K4"/>
     <mergeCell ref="D28:E28"/>
+    <mergeCell ref="Q44:R44"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="AE9:AI9"/>
     <mergeCell ref="D39:E39"/>
@@ -4154,7 +4862,7 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AL59" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+    <ignoredError sqref="A1:AL73" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4165,7 +4873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL39"/>
+  <dimension ref="A1:AL53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="4" customWidth="1" style="71" min="1" max="1"/>
@@ -4399,28 +5107,28 @@
         </is>
       </c>
       <c r="O9" s="63" t="n"/>
-      <c r="P9" s="180" t="n">
+      <c r="P9" s="186" t="n">
         <v>0.3</v>
       </c>
       <c r="Q9" s="59" t="n"/>
       <c r="R9" s="59" t="n"/>
       <c r="S9" s="59" t="n"/>
       <c r="T9" s="60" t="n"/>
-      <c r="U9" s="181" t="n">
+      <c r="U9" s="187" t="n">
         <v>0.25</v>
       </c>
       <c r="V9" s="59" t="n"/>
       <c r="W9" s="59" t="n"/>
       <c r="X9" s="59" t="n"/>
       <c r="Y9" s="60" t="n"/>
-      <c r="Z9" s="180" t="n">
+      <c r="Z9" s="186" t="n">
         <v>0.2</v>
       </c>
       <c r="AA9" s="59" t="n"/>
       <c r="AB9" s="59" t="n"/>
       <c r="AC9" s="59" t="n"/>
       <c r="AD9" s="60" t="n"/>
-      <c r="AE9" s="181" t="n">
+      <c r="AE9" s="187" t="n">
         <v>0.15</v>
       </c>
       <c r="AF9" s="59" t="n"/>
@@ -5480,8 +6188,6 @@
         <v>0.8823803336980306</v>
       </c>
     </row>
-    <row r="17"/>
-    <row r="18"/>
     <row r="19" ht="28.05" customHeight="1" s="71">
       <c r="A19" s="26" t="n"/>
       <c r="B19" s="88" t="inlineStr">
@@ -6276,13 +6982,598 @@
         <v>109.46946170678342</v>
       </c>
     </row>
+    <row r="42" ht="26" customHeight="1" s="71">
+      <c r="B42" s="188" t="inlineStr">
+        <is>
+          <t>BEFORE → AFTER · shelf price at the current purchase price and at the SIAS request</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1" s="71">
+      <c r="B43" s="189" t="str">
+        <f>"Chain bonus "&amp;ROUND('Price 120 UAH - 33 pallets'!D14*100,0)&amp;" % · margin "&amp;ROUND('Price 120 UAH - 33 pallets'!C14*100,0)&amp;" % · markup ×"&amp;'Price 120 UAH - 33 pallets'!E14</f>
+        <v>Chain bonus 35 % · margin 14 % · markup ×1.4</v>
+      </c>
+    </row>
+    <row r="44" ht="26" customHeight="1" s="71">
+      <c r="E44" s="190" t="inlineStr">
+        <is>
+          <t>BEFORE · current SIAS purchase price</t>
+        </is>
+      </c>
+      <c r="F44" s="190" t="n"/>
+      <c r="G44" s="190" t="n"/>
+      <c r="H44" s="190" t="n"/>
+      <c r="I44" s="190" t="n"/>
+      <c r="J44" s="190" t="n"/>
+      <c r="K44" s="191" t="inlineStr">
+        <is>
+          <t>AFTER · SIAS request (one price for all 6 SKUs)</t>
+        </is>
+      </c>
+      <c r="L44" s="191" t="n"/>
+      <c r="M44" s="191" t="n"/>
+      <c r="N44" s="191" t="n"/>
+      <c r="O44" s="191" t="n"/>
+      <c r="P44" s="191" t="n"/>
+      <c r="Q44" s="192" t="inlineStr">
+        <is>
+          <t>CHANGE</t>
+        </is>
+      </c>
+      <c r="R44" s="192" t="n"/>
+    </row>
+    <row r="45" ht="42" customHeight="1" s="71">
+      <c r="A45" s="193" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B45" s="193" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="C45" s="193" t="inlineStr">
+        <is>
+          <t>SIAS purchase: before → after</t>
+        </is>
+      </c>
+      <c r="D45" s="193" t="inlineStr">
+        <is>
+          <t>Weight, g</t>
+        </is>
+      </c>
+      <c r="E45" s="194" t="inlineStr">
+        <is>
+          <t>Purchase, €/pack</t>
+        </is>
+      </c>
+      <c r="F45" s="194" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴/pack</t>
+        </is>
+      </c>
+      <c r="G45" s="194" t="inlineStr">
+        <is>
+          <t>Partner price, ₴</t>
+        </is>
+      </c>
+      <c r="H45" s="194" t="inlineStr">
+        <is>
+          <t>Chain bonus, ₴</t>
+        </is>
+      </c>
+      <c r="I45" s="194" t="inlineStr">
+        <is>
+          <t>Left after bonus, ₴</t>
+        </is>
+      </c>
+      <c r="J45" s="194" t="inlineStr">
+        <is>
+          <t>Shelf price incl. VAT, ₴</t>
+        </is>
+      </c>
+      <c r="K45" s="195" t="inlineStr">
+        <is>
+          <t>Purchase, €/pack</t>
+        </is>
+      </c>
+      <c r="L45" s="195" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴/pack</t>
+        </is>
+      </c>
+      <c r="M45" s="195" t="inlineStr">
+        <is>
+          <t>Partner price, ₴</t>
+        </is>
+      </c>
+      <c r="N45" s="195" t="inlineStr">
+        <is>
+          <t>Chain bonus, ₴</t>
+        </is>
+      </c>
+      <c r="O45" s="195" t="inlineStr">
+        <is>
+          <t>Left after bonus, ₴</t>
+        </is>
+      </c>
+      <c r="P45" s="195" t="inlineStr">
+        <is>
+          <t>Shelf price incl. VAT, ₴</t>
+        </is>
+      </c>
+      <c r="Q45" s="196" t="inlineStr">
+        <is>
+          <t>Δ shelf, ₴</t>
+        </is>
+      </c>
+      <c r="R45" s="196" t="inlineStr">
+        <is>
+          <t>Δ shelf, %</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1" s="71">
+      <c r="A46" s="197">
+        <f>A11</f>
+        <v>1</v>
+      </c>
+      <c r="B46" s="198" t="str">
+        <f>C11</f>
+        <v>Gouda Cheese 123 g</v>
+      </c>
+      <c r="C46" s="197" t="str">
+        <f>"€"&amp;ROUND(E46,2)&amp;" → €"&amp;ROUND(K46,2)</f>
+        <v>€0.75 → €0.54</v>
+      </c>
+      <c r="D46" s="197">
+        <f>D11</f>
+        <v>123</v>
+      </c>
+      <c r="E46" s="199">
+        <f>'Price 120 UAH - 33 pallets'!$B$7</f>
+        <v>0.75</v>
+      </c>
+      <c r="F46" s="200">
+        <f>F11</f>
+        <v>58.64435448577679</v>
+      </c>
+      <c r="G46" s="200">
+        <f>G11</f>
+        <v>115.84070021881836</v>
+      </c>
+      <c r="H46" s="200">
+        <f>H11</f>
+        <v>40.54424507658642</v>
+      </c>
+      <c r="I46" s="200">
+        <f>I11</f>
+        <v>16.652100656455147</v>
+      </c>
+      <c r="J46" s="201">
+        <f>K11</f>
+        <v>162.17698030634568</v>
+      </c>
+      <c r="K46" s="202">
+        <f>'Price 120 UAH - 33 pallets'!$B$19</f>
+        <v>0.54</v>
+      </c>
+      <c r="L46" s="203">
+        <f>'Price 120 UAH - 33 pallets'!$C$8</f>
+        <v>43.34341090909091</v>
+      </c>
+      <c r="M46" s="203">
+        <f>L46/(1-$D$4-$D$5)</f>
+        <v>85.61661414141415</v>
+      </c>
+      <c r="N46" s="203">
+        <f>M46*$D$4</f>
+        <v>29.96581494949495</v>
+      </c>
+      <c r="O46" s="203">
+        <f>M46-L46-N46</f>
+        <v>12.307388282828285</v>
+      </c>
+      <c r="P46" s="204">
+        <f>M46*$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="Q46" s="205">
+        <f>P46-J46</f>
+        <v>-42.31372050836589</v>
+      </c>
+      <c r="R46" s="206">
+        <f>Q46/J46</f>
+        <v>-0.26091076815240366</v>
+      </c>
+    </row>
+    <row r="47" ht="30" customHeight="1" s="71">
+      <c r="A47" s="197">
+        <f>A12</f>
+        <v>2</v>
+      </c>
+      <c r="B47" s="198" t="str">
+        <f>C12</f>
+        <v>Carbonara Spicy 131 g</v>
+      </c>
+      <c r="C47" s="197" t="str">
+        <f>"€"&amp;ROUND(E47,2)&amp;" → €"&amp;ROUND(K47,2)</f>
+        <v>€0.75 → €0.54</v>
+      </c>
+      <c r="D47" s="197">
+        <f>D12</f>
+        <v>131</v>
+      </c>
+      <c r="E47" s="199">
+        <f>'Price 120 UAH - 33 pallets'!$B$7</f>
+        <v>0.75</v>
+      </c>
+      <c r="F47" s="200">
+        <f>F12</f>
+        <v>58.64435448577679</v>
+      </c>
+      <c r="G47" s="200">
+        <f>G12</f>
+        <v>115.84070021881836</v>
+      </c>
+      <c r="H47" s="200">
+        <f>H12</f>
+        <v>40.54424507658642</v>
+      </c>
+      <c r="I47" s="200">
+        <f>I12</f>
+        <v>16.652100656455147</v>
+      </c>
+      <c r="J47" s="201">
+        <f>K12</f>
+        <v>162.17698030634568</v>
+      </c>
+      <c r="K47" s="202">
+        <f>'Price 120 UAH - 33 pallets'!$B$19</f>
+        <v>0.54</v>
+      </c>
+      <c r="L47" s="203">
+        <f>'Price 120 UAH - 33 pallets'!$C$8</f>
+        <v>43.34341090909091</v>
+      </c>
+      <c r="M47" s="203">
+        <f>L47/(1-$D$4-$D$5)</f>
+        <v>85.61661414141415</v>
+      </c>
+      <c r="N47" s="203">
+        <f>M47*$D$4</f>
+        <v>29.96581494949495</v>
+      </c>
+      <c r="O47" s="203">
+        <f>M47-L47-N47</f>
+        <v>12.307388282828285</v>
+      </c>
+      <c r="P47" s="204">
+        <f>M47*$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="Q47" s="205">
+        <f>P47-J47</f>
+        <v>-42.31372050836589</v>
+      </c>
+      <c r="R47" s="206">
+        <f>Q47/J47</f>
+        <v>-0.26091076815240366</v>
+      </c>
+    </row>
+    <row r="48" ht="30" customHeight="1" s="71">
+      <c r="A48" s="197">
+        <f>A13</f>
+        <v>3</v>
+      </c>
+      <c r="B48" s="198" t="str">
+        <f>C13</f>
+        <v>Vegetable Flavor 113 g</v>
+      </c>
+      <c r="C48" s="197" t="str">
+        <f>"€"&amp;ROUND(E48,2)&amp;" → €"&amp;ROUND(K48,2)</f>
+        <v>€0.65 → €0.54</v>
+      </c>
+      <c r="D48" s="197">
+        <f>D13</f>
+        <v>113</v>
+      </c>
+      <c r="E48" s="199">
+        <f>'Price 120 UAH - 33 pallets'!$B$5</f>
+        <v>0.65</v>
+      </c>
+      <c r="F48" s="200">
+        <f>F13</f>
+        <v>50.82510722100659</v>
+      </c>
+      <c r="G48" s="200">
+        <f>G13</f>
+        <v>100.39527352297598</v>
+      </c>
+      <c r="H48" s="200">
+        <f>H13</f>
+        <v>35.13834573304159</v>
+      </c>
+      <c r="I48" s="200">
+        <f>I13</f>
+        <v>14.431820568927805</v>
+      </c>
+      <c r="J48" s="201">
+        <f>K13</f>
+        <v>140.55338293216636</v>
+      </c>
+      <c r="K48" s="202">
+        <f>'Price 120 UAH - 33 pallets'!$B$19</f>
+        <v>0.54</v>
+      </c>
+      <c r="L48" s="203">
+        <f>'Price 120 UAH - 33 pallets'!$C$8</f>
+        <v>43.34341090909091</v>
+      </c>
+      <c r="M48" s="203">
+        <f>L48/(1-$D$4-$D$5)</f>
+        <v>85.61661414141415</v>
+      </c>
+      <c r="N48" s="203">
+        <f>M48*$D$4</f>
+        <v>29.96581494949495</v>
+      </c>
+      <c r="O48" s="203">
+        <f>M48-L48-N48</f>
+        <v>12.307388282828285</v>
+      </c>
+      <c r="P48" s="204">
+        <f>M48*$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="Q48" s="205">
+        <f>P48-J48</f>
+        <v>-20.690123134186564</v>
+      </c>
+      <c r="R48" s="206">
+        <f>Q48/J48</f>
+        <v>-0.14720473248354327</v>
+      </c>
+    </row>
+    <row r="49" ht="30" customHeight="1" s="71">
+      <c r="A49" s="197">
+        <f>A14</f>
+        <v>4</v>
+      </c>
+      <c r="B49" s="198" t="str">
+        <f>C14</f>
+        <v>Spicy Flavor 112.5 g</v>
+      </c>
+      <c r="C49" s="197" t="str">
+        <f>"€"&amp;ROUND(E49,2)&amp;" → €"&amp;ROUND(K49,2)</f>
+        <v>€0.65 → €0.54</v>
+      </c>
+      <c r="D49" s="197">
+        <f>D14</f>
+        <v>112.5</v>
+      </c>
+      <c r="E49" s="199">
+        <f>'Price 120 UAH - 33 pallets'!$B$5</f>
+        <v>0.65</v>
+      </c>
+      <c r="F49" s="200">
+        <f>F14</f>
+        <v>50.82510722100659</v>
+      </c>
+      <c r="G49" s="200">
+        <f>G14</f>
+        <v>100.39527352297598</v>
+      </c>
+      <c r="H49" s="200">
+        <f>H14</f>
+        <v>35.13834573304159</v>
+      </c>
+      <c r="I49" s="200">
+        <f>I14</f>
+        <v>14.431820568927805</v>
+      </c>
+      <c r="J49" s="201">
+        <f>K14</f>
+        <v>140.55338293216636</v>
+      </c>
+      <c r="K49" s="202">
+        <f>'Price 120 UAH - 33 pallets'!$B$19</f>
+        <v>0.54</v>
+      </c>
+      <c r="L49" s="203">
+        <f>'Price 120 UAH - 33 pallets'!$C$8</f>
+        <v>43.34341090909091</v>
+      </c>
+      <c r="M49" s="203">
+        <f>L49/(1-$D$4-$D$5)</f>
+        <v>85.61661414141415</v>
+      </c>
+      <c r="N49" s="203">
+        <f>M49*$D$4</f>
+        <v>29.96581494949495</v>
+      </c>
+      <c r="O49" s="203">
+        <f>M49-L49-N49</f>
+        <v>12.307388282828285</v>
+      </c>
+      <c r="P49" s="204">
+        <f>M49*$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="Q49" s="205">
+        <f>P49-J49</f>
+        <v>-20.690123134186564</v>
+      </c>
+      <c r="R49" s="206">
+        <f>Q49/J49</f>
+        <v>-0.14720473248354327</v>
+      </c>
+    </row>
+    <row r="50" ht="30" customHeight="1" s="71">
+      <c r="A50" s="197">
+        <f>A15</f>
+        <v>5</v>
+      </c>
+      <c r="B50" s="198" t="str">
+        <f>C15</f>
+        <v>Beef Flavor 113 g</v>
+      </c>
+      <c r="C50" s="197" t="str">
+        <f>"€"&amp;ROUND(E50,2)&amp;" → €"&amp;ROUND(K50,2)</f>
+        <v>€0.65 → €0.54</v>
+      </c>
+      <c r="D50" s="197">
+        <f>D15</f>
+        <v>113</v>
+      </c>
+      <c r="E50" s="199">
+        <f>'Price 120 UAH - 33 pallets'!$B$5</f>
+        <v>0.65</v>
+      </c>
+      <c r="F50" s="200">
+        <f>F15</f>
+        <v>50.82510722100659</v>
+      </c>
+      <c r="G50" s="200">
+        <f>G15</f>
+        <v>100.39527352297598</v>
+      </c>
+      <c r="H50" s="200">
+        <f>H15</f>
+        <v>35.13834573304159</v>
+      </c>
+      <c r="I50" s="200">
+        <f>I15</f>
+        <v>14.431820568927805</v>
+      </c>
+      <c r="J50" s="201">
+        <f>K15</f>
+        <v>140.55338293216636</v>
+      </c>
+      <c r="K50" s="202">
+        <f>'Price 120 UAH - 33 pallets'!$B$19</f>
+        <v>0.54</v>
+      </c>
+      <c r="L50" s="203">
+        <f>'Price 120 UAH - 33 pallets'!$C$8</f>
+        <v>43.34341090909091</v>
+      </c>
+      <c r="M50" s="203">
+        <f>L50/(1-$D$4-$D$5)</f>
+        <v>85.61661414141415</v>
+      </c>
+      <c r="N50" s="203">
+        <f>M50*$D$4</f>
+        <v>29.96581494949495</v>
+      </c>
+      <c r="O50" s="203">
+        <f>M50-L50-N50</f>
+        <v>12.307388282828285</v>
+      </c>
+      <c r="P50" s="204">
+        <f>M50*$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="Q50" s="205">
+        <f>P50-J50</f>
+        <v>-20.690123134186564</v>
+      </c>
+      <c r="R50" s="206">
+        <f>Q50/J50</f>
+        <v>-0.14720473248354327</v>
+      </c>
+    </row>
+    <row r="51" ht="30" customHeight="1" s="71">
+      <c r="A51" s="197">
+        <f>A16</f>
+        <v>6</v>
+      </c>
+      <c r="B51" s="198" t="str">
+        <f>C16</f>
+        <v>Chicken Flavor 113 g</v>
+      </c>
+      <c r="C51" s="197" t="str">
+        <f>"€"&amp;ROUND(E51,2)&amp;" → €"&amp;ROUND(K51,2)</f>
+        <v>€0.65 → €0.54</v>
+      </c>
+      <c r="D51" s="197">
+        <f>D16</f>
+        <v>113</v>
+      </c>
+      <c r="E51" s="199">
+        <f>'Price 120 UAH - 33 pallets'!$B$5</f>
+        <v>0.65</v>
+      </c>
+      <c r="F51" s="200">
+        <f>F16</f>
+        <v>50.82510722100659</v>
+      </c>
+      <c r="G51" s="200">
+        <f>G16</f>
+        <v>100.39527352297598</v>
+      </c>
+      <c r="H51" s="200">
+        <f>H16</f>
+        <v>35.13834573304159</v>
+      </c>
+      <c r="I51" s="200">
+        <f>I16</f>
+        <v>14.431820568927805</v>
+      </c>
+      <c r="J51" s="201">
+        <f>K16</f>
+        <v>140.55338293216636</v>
+      </c>
+      <c r="K51" s="202">
+        <f>'Price 120 UAH - 33 pallets'!$B$19</f>
+        <v>0.54</v>
+      </c>
+      <c r="L51" s="203">
+        <f>'Price 120 UAH - 33 pallets'!$C$8</f>
+        <v>43.34341090909091</v>
+      </c>
+      <c r="M51" s="203">
+        <f>L51/(1-$D$4-$D$5)</f>
+        <v>85.61661414141415</v>
+      </c>
+      <c r="N51" s="203">
+        <f>M51*$D$4</f>
+        <v>29.96581494949495</v>
+      </c>
+      <c r="O51" s="203">
+        <f>M51-L51-N51</f>
+        <v>12.307388282828285</v>
+      </c>
+      <c r="P51" s="204">
+        <f>M51*$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="Q51" s="205">
+        <f>P51-J51</f>
+        <v>-20.690123134186564</v>
+      </c>
+      <c r="R51" s="206">
+        <f>Q51/J51</f>
+        <v>-0.14720473248354327</v>
+      </c>
+    </row>
+    <row r="53" ht="30" customHeight="1" s="71">
+      <c r="B53" s="171" t="inlineStr">
+        <is>
+          <t>"Before" landed cost per Self-Cost (incl. the uplift from G14 on the "Price 120 UAH" sheets); "after" is calculated at the SIAS request (logistics spread evenly per pack). Bonus, margin and markup come from the "Price 120 UAH" sheets.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="63">
+  <mergeCells count="69">
     <mergeCell ref="U9:Y9"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B25:C25"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="D34:E34"/>
+    <mergeCell ref="K44:P44"/>
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="B31:C31"/>
@@ -6298,22 +7589,27 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="G9:J9"/>
+    <mergeCell ref="B43:R43"/>
     <mergeCell ref="E3:K3"/>
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="D32:E32"/>
+    <mergeCell ref="B42:R42"/>
+    <mergeCell ref="E44:J44"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="E9:F9"/>
     <mergeCell ref="E5:K5"/>
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="E8:K8"/>
     <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B53:R53"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="D37:E37"/>
     <mergeCell ref="E4:K4"/>
     <mergeCell ref="D28:E28"/>
+    <mergeCell ref="Q44:R44"/>
     <mergeCell ref="L9:M9"/>
     <mergeCell ref="AE9:AI9"/>
     <mergeCell ref="D39:E39"/>
@@ -6349,7 +7645,7 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AL59" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+    <ignoredError sqref="A1:AL73" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -6880,7 +8176,6 @@
         <v>1600</v>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="54" t="inlineStr">
         <is>
@@ -6914,7 +8209,6 @@
         <v>42.92945999999999</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24" ht="30" customHeight="1" s="71">
       <c r="A24" s="54" t="inlineStr">
         <is>
@@ -7522,7 +8816,6 @@
         <v>43.34341090909091</v>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="30" customHeight="1" s="71">
       <c r="A23" s="54" t="inlineStr">
         <is>
@@ -7611,7 +8904,6 @@
         <v>Allowed (shown) landed cost = partner price × (1 − bonus − margin); product landed cost = that budget ÷ (1 + uplift). 1 p.p. of margin or bonus = 0.86 ₴ per pack = €0.0136 on the request.</v>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="24" customHeight="1" s="71">
       <c r="A4" s="155" t="inlineStr">
         <is>
@@ -7679,7 +8971,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7" ht="52" customHeight="1" s="71">
       <c r="A7" s="161" t="inlineStr">
         <is>
@@ -8517,7 +9808,6 @@
         <v>-0.29230769230769227</v>
       </c>
     </row>
-    <row r="26"/>
     <row r="27" ht="28" customHeight="1" s="71">
       <c r="A27" s="171" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Both models: margin scenarios (35-10 %) BEFORE vs AFTER on Model and Price tabs; Scenarios sheet before/after shelf
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VBVdxY5GcRU6xZ4qeSea35
</commit_message>
<xml_diff>
--- a/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
+++ b/RAMEN_FINMODEL_INTERNAL_EN_PROPORTIONAL_COST.xlsx
@@ -39,14 +39,14 @@
     <numFmt numFmtId="179" formatCode="+0%;-0%;0%"/>
     <numFmt numFmtId="180" formatCode="0.00;-0.00;&quot;OK&quot;"/>
     <numFmt numFmtId="181" formatCode="&quot;MARGIN &quot;0%"/>
-    <numFmt numFmtId="182" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
-    <numFmt numFmtId="183" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-_);_(@_)"/>
-    <numFmt numFmtId="184" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
-    <numFmt numFmtId="185" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
-    <numFmt numFmtId="186" formatCode="+#,##0.00&quot; ₴&quot;;-#,##0.00&quot; ₴&quot;"/>
-    <numFmt numFmtId="187" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="182" formatCode="+#,##0.00&quot; ₴&quot;;-#,##0.00&quot; ₴&quot;"/>
+    <numFmt numFmtId="183" formatCode="+0.0%;-0.0%"/>
+    <numFmt numFmtId="184" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* \-??_);_(@_)"/>
+    <numFmt numFmtId="185" formatCode="_(* #,##0_);_(* \(#,##0\);_(* \-_);_(@_)"/>
+    <numFmt numFmtId="186" formatCode="_(\$* #,##0.00_);_(\$* \(#,##0.00\);_(\$* \-??_);_(@_)"/>
+    <numFmt numFmtId="187" formatCode="_(\$* #,##0_);_(\$* \(#,##0\);_(\$* \-_);_(@_)"/>
   </numFmts>
-  <fonts count="45">
+  <fonts count="48">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -302,6 +302,23 @@
       <color rgb="FFA33A3A"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FFA33A3A"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF222222"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="FF203864"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="38">
     <fill>
@@ -489,7 +506,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="32">
+  <borders count="36">
     <border>
       <left/>
       <right/>
@@ -837,17 +854,61 @@
       </bottom>
     </border>
     <border/>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9D3E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9D3E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D3E0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00C9D3E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9D3E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00C9D3E0"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C9D3E0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00C9D3E0"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="7">
     <xf numFmtId="0" fontId="11" fillId="19" borderId="10"/>
-    <xf numFmtId="182" fontId="1" fillId="19" borderId="10"/>
-    <xf numFmtId="183" fontId="1" fillId="19" borderId="10"/>
     <xf numFmtId="184" fontId="1" fillId="19" borderId="10"/>
     <xf numFmtId="185" fontId="1" fillId="19" borderId="10"/>
+    <xf numFmtId="186" fontId="1" fillId="19" borderId="10"/>
+    <xf numFmtId="187" fontId="1" fillId="19" borderId="10"/>
     <xf numFmtId="0" fontId="11" fillId="19" borderId="10"/>
     <xf numFmtId="9" fontId="1" fillId="19" borderId="10"/>
   </cellStyleXfs>
-  <cellXfs count="207">
+  <cellXfs count="220">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="5">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1419,10 +1480,45 @@
     <xf numFmtId="171" fontId="5" fillId="21" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="186" fontId="44" fillId="37" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="187" fontId="44" fillId="37" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="182" fontId="44" fillId="37" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="44" fillId="37" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="35" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="182" fontId="44" fillId="37" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="183" fontId="44" fillId="37" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="23" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="45" fillId="23" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="46" fillId="23" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="3" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="3" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="173" fontId="47" fillId="21" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="14" fillId="36" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="36" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="25" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2090,7 +2186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL53"/>
+  <dimension ref="A1:AL65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="4" customWidth="1" style="71" min="1" max="1"/>
@@ -4218,27 +4314,27 @@
           <t>BEFORE · current SIAS purchase price</t>
         </is>
       </c>
-      <c r="F44" s="190" t="n"/>
-      <c r="G44" s="190" t="n"/>
-      <c r="H44" s="190" t="n"/>
-      <c r="I44" s="190" t="n"/>
-      <c r="J44" s="190" t="n"/>
+      <c r="F44" s="207" t="n"/>
+      <c r="G44" s="207" t="n"/>
+      <c r="H44" s="207" t="n"/>
+      <c r="I44" s="207" t="n"/>
+      <c r="J44" s="208" t="n"/>
       <c r="K44" s="191" t="inlineStr">
         <is>
           <t>AFTER · SIAS request (one price for all 6 SKUs)</t>
         </is>
       </c>
-      <c r="L44" s="191" t="n"/>
-      <c r="M44" s="191" t="n"/>
-      <c r="N44" s="191" t="n"/>
-      <c r="O44" s="191" t="n"/>
-      <c r="P44" s="191" t="n"/>
+      <c r="L44" s="207" t="n"/>
+      <c r="M44" s="207" t="n"/>
+      <c r="N44" s="207" t="n"/>
+      <c r="O44" s="207" t="n"/>
+      <c r="P44" s="208" t="n"/>
       <c r="Q44" s="192" t="inlineStr">
         <is>
           <t>CHANGE</t>
         </is>
       </c>
-      <c r="R44" s="192" t="n"/>
+      <c r="R44" s="208" t="n"/>
     </row>
     <row r="45" ht="42" customHeight="1" s="71">
       <c r="A45" s="193" t="inlineStr">
@@ -4397,11 +4493,11 @@
         <f>M46*$D$6</f>
         <v>118.71850666666664</v>
       </c>
-      <c r="Q46" s="205">
+      <c r="Q46" s="209">
         <f>P46-J46</f>
         <v>-89.71349333333337</v>
       </c>
-      <c r="R46" s="206">
+      <c r="R46" s="210">
         <f>Q46/J46</f>
         <v>-0.4304209206519794</v>
       </c>
@@ -4471,11 +4567,11 @@
         <f>M47*$D$6</f>
         <v>118.71850666666664</v>
       </c>
-      <c r="Q47" s="205">
+      <c r="Q47" s="209">
         <f>P47-J47</f>
         <v>-89.71349333333337</v>
       </c>
-      <c r="R47" s="206">
+      <c r="R47" s="210">
         <f>Q47/J47</f>
         <v>-0.4304209206519794</v>
       </c>
@@ -4545,11 +4641,11 @@
         <f>M48*$D$6</f>
         <v>118.71850666666664</v>
       </c>
-      <c r="Q48" s="205">
+      <c r="Q48" s="209">
         <f>P48-J48</f>
         <v>-61.92255999999999</v>
       </c>
-      <c r="R48" s="206">
+      <c r="R48" s="210">
         <f>Q48/J48</f>
         <v>-0.342793369983053</v>
       </c>
@@ -4619,11 +4715,11 @@
         <f>M49*$D$6</f>
         <v>118.71850666666664</v>
       </c>
-      <c r="Q49" s="205">
+      <c r="Q49" s="209">
         <f>P49-J49</f>
         <v>-61.92255999999999</v>
       </c>
-      <c r="R49" s="206">
+      <c r="R49" s="210">
         <f>Q49/J49</f>
         <v>-0.342793369983053</v>
       </c>
@@ -4693,11 +4789,11 @@
         <f>M50*$D$6</f>
         <v>118.71850666666664</v>
       </c>
-      <c r="Q50" s="205">
+      <c r="Q50" s="209">
         <f>P50-J50</f>
         <v>-61.92255999999999</v>
       </c>
-      <c r="R50" s="206">
+      <c r="R50" s="210">
         <f>Q50/J50</f>
         <v>-0.342793369983053</v>
       </c>
@@ -4767,11 +4863,11 @@
         <f>M51*$D$6</f>
         <v>118.71850666666664</v>
       </c>
-      <c r="Q51" s="205">
+      <c r="Q51" s="209">
         <f>P51-J51</f>
         <v>-61.92255999999999</v>
       </c>
-      <c r="R51" s="206">
+      <c r="R51" s="210">
         <f>Q51/J51</f>
         <v>-0.342793369983053</v>
       </c>
@@ -4783,8 +4879,397 @@
         </is>
       </c>
     </row>
+    <row r="56" ht="26" customHeight="1" s="71">
+      <c r="B56" s="188" t="inlineStr">
+        <is>
+          <t>MARGIN SCENARIOS · BEFORE vs AFTER the SIAS request</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1" s="71">
+      <c r="B57" s="54" t="inlineStr">
+        <is>
+          <t>For each margin: shelf price at the current purchase price (BEFORE) and the purchase price SIAS must accept so that the shelf price is 120 ₴ (AFTER). Chain bonus and markup as on the "Price 120 UAH" sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="24" customHeight="1" s="71">
+      <c r="E58" s="190" t="inlineStr">
+        <is>
+          <t>BEFORE · current purchase price</t>
+        </is>
+      </c>
+      <c r="F58" s="190" t="n"/>
+      <c r="G58" s="191" t="inlineStr">
+        <is>
+          <t>AFTER · request for a 120 ₴ shelf</t>
+        </is>
+      </c>
+      <c r="H58" s="191" t="n"/>
+      <c r="I58" s="191" t="n"/>
+      <c r="J58" s="192" t="inlineStr">
+        <is>
+          <t>CHANGE vs BEFORE</t>
+        </is>
+      </c>
+      <c r="K58" s="192" t="n"/>
+      <c r="L58" s="192" t="n"/>
+      <c r="M58" s="192" t="n"/>
+    </row>
+    <row r="59" ht="38" customHeight="1" s="71">
+      <c r="B59" s="193" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="C59" s="193" t="inlineStr"/>
+      <c r="D59" s="193" t="inlineStr">
+        <is>
+          <t>Share of price for cost</t>
+        </is>
+      </c>
+      <c r="E59" s="194" t="inlineStr">
+        <is>
+          <t>Shelf 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="F59" s="194" t="inlineStr">
+        <is>
+          <t>Shelf 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="G59" s="195" t="inlineStr">
+        <is>
+          <t>Request, €/pack</t>
+        </is>
+      </c>
+      <c r="H59" s="195" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴</t>
+        </is>
+      </c>
+      <c r="I59" s="195" t="inlineStr">
+        <is>
+          <t>Shelf, ₴</t>
+        </is>
+      </c>
+      <c r="J59" s="196" t="inlineStr">
+        <is>
+          <t>Δ 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="K59" s="196" t="inlineStr">
+        <is>
+          <t>Δ 4 SKUs, %</t>
+        </is>
+      </c>
+      <c r="L59" s="196" t="inlineStr">
+        <is>
+          <t>Δ 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="M59" s="196" t="inlineStr">
+        <is>
+          <t>Δ 2 SKUs, %</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1" s="71">
+      <c r="B60" s="211" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C60" s="212" t="str">
+        <f>IF(ABS(B60-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D60" s="213">
+        <f>1-'Model 6 pallets'!$D$4-B60</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="E60" s="214">
+        <f>'Model 6 pallets'!$F$13/D60*'Model 6 pallets'!$D$6</f>
+        <v>304.8317999999999</v>
+      </c>
+      <c r="F60" s="215">
+        <f>'Model 6 pallets'!$F$11/D60*'Model 6 pallets'!$D$6</f>
+        <v>351.729</v>
+      </c>
+      <c r="G60" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*D60/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.07</v>
+      </c>
+      <c r="H60" s="217">
+        <f>(G60*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(G60+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(G60+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>25.217459999999996</v>
+      </c>
+      <c r="I60" s="218">
+        <f>H60/D60*'Model 6 pallets'!$D$6</f>
+        <v>117.68147999999995</v>
+      </c>
+      <c r="J60" s="209">
+        <f>I60-E60</f>
+        <v>-187.1503199999999</v>
+      </c>
+      <c r="K60" s="210">
+        <f>J60/E60</f>
+        <v>-0.613946182780143</v>
+      </c>
+      <c r="L60" s="209">
+        <f>I60-F60</f>
+        <v>-234.04752000000002</v>
+      </c>
+      <c r="M60" s="210">
+        <f>L60/F60</f>
+        <v>-0.6654200250761241</v>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1" s="71">
+      <c r="B61" s="211" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C61" s="212" t="str">
+        <f>IF(ABS(B61-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D61" s="213">
+        <f>1-'Model 6 pallets'!$D$4-B61</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="E61" s="214">
+        <f>'Model 6 pallets'!$F$13/D61*'Model 6 pallets'!$D$6</f>
+        <v>261.2843999999999</v>
+      </c>
+      <c r="F61" s="215">
+        <f>'Model 6 pallets'!$F$11/D61*'Model 6 pallets'!$D$6</f>
+        <v>301.48199999999997</v>
+      </c>
+      <c r="G61" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*D61/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.13</v>
+      </c>
+      <c r="H61" s="217">
+        <f>(G61*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(G61+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(G61+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>29.468340000000005</v>
+      </c>
+      <c r="I61" s="218">
+        <f>H61/D61*'Model 6 pallets'!$D$6</f>
+        <v>117.87335999999999</v>
+      </c>
+      <c r="J61" s="209">
+        <f>I61-E61</f>
+        <v>-143.4110399999999</v>
+      </c>
+      <c r="K61" s="210">
+        <f>J61/E61</f>
+        <v>-0.5488695077088412</v>
+      </c>
+      <c r="L61" s="209">
+        <f>I61-F61</f>
+        <v>-183.60863999999998</v>
+      </c>
+      <c r="M61" s="210">
+        <f>L61/F61</f>
+        <v>-0.6090202400143292</v>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1" s="71">
+      <c r="B62" s="211" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C62" s="212" t="str">
+        <f>IF(ABS(B62-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D62" s="213">
+        <f>1-'Model 6 pallets'!$D$4-B62</f>
+        <v>0.4</v>
+      </c>
+      <c r="E62" s="214">
+        <f>'Model 6 pallets'!$F$13/D62*'Model 6 pallets'!$D$6</f>
+        <v>228.62384999999992</v>
+      </c>
+      <c r="F62" s="215">
+        <f>'Model 6 pallets'!$F$11/D62*'Model 6 pallets'!$D$6</f>
+        <v>263.79675</v>
+      </c>
+      <c r="G62" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*D62/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.19</v>
+      </c>
+      <c r="H62" s="217">
+        <f>(G62*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(G62+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(G62+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>33.71922</v>
+      </c>
+      <c r="I62" s="218">
+        <f>H62/D62*'Model 6 pallets'!$D$6</f>
+        <v>118.01726999999998</v>
+      </c>
+      <c r="J62" s="209">
+        <f>I62-E62</f>
+        <v>-110.60657999999994</v>
+      </c>
+      <c r="K62" s="210">
+        <f>J62/E62</f>
+        <v>-0.4837928326375397</v>
+      </c>
+      <c r="L62" s="209">
+        <f>I62-F62</f>
+        <v>-145.77947999999998</v>
+      </c>
+      <c r="M62" s="210">
+        <f>L62/F62</f>
+        <v>-0.5526204549525344</v>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1" s="71">
+      <c r="B63" s="211" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C63" s="212" t="str">
+        <f>IF(ABS(B63-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D63" s="213">
+        <f>1-'Model 6 pallets'!$D$4-B63</f>
+        <v>0.45</v>
+      </c>
+      <c r="E63" s="214">
+        <f>'Model 6 pallets'!$F$13/D63*'Model 6 pallets'!$D$6</f>
+        <v>203.22119999999993</v>
+      </c>
+      <c r="F63" s="215">
+        <f>'Model 6 pallets'!$F$11/D63*'Model 6 pallets'!$D$6</f>
+        <v>234.486</v>
+      </c>
+      <c r="G63" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*D63/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.25</v>
+      </c>
+      <c r="H63" s="217">
+        <f>(G63*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(G63+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(G63+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>37.9701</v>
+      </c>
+      <c r="I63" s="218">
+        <f>H63/D63*'Model 6 pallets'!$D$6</f>
+        <v>118.1292</v>
+      </c>
+      <c r="J63" s="209">
+        <f>I63-E63</f>
+        <v>-85.09199999999993</v>
+      </c>
+      <c r="K63" s="210">
+        <f>J63/E63</f>
+        <v>-0.418716157566238</v>
+      </c>
+      <c r="L63" s="209">
+        <f>I63-F63</f>
+        <v>-116.35679999999999</v>
+      </c>
+      <c r="M63" s="210">
+        <f>L63/F63</f>
+        <v>-0.49622066989073976</v>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1" s="71">
+      <c r="B64" s="211" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C64" s="212" t="str">
+        <f>IF(ABS(B64-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v>◄ ≈ current</v>
+      </c>
+      <c r="D64" s="213">
+        <f>1-'Model 6 pallets'!$D$4-B64</f>
+        <v>0.5</v>
+      </c>
+      <c r="E64" s="214">
+        <f>'Model 6 pallets'!$F$13/D64*'Model 6 pallets'!$D$6</f>
+        <v>182.89907999999994</v>
+      </c>
+      <c r="F64" s="215">
+        <f>'Model 6 pallets'!$F$11/D64*'Model 6 pallets'!$D$6</f>
+        <v>211.03740000000002</v>
+      </c>
+      <c r="G64" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*D64/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.31</v>
+      </c>
+      <c r="H64" s="217">
+        <f>(G64*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(G64+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(G64+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>42.220980000000004</v>
+      </c>
+      <c r="I64" s="218">
+        <f>H64/D64*'Model 6 pallets'!$D$6</f>
+        <v>118.218744</v>
+      </c>
+      <c r="J64" s="209">
+        <f>I64-E64</f>
+        <v>-64.68033599999994</v>
+      </c>
+      <c r="K64" s="210">
+        <f>J64/E64</f>
+        <v>-0.3536394824949363</v>
+      </c>
+      <c r="L64" s="209">
+        <f>I64-F64</f>
+        <v>-92.81865600000002</v>
+      </c>
+      <c r="M64" s="210">
+        <f>L64/F64</f>
+        <v>-0.43982088482894505</v>
+      </c>
+    </row>
+    <row r="65" ht="28" customHeight="1" s="71">
+      <c r="B65" s="211" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C65" s="212" t="str">
+        <f>IF(ABS(B65-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D65" s="213">
+        <f>1-'Model 6 pallets'!$D$4-B65</f>
+        <v>0.55</v>
+      </c>
+      <c r="E65" s="214">
+        <f>'Model 6 pallets'!$F$13/D65*'Model 6 pallets'!$D$6</f>
+        <v>166.27189090909084</v>
+      </c>
+      <c r="F65" s="215">
+        <f>'Model 6 pallets'!$F$11/D65*'Model 6 pallets'!$D$6</f>
+        <v>191.8521818181818</v>
+      </c>
+      <c r="G65" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*D65/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.37</v>
+      </c>
+      <c r="H65" s="217">
+        <f>(G65*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(G65+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(G65+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>46.47186</v>
+      </c>
+      <c r="I65" s="218">
+        <f>H65/D65*'Model 6 pallets'!$D$6</f>
+        <v>118.29200727272726</v>
+      </c>
+      <c r="J65" s="209">
+        <f>I65-E65</f>
+        <v>-47.97988363636358</v>
+      </c>
+      <c r="K65" s="210">
+        <f>J65/E65</f>
+        <v>-0.2885628074236347</v>
+      </c>
+      <c r="L65" s="209">
+        <f>I65-F65</f>
+        <v>-73.56017454545454</v>
+      </c>
+      <c r="M65" s="210">
+        <f>L65/F65</f>
+        <v>-0.3834210997671503</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="69">
+  <mergeCells count="74">
     <mergeCell ref="U9:Y9"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B25:C25"/>
@@ -4794,6 +5279,7 @@
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B57:M57"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="D36:E36"/>
@@ -4806,6 +5292,8 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="G9:J9"/>
+    <mergeCell ref="G58:I58"/>
+    <mergeCell ref="J58:M58"/>
     <mergeCell ref="B43:R43"/>
     <mergeCell ref="E3:K3"/>
     <mergeCell ref="D27:E27"/>
@@ -4820,6 +5308,7 @@
     <mergeCell ref="E8:K8"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B53:R53"/>
+    <mergeCell ref="E58:F58"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B28:C28"/>
@@ -4848,6 +5337,7 @@
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="E6:K6"/>
     <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B56:M56"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="Z9:AD9"/>
     <mergeCell ref="D26:E26"/>
@@ -4862,7 +5352,7 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AL73" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+    <ignoredError sqref="A1:AL85" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4873,7 +5363,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AL53"/>
+  <dimension ref="A1:AL65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6640625" defaultRowHeight="14.4"/>
   <cols>
     <col width="4" customWidth="1" style="71" min="1" max="1"/>
@@ -7001,27 +7491,27 @@
           <t>BEFORE · current SIAS purchase price</t>
         </is>
       </c>
-      <c r="F44" s="190" t="n"/>
-      <c r="G44" s="190" t="n"/>
-      <c r="H44" s="190" t="n"/>
-      <c r="I44" s="190" t="n"/>
-      <c r="J44" s="190" t="n"/>
+      <c r="F44" s="207" t="n"/>
+      <c r="G44" s="207" t="n"/>
+      <c r="H44" s="207" t="n"/>
+      <c r="I44" s="207" t="n"/>
+      <c r="J44" s="208" t="n"/>
       <c r="K44" s="191" t="inlineStr">
         <is>
           <t>AFTER · SIAS request (one price for all 6 SKUs)</t>
         </is>
       </c>
-      <c r="L44" s="191" t="n"/>
-      <c r="M44" s="191" t="n"/>
-      <c r="N44" s="191" t="n"/>
-      <c r="O44" s="191" t="n"/>
-      <c r="P44" s="191" t="n"/>
+      <c r="L44" s="207" t="n"/>
+      <c r="M44" s="207" t="n"/>
+      <c r="N44" s="207" t="n"/>
+      <c r="O44" s="207" t="n"/>
+      <c r="P44" s="208" t="n"/>
       <c r="Q44" s="192" t="inlineStr">
         <is>
           <t>CHANGE</t>
         </is>
       </c>
-      <c r="R44" s="192" t="n"/>
+      <c r="R44" s="208" t="n"/>
     </row>
     <row r="45" ht="42" customHeight="1" s="71">
       <c r="A45" s="193" t="inlineStr">
@@ -7180,11 +7670,11 @@
         <f>M46*$D$6</f>
         <v>119.8632597979798</v>
       </c>
-      <c r="Q46" s="205">
+      <c r="Q46" s="209">
         <f>P46-J46</f>
         <v>-42.31372050836589</v>
       </c>
-      <c r="R46" s="206">
+      <c r="R46" s="210">
         <f>Q46/J46</f>
         <v>-0.26091076815240366</v>
       </c>
@@ -7254,11 +7744,11 @@
         <f>M47*$D$6</f>
         <v>119.8632597979798</v>
       </c>
-      <c r="Q47" s="205">
+      <c r="Q47" s="209">
         <f>P47-J47</f>
         <v>-42.31372050836589</v>
       </c>
-      <c r="R47" s="206">
+      <c r="R47" s="210">
         <f>Q47/J47</f>
         <v>-0.26091076815240366</v>
       </c>
@@ -7328,11 +7818,11 @@
         <f>M48*$D$6</f>
         <v>119.8632597979798</v>
       </c>
-      <c r="Q48" s="205">
+      <c r="Q48" s="209">
         <f>P48-J48</f>
         <v>-20.690123134186564</v>
       </c>
-      <c r="R48" s="206">
+      <c r="R48" s="210">
         <f>Q48/J48</f>
         <v>-0.14720473248354327</v>
       </c>
@@ -7402,11 +7892,11 @@
         <f>M49*$D$6</f>
         <v>119.8632597979798</v>
       </c>
-      <c r="Q49" s="205">
+      <c r="Q49" s="209">
         <f>P49-J49</f>
         <v>-20.690123134186564</v>
       </c>
-      <c r="R49" s="206">
+      <c r="R49" s="210">
         <f>Q49/J49</f>
         <v>-0.14720473248354327</v>
       </c>
@@ -7476,11 +7966,11 @@
         <f>M50*$D$6</f>
         <v>119.8632597979798</v>
       </c>
-      <c r="Q50" s="205">
+      <c r="Q50" s="209">
         <f>P50-J50</f>
         <v>-20.690123134186564</v>
       </c>
-      <c r="R50" s="206">
+      <c r="R50" s="210">
         <f>Q50/J50</f>
         <v>-0.14720473248354327</v>
       </c>
@@ -7550,11 +8040,11 @@
         <f>M51*$D$6</f>
         <v>119.8632597979798</v>
       </c>
-      <c r="Q51" s="205">
+      <c r="Q51" s="209">
         <f>P51-J51</f>
         <v>-20.690123134186564</v>
       </c>
-      <c r="R51" s="206">
+      <c r="R51" s="210">
         <f>Q51/J51</f>
         <v>-0.14720473248354327</v>
       </c>
@@ -7566,8 +8056,397 @@
         </is>
       </c>
     </row>
+    <row r="56" ht="26" customHeight="1" s="71">
+      <c r="B56" s="188" t="inlineStr">
+        <is>
+          <t>MARGIN SCENARIOS · BEFORE vs AFTER the SIAS request</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1" s="71">
+      <c r="B57" s="54" t="inlineStr">
+        <is>
+          <t>For each margin: shelf price at the current purchase price (BEFORE) and the purchase price SIAS must accept so that the shelf price is 120 ₴ (AFTER). Chain bonus and markup as on the "Price 120 UAH" sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="24" customHeight="1" s="71">
+      <c r="E58" s="190" t="inlineStr">
+        <is>
+          <t>BEFORE · current purchase price</t>
+        </is>
+      </c>
+      <c r="F58" s="190" t="n"/>
+      <c r="G58" s="191" t="inlineStr">
+        <is>
+          <t>AFTER · request for a 120 ₴ shelf</t>
+        </is>
+      </c>
+      <c r="H58" s="191" t="n"/>
+      <c r="I58" s="191" t="n"/>
+      <c r="J58" s="192" t="inlineStr">
+        <is>
+          <t>CHANGE vs BEFORE</t>
+        </is>
+      </c>
+      <c r="K58" s="192" t="n"/>
+      <c r="L58" s="192" t="n"/>
+      <c r="M58" s="192" t="n"/>
+    </row>
+    <row r="59" ht="38" customHeight="1" s="71">
+      <c r="B59" s="193" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="C59" s="193" t="inlineStr"/>
+      <c r="D59" s="193" t="inlineStr">
+        <is>
+          <t>Share of price for cost</t>
+        </is>
+      </c>
+      <c r="E59" s="194" t="inlineStr">
+        <is>
+          <t>Shelf 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="F59" s="194" t="inlineStr">
+        <is>
+          <t>Shelf 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="G59" s="195" t="inlineStr">
+        <is>
+          <t>Request, €/pack</t>
+        </is>
+      </c>
+      <c r="H59" s="195" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴</t>
+        </is>
+      </c>
+      <c r="I59" s="195" t="inlineStr">
+        <is>
+          <t>Shelf, ₴</t>
+        </is>
+      </c>
+      <c r="J59" s="196" t="inlineStr">
+        <is>
+          <t>Δ 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="K59" s="196" t="inlineStr">
+        <is>
+          <t>Δ 4 SKUs, %</t>
+        </is>
+      </c>
+      <c r="L59" s="196" t="inlineStr">
+        <is>
+          <t>Δ 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="M59" s="196" t="inlineStr">
+        <is>
+          <t>Δ 2 SKUs, %</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="28" customHeight="1" s="71">
+      <c r="B60" s="211" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C60" s="212" t="str">
+        <f>IF(ABS(B60-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D60" s="213">
+        <f>1-'Model 33 pallets'!$D$4-B60</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="E60" s="214">
+        <f>'Model 33 pallets'!$F$13/D60*'Model 33 pallets'!$D$6</f>
+        <v>237.1838336980307</v>
+      </c>
+      <c r="F60" s="215">
+        <f>'Model 33 pallets'!$F$11/D60*'Model 33 pallets'!$D$6</f>
+        <v>273.6736542669583</v>
+      </c>
+      <c r="G60" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*D60/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.29</v>
+      </c>
+      <c r="H60" s="217">
+        <f>(G60*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(G60+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(G60+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>25.631410909090906</v>
+      </c>
+      <c r="I60" s="218">
+        <f>H60/D60*'Model 33 pallets'!$D$6</f>
+        <v>119.61325090909087</v>
+      </c>
+      <c r="J60" s="209">
+        <f>I60-E60</f>
+        <v>-117.57058278893983</v>
+      </c>
+      <c r="K60" s="210">
+        <f>J60/E60</f>
+        <v>-0.4956939136864791</v>
+      </c>
+      <c r="L60" s="209">
+        <f>I60-F60</f>
+        <v>-154.06040335786741</v>
+      </c>
+      <c r="M60" s="210">
+        <f>L60/F60</f>
+        <v>-0.5629347251949481</v>
+      </c>
+    </row>
+    <row r="61" ht="28" customHeight="1" s="71">
+      <c r="B61" s="211" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C61" s="212" t="str">
+        <f>IF(ABS(B61-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D61" s="213">
+        <f>1-'Model 33 pallets'!$D$4-B61</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="E61" s="214">
+        <f>'Model 33 pallets'!$F$13/D61*'Model 33 pallets'!$D$6</f>
+        <v>203.30042888402633</v>
+      </c>
+      <c r="F61" s="215">
+        <f>'Model 33 pallets'!$F$11/D61*'Model 33 pallets'!$D$6</f>
+        <v>234.5774179431071</v>
+      </c>
+      <c r="G61" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*D61/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.35</v>
+      </c>
+      <c r="H61" s="217">
+        <f>(G61*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(G61+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(G61+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>29.88229090909091</v>
+      </c>
+      <c r="I61" s="218">
+        <f>H61/D61*'Model 33 pallets'!$D$6</f>
+        <v>119.5291636363636</v>
+      </c>
+      <c r="J61" s="209">
+        <f>I61-E61</f>
+        <v>-83.77126524766273</v>
+      </c>
+      <c r="K61" s="210">
+        <f>J61/E61</f>
+        <v>-0.4120565101977745</v>
+      </c>
+      <c r="L61" s="209">
+        <f>I61-F61</f>
+        <v>-115.04825430674349</v>
+      </c>
+      <c r="M61" s="210">
+        <f>L61/F61</f>
+        <v>-0.4904489755047374</v>
+      </c>
+    </row>
+    <row r="62" ht="28" customHeight="1" s="71">
+      <c r="B62" s="211" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C62" s="212" t="str">
+        <f>IF(ABS(B62-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D62" s="213">
+        <f>1-'Model 33 pallets'!$D$4-B62</f>
+        <v>0.4</v>
+      </c>
+      <c r="E62" s="214">
+        <f>'Model 33 pallets'!$F$13/D62*'Model 33 pallets'!$D$6</f>
+        <v>177.88787527352306</v>
+      </c>
+      <c r="F62" s="215">
+        <f>'Model 33 pallets'!$F$11/D62*'Model 33 pallets'!$D$6</f>
+        <v>205.25524070021874</v>
+      </c>
+      <c r="G62" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*D62/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.41</v>
+      </c>
+      <c r="H62" s="217">
+        <f>(G62*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(G62+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(G62+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>34.13317090909091</v>
+      </c>
+      <c r="I62" s="218">
+        <f>H62/D62*'Model 33 pallets'!$D$6</f>
+        <v>119.46609818181815</v>
+      </c>
+      <c r="J62" s="209">
+        <f>I62-E62</f>
+        <v>-58.42177709170491</v>
+      </c>
+      <c r="K62" s="210">
+        <f>J62/E62</f>
+        <v>-0.32841910670907004</v>
+      </c>
+      <c r="L62" s="209">
+        <f>I62-F62</f>
+        <v>-85.78914251840058</v>
+      </c>
+      <c r="M62" s="210">
+        <f>L62/F62</f>
+        <v>-0.41796322581452683</v>
+      </c>
+    </row>
+    <row r="63" ht="28" customHeight="1" s="71">
+      <c r="B63" s="211" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C63" s="212" t="str">
+        <f>IF(ABS(B63-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D63" s="213">
+        <f>1-'Model 33 pallets'!$D$4-B63</f>
+        <v>0.45</v>
+      </c>
+      <c r="E63" s="214">
+        <f>'Model 33 pallets'!$F$13/D63*'Model 33 pallets'!$D$6</f>
+        <v>158.12255579868716</v>
+      </c>
+      <c r="F63" s="215">
+        <f>'Model 33 pallets'!$F$11/D63*'Model 33 pallets'!$D$6</f>
+        <v>182.44910284463887</v>
+      </c>
+      <c r="G63" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*D63/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.47</v>
+      </c>
+      <c r="H63" s="217">
+        <f>(G63*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(G63+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(G63+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>38.3840509090909</v>
+      </c>
+      <c r="I63" s="218">
+        <f>H63/D63*'Model 33 pallets'!$D$6</f>
+        <v>119.41704727272725</v>
+      </c>
+      <c r="J63" s="209">
+        <f>I63-E63</f>
+        <v>-38.705508525959914</v>
+      </c>
+      <c r="K63" s="210">
+        <f>J63/E63</f>
+        <v>-0.24478170322036544</v>
+      </c>
+      <c r="L63" s="209">
+        <f>I63-F63</f>
+        <v>-63.03205557191163</v>
+      </c>
+      <c r="M63" s="210">
+        <f>L63/F63</f>
+        <v>-0.3454774761243161</v>
+      </c>
+    </row>
+    <row r="64" ht="28" customHeight="1" s="71">
+      <c r="B64" s="211" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C64" s="212" t="str">
+        <f>IF(ABS(B64-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v>◄ ≈ current</v>
+      </c>
+      <c r="D64" s="213">
+        <f>1-'Model 33 pallets'!$D$4-B64</f>
+        <v>0.5</v>
+      </c>
+      <c r="E64" s="214">
+        <f>'Model 33 pallets'!$F$13/D64*'Model 33 pallets'!$D$6</f>
+        <v>142.31030021881844</v>
+      </c>
+      <c r="F64" s="215">
+        <f>'Model 33 pallets'!$F$11/D64*'Model 33 pallets'!$D$6</f>
+        <v>164.204192560175</v>
+      </c>
+      <c r="G64" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*D64/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.53</v>
+      </c>
+      <c r="H64" s="217">
+        <f>(G64*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(G64+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(G64+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>42.63493090909091</v>
+      </c>
+      <c r="I64" s="218">
+        <f>H64/D64*'Model 33 pallets'!$D$6</f>
+        <v>119.37780654545455</v>
+      </c>
+      <c r="J64" s="209">
+        <f>I64-E64</f>
+        <v>-22.932493673363894</v>
+      </c>
+      <c r="K64" s="210">
+        <f>J64/E64</f>
+        <v>-0.16114429973166067</v>
+      </c>
+      <c r="L64" s="209">
+        <f>I64-F64</f>
+        <v>-44.82638601472044</v>
+      </c>
+      <c r="M64" s="210">
+        <f>L64/F64</f>
+        <v>-0.2729917264341053</v>
+      </c>
+    </row>
+    <row r="65" ht="28" customHeight="1" s="71">
+      <c r="B65" s="211" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C65" s="212" t="str">
+        <f>IF(ABS(B65-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="D65" s="213">
+        <f>1-'Model 33 pallets'!$D$4-B65</f>
+        <v>0.55</v>
+      </c>
+      <c r="E65" s="214">
+        <f>'Model 33 pallets'!$F$13/D65*'Model 33 pallets'!$D$6</f>
+        <v>129.37300019892584</v>
+      </c>
+      <c r="F65" s="215">
+        <f>'Model 33 pallets'!$F$11/D65*'Model 33 pallets'!$D$6</f>
+        <v>149.27653869106817</v>
+      </c>
+      <c r="G65" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*D65/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.59</v>
+      </c>
+      <c r="H65" s="217">
+        <f>(G65*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(G65+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(G65+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>46.8858109090909</v>
+      </c>
+      <c r="I65" s="218">
+        <f>H65/D65*'Model 33 pallets'!$D$6</f>
+        <v>119.34570049586773</v>
+      </c>
+      <c r="J65" s="209">
+        <f>I65-E65</f>
+        <v>-10.027299703058105</v>
+      </c>
+      <c r="K65" s="210">
+        <f>J65/E65</f>
+        <v>-0.07750689624295627</v>
+      </c>
+      <c r="L65" s="209">
+        <f>I65-F65</f>
+        <v>-29.930838195200437</v>
+      </c>
+      <c r="M65" s="210">
+        <f>L65/F65</f>
+        <v>-0.20050597674389486</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="69">
+  <mergeCells count="74">
     <mergeCell ref="U9:Y9"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B25:C25"/>
@@ -7577,6 +8456,7 @@
     <mergeCell ref="B22:C22"/>
     <mergeCell ref="D22:E22"/>
     <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B57:M57"/>
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="D31:E31"/>
     <mergeCell ref="D36:E36"/>
@@ -7589,6 +8469,8 @@
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="A9:D9"/>
     <mergeCell ref="G9:J9"/>
+    <mergeCell ref="G58:I58"/>
+    <mergeCell ref="J58:M58"/>
     <mergeCell ref="B43:R43"/>
     <mergeCell ref="E3:K3"/>
     <mergeCell ref="D27:E27"/>
@@ -7603,6 +8485,7 @@
     <mergeCell ref="E8:K8"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B53:R53"/>
+    <mergeCell ref="E58:F58"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="B28:C28"/>
@@ -7631,6 +8514,7 @@
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="E6:K6"/>
     <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B56:M56"/>
     <mergeCell ref="B26:C26"/>
     <mergeCell ref="Z9:AD9"/>
     <mergeCell ref="D26:E26"/>
@@ -7645,7 +8529,7 @@
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:AL73" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+    <ignoredError sqref="A1:AL85" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -7657,7 +8541,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="38" customWidth="1" style="71" min="1" max="1"/>
@@ -7665,7 +8549,10 @@
     <col width="23.88671875" customWidth="1" style="71" min="3" max="3"/>
     <col width="17" customWidth="1" style="71" min="4" max="8"/>
     <col width="22" customWidth="1" style="71" min="8" max="8"/>
-    <col width="2" customWidth="1" style="71" min="9" max="9"/>
+    <col width="14" customWidth="1" style="71" min="9" max="9"/>
+    <col width="14" customWidth="1" style="71" min="10" max="10"/>
+    <col width="14" customWidth="1" style="71" min="11" max="11"/>
+    <col width="14" customWidth="1" style="71" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8239,14 +9126,408 @@
         <v>1.472080078125</v>
       </c>
     </row>
+    <row r="28" ht="26" customHeight="1" s="71">
+      <c r="A28" s="188" t="inlineStr">
+        <is>
+          <t>MARGIN SCENARIOS · BEFORE vs AFTER the SIAS request</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1" s="71">
+      <c r="A29" s="54" t="inlineStr">
+        <is>
+          <t>For each margin: shelf price at the current purchase price (BEFORE) and the purchase price SIAS must accept so that the shelf price is 120 ₴ (AFTER). Chain bonus and markup as on the "Price 120 UAH" sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1" s="71">
+      <c r="D30" s="190" t="inlineStr">
+        <is>
+          <t>BEFORE · current purchase price</t>
+        </is>
+      </c>
+      <c r="E30" s="190" t="n"/>
+      <c r="F30" s="191" t="inlineStr">
+        <is>
+          <t>AFTER · request for a 120 ₴ shelf</t>
+        </is>
+      </c>
+      <c r="G30" s="191" t="n"/>
+      <c r="H30" s="191" t="n"/>
+      <c r="I30" s="192" t="inlineStr">
+        <is>
+          <t>CHANGE vs BEFORE</t>
+        </is>
+      </c>
+      <c r="J30" s="192" t="n"/>
+      <c r="K30" s="192" t="n"/>
+      <c r="L30" s="192" t="n"/>
+    </row>
+    <row r="31" ht="38" customHeight="1" s="71">
+      <c r="A31" s="193" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="B31" s="193" t="inlineStr"/>
+      <c r="C31" s="193" t="inlineStr">
+        <is>
+          <t>Share of price for cost</t>
+        </is>
+      </c>
+      <c r="D31" s="194" t="inlineStr">
+        <is>
+          <t>Shelf 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="E31" s="194" t="inlineStr">
+        <is>
+          <t>Shelf 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="F31" s="195" t="inlineStr">
+        <is>
+          <t>Request, €/pack</t>
+        </is>
+      </c>
+      <c r="G31" s="195" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴</t>
+        </is>
+      </c>
+      <c r="H31" s="195" t="inlineStr">
+        <is>
+          <t>Shelf, ₴</t>
+        </is>
+      </c>
+      <c r="I31" s="196" t="inlineStr">
+        <is>
+          <t>Δ 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="J31" s="196" t="inlineStr">
+        <is>
+          <t>Δ 4 SKUs, %</t>
+        </is>
+      </c>
+      <c r="K31" s="196" t="inlineStr">
+        <is>
+          <t>Δ 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="L31" s="196" t="inlineStr">
+        <is>
+          <t>Δ 2 SKUs, %</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1" s="71">
+      <c r="A32" s="211" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B32" s="212" t="str">
+        <f>IF(ABS(A32-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C32" s="213">
+        <f>1-'Model 6 pallets'!$D$4-A32</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="D32" s="214">
+        <f>'Model 6 pallets'!$F$13/C32*'Model 6 pallets'!$D$6</f>
+        <v>304.8317999999999</v>
+      </c>
+      <c r="E32" s="215">
+        <f>'Model 6 pallets'!$F$11/C32*'Model 6 pallets'!$D$6</f>
+        <v>351.729</v>
+      </c>
+      <c r="F32" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*C32/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.07</v>
+      </c>
+      <c r="G32" s="217">
+        <f>(F32*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(F32+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(F32+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>25.217459999999996</v>
+      </c>
+      <c r="H32" s="218">
+        <f>G32/C32*'Model 6 pallets'!$D$6</f>
+        <v>117.68147999999995</v>
+      </c>
+      <c r="I32" s="209">
+        <f>H32-D32</f>
+        <v>-187.1503199999999</v>
+      </c>
+      <c r="J32" s="210">
+        <f>I32/D32</f>
+        <v>-0.613946182780143</v>
+      </c>
+      <c r="K32" s="209">
+        <f>H32-E32</f>
+        <v>-234.04752000000002</v>
+      </c>
+      <c r="L32" s="210">
+        <f>K32/E32</f>
+        <v>-0.6654200250761241</v>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1" s="71">
+      <c r="A33" s="211" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B33" s="212" t="str">
+        <f>IF(ABS(A33-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C33" s="213">
+        <f>1-'Model 6 pallets'!$D$4-A33</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="D33" s="214">
+        <f>'Model 6 pallets'!$F$13/C33*'Model 6 pallets'!$D$6</f>
+        <v>261.2843999999999</v>
+      </c>
+      <c r="E33" s="215">
+        <f>'Model 6 pallets'!$F$11/C33*'Model 6 pallets'!$D$6</f>
+        <v>301.48199999999997</v>
+      </c>
+      <c r="F33" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*C33/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.13</v>
+      </c>
+      <c r="G33" s="217">
+        <f>(F33*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(F33+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(F33+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>29.468340000000005</v>
+      </c>
+      <c r="H33" s="218">
+        <f>G33/C33*'Model 6 pallets'!$D$6</f>
+        <v>117.87335999999999</v>
+      </c>
+      <c r="I33" s="209">
+        <f>H33-D33</f>
+        <v>-143.4110399999999</v>
+      </c>
+      <c r="J33" s="210">
+        <f>I33/D33</f>
+        <v>-0.5488695077088412</v>
+      </c>
+      <c r="K33" s="209">
+        <f>H33-E33</f>
+        <v>-183.60863999999998</v>
+      </c>
+      <c r="L33" s="210">
+        <f>K33/E33</f>
+        <v>-0.6090202400143292</v>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1" s="71">
+      <c r="A34" s="211" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B34" s="212" t="str">
+        <f>IF(ABS(A34-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C34" s="213">
+        <f>1-'Model 6 pallets'!$D$4-A34</f>
+        <v>0.4</v>
+      </c>
+      <c r="D34" s="214">
+        <f>'Model 6 pallets'!$F$13/C34*'Model 6 pallets'!$D$6</f>
+        <v>228.62384999999992</v>
+      </c>
+      <c r="E34" s="215">
+        <f>'Model 6 pallets'!$F$11/C34*'Model 6 pallets'!$D$6</f>
+        <v>263.79675</v>
+      </c>
+      <c r="F34" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*C34/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.19</v>
+      </c>
+      <c r="G34" s="217">
+        <f>(F34*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(F34+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(F34+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>33.71922</v>
+      </c>
+      <c r="H34" s="218">
+        <f>G34/C34*'Model 6 pallets'!$D$6</f>
+        <v>118.01726999999998</v>
+      </c>
+      <c r="I34" s="209">
+        <f>H34-D34</f>
+        <v>-110.60657999999994</v>
+      </c>
+      <c r="J34" s="210">
+        <f>I34/D34</f>
+        <v>-0.4837928326375397</v>
+      </c>
+      <c r="K34" s="209">
+        <f>H34-E34</f>
+        <v>-145.77947999999998</v>
+      </c>
+      <c r="L34" s="210">
+        <f>K34/E34</f>
+        <v>-0.5526204549525344</v>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1" s="71">
+      <c r="A35" s="211" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B35" s="212" t="str">
+        <f>IF(ABS(A35-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C35" s="213">
+        <f>1-'Model 6 pallets'!$D$4-A35</f>
+        <v>0.45</v>
+      </c>
+      <c r="D35" s="214">
+        <f>'Model 6 pallets'!$F$13/C35*'Model 6 pallets'!$D$6</f>
+        <v>203.22119999999993</v>
+      </c>
+      <c r="E35" s="215">
+        <f>'Model 6 pallets'!$F$11/C35*'Model 6 pallets'!$D$6</f>
+        <v>234.486</v>
+      </c>
+      <c r="F35" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*C35/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.25</v>
+      </c>
+      <c r="G35" s="217">
+        <f>(F35*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(F35+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(F35+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>37.9701</v>
+      </c>
+      <c r="H35" s="218">
+        <f>G35/C35*'Model 6 pallets'!$D$6</f>
+        <v>118.1292</v>
+      </c>
+      <c r="I35" s="209">
+        <f>H35-D35</f>
+        <v>-85.09199999999993</v>
+      </c>
+      <c r="J35" s="210">
+        <f>I35/D35</f>
+        <v>-0.418716157566238</v>
+      </c>
+      <c r="K35" s="209">
+        <f>H35-E35</f>
+        <v>-116.35679999999999</v>
+      </c>
+      <c r="L35" s="210">
+        <f>K35/E35</f>
+        <v>-0.49622066989073976</v>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1" s="71">
+      <c r="A36" s="211" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B36" s="212" t="str">
+        <f>IF(ABS(A36-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v>◄ ≈ current</v>
+      </c>
+      <c r="C36" s="213">
+        <f>1-'Model 6 pallets'!$D$4-A36</f>
+        <v>0.5</v>
+      </c>
+      <c r="D36" s="214">
+        <f>'Model 6 pallets'!$F$13/C36*'Model 6 pallets'!$D$6</f>
+        <v>182.89907999999994</v>
+      </c>
+      <c r="E36" s="215">
+        <f>'Model 6 pallets'!$F$11/C36*'Model 6 pallets'!$D$6</f>
+        <v>211.03740000000002</v>
+      </c>
+      <c r="F36" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*C36/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.31</v>
+      </c>
+      <c r="G36" s="217">
+        <f>(F36*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(F36+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(F36+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>42.220980000000004</v>
+      </c>
+      <c r="H36" s="218">
+        <f>G36/C36*'Model 6 pallets'!$D$6</f>
+        <v>118.218744</v>
+      </c>
+      <c r="I36" s="209">
+        <f>H36-D36</f>
+        <v>-64.68033599999994</v>
+      </c>
+      <c r="J36" s="210">
+        <f>I36/D36</f>
+        <v>-0.3536394824949363</v>
+      </c>
+      <c r="K36" s="209">
+        <f>H36-E36</f>
+        <v>-92.81865600000002</v>
+      </c>
+      <c r="L36" s="210">
+        <f>K36/E36</f>
+        <v>-0.43982088482894505</v>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1" s="71">
+      <c r="A37" s="211" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B37" s="212" t="str">
+        <f>IF(ABS(A37-'Price 120 UAH - 6 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C37" s="213">
+        <f>1-'Model 6 pallets'!$D$4-A37</f>
+        <v>0.55</v>
+      </c>
+      <c r="D37" s="214">
+        <f>'Model 6 pallets'!$F$13/C37*'Model 6 pallets'!$D$6</f>
+        <v>166.27189090909084</v>
+      </c>
+      <c r="E37" s="215">
+        <f>'Model 6 pallets'!$F$11/C37*'Model 6 pallets'!$D$6</f>
+        <v>191.8521818181818</v>
+      </c>
+      <c r="F37" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 6 pallets'!$B$14/'Price 120 UAH - 6 pallets'!$E$14*C37/(1+'Price 120 UAH - 6 pallets'!$G$14))/'Model 6 pallets'!$D$3/(1+'Price 120 UAH - 6 pallets'!$C$16)-('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18*('Price 120 UAH - 6 pallets'!$D$16+'Price 120 UAH - 6 pallets'!$B$16*(1+'Price 120 UAH - 6 pallets'!$D$16)))/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))/((1+'Price 120 UAH - 6 pallets'!$D$16)*(1+'Price 120 UAH - 6 pallets'!$B$16)),2)</f>
+        <v>0.37</v>
+      </c>
+      <c r="G37" s="217">
+        <f>(F37*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+(F37+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+(F37+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+'Price 120 UAH - 6 pallets'!$G$14)</f>
+        <v>46.47186</v>
+      </c>
+      <c r="H37" s="218">
+        <f>G37/C37*'Model 6 pallets'!$D$6</f>
+        <v>118.29200727272726</v>
+      </c>
+      <c r="I37" s="209">
+        <f>H37-D37</f>
+        <v>-47.97988363636358</v>
+      </c>
+      <c r="J37" s="210">
+        <f>I37/D37</f>
+        <v>-0.2885628074236347</v>
+      </c>
+      <c r="K37" s="209">
+        <f>H37-E37</f>
+        <v>-73.56017454545454</v>
+      </c>
+      <c r="L37" s="210">
+        <f>K37/E37</f>
+        <v>-0.3834210997671503</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="14">
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A29:L29"/>
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D30:E30"/>
     <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="I30:L30"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="A6:A7"/>
@@ -8254,7 +9535,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H45" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+    <ignoredError sqref="A1:L57" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8266,13 +9547,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="38" customWidth="1" style="71" min="1" max="1"/>
     <col width="17" customWidth="1" style="71" min="2" max="8"/>
     <col width="22" customWidth="1" style="71" min="8" max="8"/>
-    <col width="2" customWidth="1" style="71" min="9" max="9"/>
+    <col width="14" customWidth="1" style="71" min="9" max="9"/>
+    <col width="14" customWidth="1" style="71" min="10" max="10"/>
+    <col width="14" customWidth="1" style="71" min="11" max="11"/>
+    <col width="14" customWidth="1" style="71" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8846,14 +10130,408 @@
         <v>1.1453975485503278</v>
       </c>
     </row>
+    <row r="28" ht="26" customHeight="1" s="71">
+      <c r="A28" s="188" t="inlineStr">
+        <is>
+          <t>MARGIN SCENARIOS · BEFORE vs AFTER the SIAS request</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1" s="71">
+      <c r="A29" s="54" t="inlineStr">
+        <is>
+          <t>For each margin: shelf price at the current purchase price (BEFORE) and the purchase price SIAS must accept so that the shelf price is 120 ₴ (AFTER). Chain bonus and markup as on the "Price 120 UAH" sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="24" customHeight="1" s="71">
+      <c r="D30" s="190" t="inlineStr">
+        <is>
+          <t>BEFORE · current purchase price</t>
+        </is>
+      </c>
+      <c r="E30" s="190" t="n"/>
+      <c r="F30" s="191" t="inlineStr">
+        <is>
+          <t>AFTER · request for a 120 ₴ shelf</t>
+        </is>
+      </c>
+      <c r="G30" s="191" t="n"/>
+      <c r="H30" s="191" t="n"/>
+      <c r="I30" s="192" t="inlineStr">
+        <is>
+          <t>CHANGE vs BEFORE</t>
+        </is>
+      </c>
+      <c r="J30" s="192" t="n"/>
+      <c r="K30" s="192" t="n"/>
+      <c r="L30" s="192" t="n"/>
+    </row>
+    <row r="31" ht="38" customHeight="1" s="71">
+      <c r="A31" s="193" t="inlineStr">
+        <is>
+          <t>Margin</t>
+        </is>
+      </c>
+      <c r="B31" s="193" t="inlineStr"/>
+      <c r="C31" s="193" t="inlineStr">
+        <is>
+          <t>Share of price for cost</t>
+        </is>
+      </c>
+      <c r="D31" s="194" t="inlineStr">
+        <is>
+          <t>Shelf 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="E31" s="194" t="inlineStr">
+        <is>
+          <t>Shelf 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="F31" s="195" t="inlineStr">
+        <is>
+          <t>Request, €/pack</t>
+        </is>
+      </c>
+      <c r="G31" s="195" t="inlineStr">
+        <is>
+          <t>Landed cost, ₴</t>
+        </is>
+      </c>
+      <c r="H31" s="195" t="inlineStr">
+        <is>
+          <t>Shelf, ₴</t>
+        </is>
+      </c>
+      <c r="I31" s="196" t="inlineStr">
+        <is>
+          <t>Δ 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="J31" s="196" t="inlineStr">
+        <is>
+          <t>Δ 4 SKUs, %</t>
+        </is>
+      </c>
+      <c r="K31" s="196" t="inlineStr">
+        <is>
+          <t>Δ 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="L31" s="196" t="inlineStr">
+        <is>
+          <t>Δ 2 SKUs, %</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="28" customHeight="1" s="71">
+      <c r="A32" s="211" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="B32" s="212" t="str">
+        <f>IF(ABS(A32-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C32" s="213">
+        <f>1-'Model 33 pallets'!$D$4-A32</f>
+        <v>0.30000000000000004</v>
+      </c>
+      <c r="D32" s="214">
+        <f>'Model 33 pallets'!$F$13/C32*'Model 33 pallets'!$D$6</f>
+        <v>237.1838336980307</v>
+      </c>
+      <c r="E32" s="215">
+        <f>'Model 33 pallets'!$F$11/C32*'Model 33 pallets'!$D$6</f>
+        <v>273.6736542669583</v>
+      </c>
+      <c r="F32" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*C32/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.29</v>
+      </c>
+      <c r="G32" s="217">
+        <f>(F32*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(F32+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(F32+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>25.631410909090906</v>
+      </c>
+      <c r="H32" s="218">
+        <f>G32/C32*'Model 33 pallets'!$D$6</f>
+        <v>119.61325090909087</v>
+      </c>
+      <c r="I32" s="209">
+        <f>H32-D32</f>
+        <v>-117.57058278893983</v>
+      </c>
+      <c r="J32" s="210">
+        <f>I32/D32</f>
+        <v>-0.4956939136864791</v>
+      </c>
+      <c r="K32" s="209">
+        <f>H32-E32</f>
+        <v>-154.06040335786741</v>
+      </c>
+      <c r="L32" s="210">
+        <f>K32/E32</f>
+        <v>-0.5629347251949481</v>
+      </c>
+    </row>
+    <row r="33" ht="28" customHeight="1" s="71">
+      <c r="A33" s="211" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="B33" s="212" t="str">
+        <f>IF(ABS(A33-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C33" s="213">
+        <f>1-'Model 33 pallets'!$D$4-A33</f>
+        <v>0.35000000000000003</v>
+      </c>
+      <c r="D33" s="214">
+        <f>'Model 33 pallets'!$F$13/C33*'Model 33 pallets'!$D$6</f>
+        <v>203.30042888402633</v>
+      </c>
+      <c r="E33" s="215">
+        <f>'Model 33 pallets'!$F$11/C33*'Model 33 pallets'!$D$6</f>
+        <v>234.5774179431071</v>
+      </c>
+      <c r="F33" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*C33/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.35</v>
+      </c>
+      <c r="G33" s="217">
+        <f>(F33*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(F33+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(F33+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>29.88229090909091</v>
+      </c>
+      <c r="H33" s="218">
+        <f>G33/C33*'Model 33 pallets'!$D$6</f>
+        <v>119.5291636363636</v>
+      </c>
+      <c r="I33" s="209">
+        <f>H33-D33</f>
+        <v>-83.77126524766273</v>
+      </c>
+      <c r="J33" s="210">
+        <f>I33/D33</f>
+        <v>-0.4120565101977745</v>
+      </c>
+      <c r="K33" s="209">
+        <f>H33-E33</f>
+        <v>-115.04825430674349</v>
+      </c>
+      <c r="L33" s="210">
+        <f>K33/E33</f>
+        <v>-0.4904489755047374</v>
+      </c>
+    </row>
+    <row r="34" ht="28" customHeight="1" s="71">
+      <c r="A34" s="211" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="B34" s="212" t="str">
+        <f>IF(ABS(A34-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C34" s="213">
+        <f>1-'Model 33 pallets'!$D$4-A34</f>
+        <v>0.4</v>
+      </c>
+      <c r="D34" s="214">
+        <f>'Model 33 pallets'!$F$13/C34*'Model 33 pallets'!$D$6</f>
+        <v>177.88787527352306</v>
+      </c>
+      <c r="E34" s="215">
+        <f>'Model 33 pallets'!$F$11/C34*'Model 33 pallets'!$D$6</f>
+        <v>205.25524070021874</v>
+      </c>
+      <c r="F34" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*C34/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.41</v>
+      </c>
+      <c r="G34" s="217">
+        <f>(F34*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(F34+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(F34+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>34.13317090909091</v>
+      </c>
+      <c r="H34" s="218">
+        <f>G34/C34*'Model 33 pallets'!$D$6</f>
+        <v>119.46609818181815</v>
+      </c>
+      <c r="I34" s="209">
+        <f>H34-D34</f>
+        <v>-58.42177709170491</v>
+      </c>
+      <c r="J34" s="210">
+        <f>I34/D34</f>
+        <v>-0.32841910670907004</v>
+      </c>
+      <c r="K34" s="209">
+        <f>H34-E34</f>
+        <v>-85.78914251840058</v>
+      </c>
+      <c r="L34" s="210">
+        <f>K34/E34</f>
+        <v>-0.41796322581452683</v>
+      </c>
+    </row>
+    <row r="35" ht="28" customHeight="1" s="71">
+      <c r="A35" s="211" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B35" s="212" t="str">
+        <f>IF(ABS(A35-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C35" s="213">
+        <f>1-'Model 33 pallets'!$D$4-A35</f>
+        <v>0.45</v>
+      </c>
+      <c r="D35" s="214">
+        <f>'Model 33 pallets'!$F$13/C35*'Model 33 pallets'!$D$6</f>
+        <v>158.12255579868716</v>
+      </c>
+      <c r="E35" s="215">
+        <f>'Model 33 pallets'!$F$11/C35*'Model 33 pallets'!$D$6</f>
+        <v>182.44910284463887</v>
+      </c>
+      <c r="F35" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*C35/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.47</v>
+      </c>
+      <c r="G35" s="217">
+        <f>(F35*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(F35+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(F35+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>38.3840509090909</v>
+      </c>
+      <c r="H35" s="218">
+        <f>G35/C35*'Model 33 pallets'!$D$6</f>
+        <v>119.41704727272725</v>
+      </c>
+      <c r="I35" s="209">
+        <f>H35-D35</f>
+        <v>-38.705508525959914</v>
+      </c>
+      <c r="J35" s="210">
+        <f>I35/D35</f>
+        <v>-0.24478170322036544</v>
+      </c>
+      <c r="K35" s="209">
+        <f>H35-E35</f>
+        <v>-63.03205557191163</v>
+      </c>
+      <c r="L35" s="210">
+        <f>K35/E35</f>
+        <v>-0.3454774761243161</v>
+      </c>
+    </row>
+    <row r="36" ht="28" customHeight="1" s="71">
+      <c r="A36" s="211" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="B36" s="212" t="str">
+        <f>IF(ABS(A36-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v>◄ ≈ current</v>
+      </c>
+      <c r="C36" s="213">
+        <f>1-'Model 33 pallets'!$D$4-A36</f>
+        <v>0.5</v>
+      </c>
+      <c r="D36" s="214">
+        <f>'Model 33 pallets'!$F$13/C36*'Model 33 pallets'!$D$6</f>
+        <v>142.31030021881844</v>
+      </c>
+      <c r="E36" s="215">
+        <f>'Model 33 pallets'!$F$11/C36*'Model 33 pallets'!$D$6</f>
+        <v>164.204192560175</v>
+      </c>
+      <c r="F36" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*C36/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.53</v>
+      </c>
+      <c r="G36" s="217">
+        <f>(F36*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(F36+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(F36+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>42.63493090909091</v>
+      </c>
+      <c r="H36" s="218">
+        <f>G36/C36*'Model 33 pallets'!$D$6</f>
+        <v>119.37780654545455</v>
+      </c>
+      <c r="I36" s="209">
+        <f>H36-D36</f>
+        <v>-22.932493673363894</v>
+      </c>
+      <c r="J36" s="210">
+        <f>I36/D36</f>
+        <v>-0.16114429973166067</v>
+      </c>
+      <c r="K36" s="209">
+        <f>H36-E36</f>
+        <v>-44.82638601472044</v>
+      </c>
+      <c r="L36" s="210">
+        <f>K36/E36</f>
+        <v>-0.2729917264341053</v>
+      </c>
+    </row>
+    <row r="37" ht="28" customHeight="1" s="71">
+      <c r="A37" s="211" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="B37" s="212" t="str">
+        <f>IF(ABS(A37-'Price 120 UAH - 33 pallets'!$C$14)&lt;0.01,"◄ ≈ current","")</f>
+        <v/>
+      </c>
+      <c r="C37" s="213">
+        <f>1-'Model 33 pallets'!$D$4-A37</f>
+        <v>0.55</v>
+      </c>
+      <c r="D37" s="214">
+        <f>'Model 33 pallets'!$F$13/C37*'Model 33 pallets'!$D$6</f>
+        <v>129.37300019892584</v>
+      </c>
+      <c r="E37" s="215">
+        <f>'Model 33 pallets'!$F$11/C37*'Model 33 pallets'!$D$6</f>
+        <v>149.27653869106817</v>
+      </c>
+      <c r="F37" s="216">
+        <f>ROUNDDOWN((('Price 120 UAH - 33 pallets'!$B$14/'Price 120 UAH - 33 pallets'!$E$14*C37/(1+'Price 120 UAH - 33 pallets'!$G$14))/'Model 33 pallets'!$D$3/(1+'Price 120 UAH - 33 pallets'!$C$16)-('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18*('Price 120 UAH - 33 pallets'!$D$16+'Price 120 UAH - 33 pallets'!$B$16*(1+'Price 120 UAH - 33 pallets'!$D$16)))/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))/((1+'Price 120 UAH - 33 pallets'!$D$16)*(1+'Price 120 UAH - 33 pallets'!$B$16)),2)</f>
+        <v>0.59</v>
+      </c>
+      <c r="G37" s="217">
+        <f>(F37*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+(F37+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+(F37+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+'Price 120 UAH - 33 pallets'!$G$14)</f>
+        <v>46.8858109090909</v>
+      </c>
+      <c r="H37" s="218">
+        <f>G37/C37*'Model 33 pallets'!$D$6</f>
+        <v>119.34570049586773</v>
+      </c>
+      <c r="I37" s="209">
+        <f>H37-D37</f>
+        <v>-10.027299703058105</v>
+      </c>
+      <c r="J37" s="210">
+        <f>I37/D37</f>
+        <v>-0.07750689624295627</v>
+      </c>
+      <c r="K37" s="209">
+        <f>H37-E37</f>
+        <v>-29.930838195200437</v>
+      </c>
+      <c r="L37" s="210">
+        <f>K37/E37</f>
+        <v>-0.20050597674389486</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="14">
     <mergeCell ref="A12:H12"/>
     <mergeCell ref="F2:G2"/>
     <mergeCell ref="A8:A9"/>
     <mergeCell ref="B2:C2"/>
+    <mergeCell ref="A29:L29"/>
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="D30:E30"/>
     <mergeCell ref="A4:A5"/>
+    <mergeCell ref="A28:L28"/>
+    <mergeCell ref="F30:H30"/>
+    <mergeCell ref="I30:L30"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A10:A11"/>
     <mergeCell ref="A6:A7"/>
@@ -8861,7 +10539,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H44" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+    <ignoredError sqref="A1:L57" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -8872,7 +10550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N29"/>
+  <dimension ref="A1:T39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="71" min="1" max="1"/>
@@ -8889,6 +10567,12 @@
     <col width="15" customWidth="1" style="71" min="12" max="12"/>
     <col width="15" customWidth="1" style="71" min="13" max="13"/>
     <col width="12" customWidth="1" style="71" min="14" max="14"/>
+    <col width="16" customWidth="1" style="71" min="15" max="15"/>
+    <col width="16" customWidth="1" style="71" min="16" max="16"/>
+    <col width="16" customWidth="1" style="71" min="17" max="17"/>
+    <col width="16" customWidth="1" style="71" min="18" max="18"/>
+    <col width="16" customWidth="1" style="71" min="19" max="19"/>
+    <col width="16" customWidth="1" style="71" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" s="71">
@@ -9042,6 +10726,36 @@
           <t>vs current €0.65, %</t>
         </is>
       </c>
+      <c r="O7" s="161" t="inlineStr">
+        <is>
+          <t>33 pallets: shelf BEFORE 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="P7" s="161" t="inlineStr">
+        <is>
+          <t>33 pallets: shelf BEFORE 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="Q7" s="161" t="inlineStr">
+        <is>
+          <t>33 pallets: shelf AFTER request, ₴</t>
+        </is>
+      </c>
+      <c r="R7" s="161" t="inlineStr">
+        <is>
+          <t>6 pallets: shelf BEFORE 4 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="S7" s="161" t="inlineStr">
+        <is>
+          <t>6 pallets: shelf BEFORE 2 SKUs, ₴</t>
+        </is>
+      </c>
+      <c r="T7" s="161" t="inlineStr">
+        <is>
+          <t>6 pallets: shelf AFTER request, ₴</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="20" customHeight="1" s="71">
       <c r="A8" s="162" t="inlineStr">
@@ -9105,6 +10819,30 @@
         <f>M9/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
+      <c r="O9" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D9)/(1-$B9-$C9)*'Model 33 pallets'!$D$6</f>
+        <v>140.55338293216636</v>
+      </c>
+      <c r="P9" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D9)/(1-$B9-$C9)*'Model 33 pallets'!$D$6</f>
+        <v>162.17698030634565</v>
+      </c>
+      <c r="Q9" s="219">
+        <f>($J9*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J9+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J9+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D9)/(1-$B9-$C9)*'Model 33 pallets'!$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="R9" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D9)/(1-$B9-$C9)*'Model 6 pallets'!$D$6</f>
+        <v>180.64106666666663</v>
+      </c>
+      <c r="S9" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D9)/(1-$B9-$C9)*'Model 6 pallets'!$D$6</f>
+        <v>208.43200000000002</v>
+      </c>
+      <c r="T9" s="219">
+        <f>($M9*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M9+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M9+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D9)/(1-$B9-$C9)*'Model 6 pallets'!$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
     </row>
     <row r="10" ht="20" customHeight="1" s="71">
       <c r="A10" s="162" t="inlineStr">
@@ -9168,6 +10906,30 @@
         <f>M11/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
+      <c r="O11" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D11)/(1-$B11-$C11)*'Model 33 pallets'!$D$6</f>
+        <v>140.55338293216636</v>
+      </c>
+      <c r="P11" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D11)/(1-$B11-$C11)*'Model 33 pallets'!$D$6</f>
+        <v>162.17698030634565</v>
+      </c>
+      <c r="Q11" s="219">
+        <f>($J11*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J11+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J11+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D11)/(1-$B11-$C11)*'Model 33 pallets'!$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="R11" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D11)/(1-$B11-$C11)*'Model 6 pallets'!$D$6</f>
+        <v>180.64106666666663</v>
+      </c>
+      <c r="S11" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D11)/(1-$B11-$C11)*'Model 6 pallets'!$D$6</f>
+        <v>208.43200000000002</v>
+      </c>
+      <c r="T11" s="219">
+        <f>($M11*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M11+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M11+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D11)/(1-$B11-$C11)*'Model 6 pallets'!$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
     </row>
     <row r="12" ht="34" customHeight="1" s="71">
       <c r="A12" s="163" t="inlineStr">
@@ -9224,6 +10986,30 @@
         <f>M12/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
+      <c r="O12" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D12)/(1-$B12-$C12)*'Model 33 pallets'!$D$6</f>
+        <v>140.5533829321664</v>
+      </c>
+      <c r="P12" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D12)/(1-$B12-$C12)*'Model 33 pallets'!$D$6</f>
+        <v>162.17698030634565</v>
+      </c>
+      <c r="Q12" s="219">
+        <f>($J12*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J12+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J12+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D12)/(1-$B12-$C12)*'Model 33 pallets'!$D$6</f>
+        <v>119.86325979797982</v>
+      </c>
+      <c r="R12" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D12)/(1-$B12-$C12)*'Model 6 pallets'!$D$6</f>
+        <v>180.64106666666666</v>
+      </c>
+      <c r="S12" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D12)/(1-$B12-$C12)*'Model 6 pallets'!$D$6</f>
+        <v>208.43200000000002</v>
+      </c>
+      <c r="T12" s="219">
+        <f>($M12*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M12+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M12+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D12)/(1-$B12-$C12)*'Model 6 pallets'!$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
     </row>
     <row r="13" ht="34" customHeight="1" s="71">
       <c r="A13" s="163" t="inlineStr">
@@ -9281,6 +11067,30 @@
         <f>M13/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
+      <c r="O13" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D13)/(1-$B13-$C13)*'Model 33 pallets'!$D$6</f>
+        <v>140.55338293216636</v>
+      </c>
+      <c r="P13" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D13)/(1-$B13-$C13)*'Model 33 pallets'!$D$6</f>
+        <v>162.17698030634565</v>
+      </c>
+      <c r="Q13" s="219">
+        <f>($J13*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J13+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J13+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D13)/(1-$B13-$C13)*'Model 33 pallets'!$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="R13" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D13)/(1-$B13-$C13)*'Model 6 pallets'!$D$6</f>
+        <v>180.64106666666663</v>
+      </c>
+      <c r="S13" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D13)/(1-$B13-$C13)*'Model 6 pallets'!$D$6</f>
+        <v>208.43200000000002</v>
+      </c>
+      <c r="T13" s="219">
+        <f>($M13*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M13+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M13+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D13)/(1-$B13-$C13)*'Model 6 pallets'!$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
     </row>
     <row r="14" ht="34" customHeight="1" s="71">
       <c r="A14" s="163" t="inlineStr">
@@ -9338,6 +11148,30 @@
         <f>M14/0.65-1</f>
         <v>-0.5076923076923077</v>
       </c>
+      <c r="O14" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D14)/(1-$B14-$C14)*'Model 33 pallets'!$D$6</f>
+        <v>140.55338293216636</v>
+      </c>
+      <c r="P14" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D14)/(1-$B14-$C14)*'Model 33 pallets'!$D$6</f>
+        <v>162.17698030634565</v>
+      </c>
+      <c r="Q14" s="219">
+        <f>($J14*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J14+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J14+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D14)/(1-$B14-$C14)*'Model 33 pallets'!$D$6</f>
+        <v>119.8632597979798</v>
+      </c>
+      <c r="R14" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D14)/(1-$B14-$C14)*'Model 6 pallets'!$D$6</f>
+        <v>180.64106666666666</v>
+      </c>
+      <c r="S14" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D14)/(1-$B14-$C14)*'Model 6 pallets'!$D$6</f>
+        <v>208.43200000000002</v>
+      </c>
+      <c r="T14" s="219">
+        <f>($M14*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M14+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M14+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D14)/(1-$B14-$C14)*'Model 6 pallets'!$D$6</f>
+        <v>118.71850666666664</v>
+      </c>
     </row>
     <row r="15" ht="20" customHeight="1" s="71">
       <c r="A15" s="162" t="inlineStr">
@@ -9401,6 +11235,30 @@
         <f>M16/0.65-1</f>
         <v>-0.4</v>
       </c>
+      <c r="O16" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D16)/(1-$B16-$C16)*'Model 33 pallets'!$D$6</f>
+        <v>126.49804463894974</v>
+      </c>
+      <c r="P16" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D16)/(1-$B16-$C16)*'Model 33 pallets'!$D$6</f>
+        <v>145.95928227571108</v>
+      </c>
+      <c r="Q16" s="219">
+        <f>($J16*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J16+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D16)/(1-$B16-$C16)*'Model 33 pallets'!$D$6</f>
+        <v>118.45690181818179</v>
+      </c>
+      <c r="R16" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D16)/(1-$B16-$C16)*'Model 6 pallets'!$D$6</f>
+        <v>162.57695999999999</v>
+      </c>
+      <c r="S16" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D16)/(1-$B16-$C16)*'Model 6 pallets'!$D$6</f>
+        <v>187.58880000000002</v>
+      </c>
+      <c r="T16" s="219">
+        <f>($M16*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M16+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D16)/(1-$B16-$C16)*'Model 6 pallets'!$D$6</f>
+        <v>119.18995199999998</v>
+      </c>
     </row>
     <row r="17" ht="34" customHeight="1" s="71">
       <c r="A17" s="163" t="inlineStr">
@@ -9457,6 +11315,30 @@
         <f>M17/0.65-1</f>
         <v>-0.49230769230769234</v>
       </c>
+      <c r="O17" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D17)/(1-$B17-$C17)*'Model 33 pallets'!$D$6</f>
+        <v>139.14784910284473</v>
+      </c>
+      <c r="P17" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D17)/(1-$B17-$C17)*'Model 33 pallets'!$D$6</f>
+        <v>160.5552105032822</v>
+      </c>
+      <c r="Q17" s="219">
+        <f>($J17*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J17+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J17+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D17)/(1-$B17-$C17)*'Model 33 pallets'!$D$6</f>
+        <v>118.66462720000001</v>
+      </c>
+      <c r="R17" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D17)/(1-$B17-$C17)*'Model 6 pallets'!$D$6</f>
+        <v>178.834656</v>
+      </c>
+      <c r="S17" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D17)/(1-$B17-$C17)*'Model 6 pallets'!$D$6</f>
+        <v>206.34768000000003</v>
+      </c>
+      <c r="T17" s="219">
+        <f>($M17*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M17+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M17+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D17)/(1-$B17-$C17)*'Model 6 pallets'!$D$6</f>
+        <v>119.47098239999997</v>
+      </c>
     </row>
     <row r="18" ht="34" customHeight="1" s="71">
       <c r="A18" s="163" t="inlineStr">
@@ -9513,6 +11395,30 @@
         <f>M18/0.65-1</f>
         <v>-0.5846153846153845</v>
       </c>
+      <c r="O18" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D18)/(1-$B18-$C18)*'Model 33 pallets'!$D$6</f>
+        <v>154.60872122538302</v>
+      </c>
+      <c r="P18" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D18)/(1-$B18-$C18)*'Model 33 pallets'!$D$6</f>
+        <v>178.39467833698023</v>
+      </c>
+      <c r="Q18" s="219">
+        <f>($J18*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J18+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J18+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D18)/(1-$B18-$C18)*'Model 33 pallets'!$D$6</f>
+        <v>118.91851377777775</v>
+      </c>
+      <c r="R18" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D18)/(1-$B18-$C18)*'Model 6 pallets'!$D$6</f>
+        <v>198.7051733333333</v>
+      </c>
+      <c r="S18" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D18)/(1-$B18-$C18)*'Model 6 pallets'!$D$6</f>
+        <v>229.2752</v>
+      </c>
+      <c r="T18" s="219">
+        <f>($M18*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M18+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M18+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D18)/(1-$B18-$C18)*'Model 6 pallets'!$D$6</f>
+        <v>119.814464</v>
+      </c>
     </row>
     <row r="19" ht="34" customHeight="1" s="71">
       <c r="A19" s="163" t="inlineStr">
@@ -9569,6 +11475,30 @@
         <f>M19/0.65-1</f>
         <v>-0.6923076923076923</v>
       </c>
+      <c r="O19" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D19)/(1-$B19-$C19)*'Model 33 pallets'!$D$6</f>
+        <v>173.9348113785559</v>
+      </c>
+      <c r="P19" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D19)/(1-$B19-$C19)*'Model 33 pallets'!$D$6</f>
+        <v>200.69401312910276</v>
+      </c>
+      <c r="Q19" s="219">
+        <f>($J19*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J19+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J19+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D19)/(1-$B19-$C19)*'Model 33 pallets'!$D$6</f>
+        <v>119.235872</v>
+      </c>
+      <c r="R19" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D19)/(1-$B19-$C19)*'Model 6 pallets'!$D$6</f>
+        <v>223.54332</v>
+      </c>
+      <c r="S19" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D19)/(1-$B19-$C19)*'Model 6 pallets'!$D$6</f>
+        <v>257.93460000000005</v>
+      </c>
+      <c r="T19" s="219">
+        <f>($M19*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M19+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M19+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D19)/(1-$B19-$C19)*'Model 6 pallets'!$D$6</f>
+        <v>117.81924</v>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1" s="71">
       <c r="A20" s="162" t="inlineStr">
@@ -9632,6 +11562,30 @@
         <f>M21/0.65-1</f>
         <v>-0.6153846153846154</v>
       </c>
+      <c r="O21" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D21)/(1-$B21-$C21)*'Model 33 pallets'!$D$6</f>
+        <v>158.12255579868716</v>
+      </c>
+      <c r="P21" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D21)/(1-$B21-$C21)*'Model 33 pallets'!$D$6</f>
+        <v>182.44910284463887</v>
+      </c>
+      <c r="Q21" s="219">
+        <f>($J21*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J21+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J21+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D21)/(1-$B21-$C21)*'Model 33 pallets'!$D$6</f>
+        <v>119.41704727272723</v>
+      </c>
+      <c r="R21" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D21)/(1-$B21-$C21)*'Model 6 pallets'!$D$6</f>
+        <v>203.22119999999998</v>
+      </c>
+      <c r="S21" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D21)/(1-$B21-$C21)*'Model 6 pallets'!$D$6</f>
+        <v>234.486</v>
+      </c>
+      <c r="T21" s="219">
+        <f>($M21*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M21+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M21+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D21)/(1-$B21-$C21)*'Model 6 pallets'!$D$6</f>
+        <v>118.1292</v>
+      </c>
     </row>
     <row r="22" ht="34" customHeight="1" s="71">
       <c r="A22" s="163" t="inlineStr">
@@ -9688,6 +11642,30 @@
         <f>M22/0.65-1</f>
         <v>-0.7076923076923076</v>
       </c>
+      <c r="O22" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D22)/(1-$B22-$C22)*'Model 33 pallets'!$D$6</f>
+        <v>180.71149234135675</v>
+      </c>
+      <c r="P22" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D22)/(1-$B22-$C22)*'Model 33 pallets'!$D$6</f>
+        <v>208.51326039387297</v>
+      </c>
+      <c r="Q22" s="219">
+        <f>($J22*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J22+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J22+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D22)/(1-$B22-$C22)*'Model 33 pallets'!$D$6</f>
+        <v>118.84334545454546</v>
+      </c>
+      <c r="R22" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D22)/(1-$B22-$C22)*'Model 6 pallets'!$D$6</f>
+        <v>232.25279999999995</v>
+      </c>
+      <c r="S22" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D22)/(1-$B22-$C22)*'Model 6 pallets'!$D$6</f>
+        <v>267.984</v>
+      </c>
+      <c r="T22" s="219">
+        <f>($M22*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M22+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M22+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D22)/(1-$B22-$C22)*'Model 6 pallets'!$D$6</f>
+        <v>119.89056</v>
+      </c>
     </row>
     <row r="23" ht="20" customHeight="1" s="71">
       <c r="A23" s="162" t="inlineStr">
@@ -9751,6 +11729,30 @@
         <f>M24/0.65-1</f>
         <v>-0.4</v>
       </c>
+      <c r="O24" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D24)/(1-$B24-$C24)*'Model 33 pallets'!$D$6</f>
+        <v>126.49804463894974</v>
+      </c>
+      <c r="P24" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D24)/(1-$B24-$C24)*'Model 33 pallets'!$D$6</f>
+        <v>145.95928227571108</v>
+      </c>
+      <c r="Q24" s="219">
+        <f>($J24*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J24+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J24+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D24)/(1-$B24-$C24)*'Model 33 pallets'!$D$6</f>
+        <v>118.45690181818179</v>
+      </c>
+      <c r="R24" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D24)/(1-$B24-$C24)*'Model 6 pallets'!$D$6</f>
+        <v>162.57695999999999</v>
+      </c>
+      <c r="S24" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D24)/(1-$B24-$C24)*'Model 6 pallets'!$D$6</f>
+        <v>187.58880000000002</v>
+      </c>
+      <c r="T24" s="219">
+        <f>($M24*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M24+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M24+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D24)/(1-$B24-$C24)*'Model 6 pallets'!$D$6</f>
+        <v>119.18995199999998</v>
+      </c>
     </row>
     <row r="25" ht="34" customHeight="1" s="71">
       <c r="A25" s="163" t="inlineStr">
@@ -9807,7 +11809,32 @@
         <f>M25/0.65-1</f>
         <v>-0.29230769230769227</v>
       </c>
-    </row>
+      <c r="O25" s="166">
+        <f>'Model 33 pallets'!$AL$13*'Model 33 pallets'!$D$3*(1+$D25)/(1-$B25-$C25)*'Model 33 pallets'!$D$6</f>
+        <v>114.9982223990452</v>
+      </c>
+      <c r="P25" s="166">
+        <f>'Model 33 pallets'!$AL$11*'Model 33 pallets'!$D$3*(1+$D25)/(1-$B25-$C25)*'Model 33 pallets'!$D$6</f>
+        <v>132.6902566142828</v>
+      </c>
+      <c r="Q25" s="219">
+        <f>($J25*'Model 33 pallets'!$D$3+('Price 120 UAH - 33 pallets'!$E$16+'Price 120 UAH - 33 pallets'!$F$16+'Price 120 UAH - 33 pallets'!$G$16)/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18)*'Model 33 pallets'!$D$3+($J25+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*'Price 120 UAH - 33 pallets'!$D$16*'Model 33 pallets'!$D$3+($J25+'Price 120 UAH - 33 pallets'!$E$16*'Price 120 UAH - 33 pallets'!$B$18/('Price 120 UAH - 33 pallets'!$C$18*'Price 120 UAH - 33 pallets'!$D$18))*(1+'Price 120 UAH - 33 pallets'!$D$16)*'Price 120 UAH - 33 pallets'!$B$16*'Model 33 pallets'!$D$3)*(1+'Price 120 UAH - 33 pallets'!$C$16)*(1+$D25)/(1-$B25-$C25)*'Model 33 pallets'!$D$6</f>
+        <v>118.90927074380163</v>
+      </c>
+      <c r="R25" s="166">
+        <f>'Model 6 pallets'!$AL$13*'Model 6 pallets'!$D$3*(1+$D25)/(1-$B25-$C25)*'Model 6 pallets'!$D$6</f>
+        <v>147.79723636363633</v>
+      </c>
+      <c r="S25" s="166">
+        <f>'Model 6 pallets'!$AL$11*'Model 6 pallets'!$D$3*(1+$D25)/(1-$B25-$C25)*'Model 6 pallets'!$D$6</f>
+        <v>170.5352727272727</v>
+      </c>
+      <c r="T25" s="219">
+        <f>($M25*'Model 6 pallets'!$D$3+('Price 120 UAH - 6 pallets'!$E$16+'Price 120 UAH - 6 pallets'!$F$16+'Price 120 UAH - 6 pallets'!$G$16)/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18)*'Model 6 pallets'!$D$3+($M25+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*'Price 120 UAH - 6 pallets'!$D$16*'Model 6 pallets'!$D$3+($M25+'Price 120 UAH - 6 pallets'!$E$16*'Price 120 UAH - 6 pallets'!$B$18/('Price 120 UAH - 6 pallets'!$C$18*'Price 120 UAH - 6 pallets'!$D$18))*(1+'Price 120 UAH - 6 pallets'!$D$16)*'Price 120 UAH - 6 pallets'!$B$16*'Model 6 pallets'!$D$3)*(1+'Price 120 UAH - 6 pallets'!$C$16)*(1+$D25)/(1-$B25-$C25)*'Model 6 pallets'!$D$6</f>
+        <v>119.57567999999998</v>
+      </c>
+    </row>
+    <row r="26"/>
     <row r="27" ht="28" customHeight="1" s="71">
       <c r="A27" s="171" t="inlineStr">
         <is>
@@ -9829,6 +11856,16 @@
         </is>
       </c>
     </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
+    <row r="33"/>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36"/>
+    <row r="37"/>
+    <row r="38"/>
+    <row r="39"/>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="A27:N27"/>
@@ -9844,7 +11881,7 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:N49" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
+    <ignoredError sqref="A1:T59" evalError="1" formula="1" formulaRange="1" unlockedFormula="1" numberStoredAsText="1" emptyCellReference="1" twoDigitTextYear="1" listDataValidation="1" calculatedColumn="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>